<commit_message>
Workbook: total invested restored in account TOTAL rows
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -639,7 +639,7 @@
     <t xml:space="preserve">Holdings as of 23.10.2026. Statement prices: HDFC statement prices 23.10.2026. Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue = figures from the statement (inputs). Black = formulas. Green figures = pulled from another sheet. Green company names = marked holdings. TOTAL is at the bottom; invested base to be supplied.</t>
+    <t xml:space="preserve">Blue = figures from the statement (inputs). Black = formulas. Green figures = pulled from another sheet. Green company names = marked holdings. TOTAL is at the bottom.</t>
   </si>
   <si>
     <t xml:space="preserve">Changes between 05.10 and 23.10 statements (derived; buys at implied avg cost, sells at 05.10 statement price)</t>
@@ -2059,7 +2059,7 @@
         <v>31</v>
       </c>
       <c r="F6" s="7" t="n">
-        <f aca="false">SUM(Gautam!$E$7:$E$300)</f>
+        <f aca="false">Gautam!E38</f>
         <v>5501448</v>
       </c>
       <c r="G6" s="7" t="n">
@@ -2107,7 +2107,7 @@
         <v>53</v>
       </c>
       <c r="F7" s="7" t="n">
-        <f aca="false">SUM(DA!$E$7:$E$300)</f>
+        <f aca="false">DA!E60</f>
         <v>4574421</v>
       </c>
       <c r="G7" s="7" t="n">
@@ -2155,7 +2155,7 @@
         <v>47</v>
       </c>
       <c r="F8" s="7" t="n">
-        <f aca="false">SUM('Manish Shilpa'!$E$7:$E$300)</f>
+        <f aca="false">'Manish Shilpa'!E54</f>
         <v>9857778</v>
       </c>
       <c r="G8" s="7" t="n">
@@ -2203,7 +2203,7 @@
         <v>25</v>
       </c>
       <c r="F9" s="7" t="n">
-        <f aca="false">SUM('Saloni Mehra'!$E$7:$E$300)</f>
+        <f aca="false">'Saloni Mehra'!E32</f>
         <v>11739506</v>
       </c>
       <c r="G9" s="7" t="n">
@@ -2251,7 +2251,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="7" t="n">
-        <f aca="false">SUM('Vidushi Malhotra'!$E$7:$E$300)</f>
+        <f aca="false">'Vidushi Malhotra'!E19</f>
         <v>201361</v>
       </c>
       <c r="G10" s="7" t="n">
@@ -2299,7 +2299,7 @@
         <v>20</v>
       </c>
       <c r="F11" s="7" t="n">
-        <f aca="false">SUM('Dr Umesh Choudhry'!$E$7:$E$300)</f>
+        <f aca="false">'Dr Umesh Choudhry'!E28</f>
         <v>5222229</v>
       </c>
       <c r="G11" s="7" t="n">
@@ -29305,15 +29305,24 @@
       </c>
       <c r="C38" s="79"/>
       <c r="D38" s="79"/>
-      <c r="E38" s="79"/>
+      <c r="E38" s="80" t="n">
+        <f aca="false">SUM(E7:E37)</f>
+        <v>5501448</v>
+      </c>
       <c r="F38" s="79"/>
       <c r="G38" s="79"/>
       <c r="H38" s="80" t="n">
         <f aca="false">SUM(H7:H37)</f>
         <v>5106852.5</v>
       </c>
-      <c r="I38" s="79"/>
-      <c r="J38" s="79"/>
+      <c r="I38" s="80" t="n">
+        <f aca="false">H38-E38</f>
+        <v>-394595.5</v>
+      </c>
+      <c r="J38" s="81" t="n">
+        <f aca="false">IF(E38&gt;0,I38/E38,"")</f>
+        <v>-0.071725752929047</v>
+      </c>
       <c r="K38" s="81" t="n">
         <f aca="false">SUM(K7:K37)</f>
         <v>1</v>
@@ -32813,15 +32822,24 @@
       </c>
       <c r="C60" s="82"/>
       <c r="D60" s="82"/>
-      <c r="E60" s="82"/>
+      <c r="E60" s="83" t="n">
+        <f aca="false">SUM(E7:E59)</f>
+        <v>4574421</v>
+      </c>
       <c r="F60" s="82"/>
       <c r="G60" s="82"/>
       <c r="H60" s="83" t="n">
         <f aca="false">SUM(H7:H59)</f>
         <v>4003092.54</v>
       </c>
-      <c r="I60" s="82"/>
-      <c r="J60" s="82"/>
+      <c r="I60" s="83" t="n">
+        <f aca="false">H60-E60</f>
+        <v>-571328.46</v>
+      </c>
+      <c r="J60" s="84" t="n">
+        <f aca="false">IF(E60&gt;0,I60/E60,"")</f>
+        <v>-0.12489634425865</v>
+      </c>
       <c r="K60" s="84" t="n">
         <f aca="false">SUM(K7:K59)</f>
         <v>1</v>
@@ -35483,15 +35501,24 @@
       </c>
       <c r="C54" s="85"/>
       <c r="D54" s="85"/>
-      <c r="E54" s="85"/>
+      <c r="E54" s="86" t="n">
+        <f aca="false">SUM(E7:E53)</f>
+        <v>9857778</v>
+      </c>
       <c r="F54" s="85"/>
       <c r="G54" s="85"/>
       <c r="H54" s="86" t="n">
         <f aca="false">SUM(H7:H53)</f>
         <v>11617399.07</v>
       </c>
-      <c r="I54" s="85"/>
-      <c r="J54" s="85"/>
+      <c r="I54" s="86" t="n">
+        <f aca="false">H54-E54</f>
+        <v>1759621.07</v>
+      </c>
+      <c r="J54" s="87" t="n">
+        <f aca="false">IF(E54&gt;0,I54/E54,"")</f>
+        <v>0.178500780804762</v>
+      </c>
       <c r="K54" s="87" t="n">
         <f aca="false">SUM(K7:K53)</f>
         <v>1</v>
@@ -37422,15 +37449,24 @@
       </c>
       <c r="C32" s="88"/>
       <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
+      <c r="E32" s="89" t="n">
+        <f aca="false">SUM(E7:E31)</f>
+        <v>11739506</v>
+      </c>
       <c r="F32" s="88"/>
       <c r="G32" s="88"/>
       <c r="H32" s="89" t="n">
         <f aca="false">SUM(H7:H31)</f>
         <v>11667394.24</v>
       </c>
-      <c r="I32" s="88"/>
-      <c r="J32" s="88"/>
+      <c r="I32" s="89" t="n">
+        <f aca="false">H32-E32</f>
+        <v>-72111.7599999998</v>
+      </c>
+      <c r="J32" s="90" t="n">
+        <f aca="false">IF(E32&gt;0,I32/E32,"")</f>
+        <v>-0.00614265711010325</v>
+      </c>
       <c r="K32" s="90" t="n">
         <f aca="false">SUM(K7:K31)</f>
         <v>1</v>
@@ -38570,15 +38606,24 @@
       </c>
       <c r="C19" s="91"/>
       <c r="D19" s="91"/>
-      <c r="E19" s="91"/>
+      <c r="E19" s="92" t="n">
+        <f aca="false">SUM(E7:E18)</f>
+        <v>201361</v>
+      </c>
       <c r="F19" s="91"/>
       <c r="G19" s="91"/>
       <c r="H19" s="92" t="n">
         <f aca="false">SUM(H7:H18)</f>
         <v>220563.332921147</v>
       </c>
-      <c r="I19" s="91"/>
-      <c r="J19" s="91"/>
+      <c r="I19" s="92" t="n">
+        <f aca="false">H19-E19</f>
+        <v>19202.3329211469</v>
+      </c>
+      <c r="J19" s="93" t="n">
+        <f aca="false">IF(E19&gt;0,I19/E19,"")</f>
+        <v>0.0953627212873741</v>
+      </c>
       <c r="K19" s="93" t="n">
         <f aca="false">SUM(K7:K18)</f>
         <v>1</v>
@@ -40100,15 +40145,24 @@
       </c>
       <c r="C28" s="94"/>
       <c r="D28" s="94"/>
-      <c r="E28" s="94"/>
+      <c r="E28" s="95" t="n">
+        <f aca="false">SUM(E7:E27)</f>
+        <v>5222229</v>
+      </c>
       <c r="F28" s="94"/>
       <c r="G28" s="94"/>
       <c r="H28" s="95" t="n">
         <f aca="false">SUM(H7:H27)</f>
         <v>5291042.62</v>
       </c>
-      <c r="I28" s="94"/>
-      <c r="J28" s="94"/>
+      <c r="I28" s="95" t="n">
+        <f aca="false">H28-E28</f>
+        <v>68813.6200000001</v>
+      </c>
+      <c r="J28" s="96" t="n">
+        <f aca="false">IF(E28&gt;0,I28/E28,"")</f>
+        <v>0.0131770590680723</v>
+      </c>
       <c r="K28" s="96" t="n">
         <f aca="false">SUM(K7:K27)</f>
         <v>1</v>

</xml_diff>

<commit_message>
Dr Umesh base corrected to 45,29,555
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -969,7 +969,7 @@
     <t xml:space="preserve">{"built": "28.10.2026", "close_date": "27.10.2026", "prev_date": "26.10.2026", "closes": {"Bajaj Finance Ltd": [912.0, 918.7], "Titan Company Ltd": [4365.9, 4323.0], "Poonawalla Fincorp Ltd": [402.8, 408.6], "HDFC Bank Ltd": [680.2, 688.05], "HCL Technologies Ltd": [1420.0, 1417.0], "Bajaj Housing Finance Ltd": [77.64, 78.58], "LTM Ltd (formerly LTIMindtree)": [4059.7, 4074.9], "Affle 3i Ltd": [1354.8, 1316.9], "L&amp;T Technology Services Ltd": [4174.2, 4035.6], "Fineotex Chemical Ltd": [48.31, 47.81], "AFCOM Holdings Ltd": [1314.65, 1317.65], "Connplex Cinemas Ltd": [236.8, 225.0], "Vinati Organics Ltd": [1095.3, 1057.3], "Persistent Systems Ltd": [5832.5, 5850.0], "Tata Consultancy Services Ltd": [2496.9, 2535.0], "Tata Elxsi Ltd": [3723.4, 3724.0], "Trent Ltd": [2820.6, 2754.0], "Avenue Supermarts (DMart) Ltd": [3200.0, 3150.0], "Nestle India Ltd": [1180.5, 1173.5], "Eicher Motors Ltd": [7165.0, 7099.5], "InterGlobe Aviation Ltd (IndiGo)": [4596.5, 4608.0], "Waaree Energies Ltd": [2275.0, 2319.0], "Rategain Travel Technologies Ltd": [800.4, 782.35], "Shriram Properties Ltd": [64.05, 63.79], "Bagmane Prime Office REIT": [104.25, 104.68], "Bharti Airtel Ltd": [1978.8, 1917.5], "Orient Electric Ltd": [187.44, 184.98], "Reliance Industries Ltd": [1196.2, 1201.8], "Jio Financial Services Ltd": [207.24, 205.23], "NCC Ltd": [115.41, 115.62], "Capacite Infraprojects Ltd": [149.43, 147.78], "Indus Towers Ltd": [385.3, 389.0], "Vedanta Power (VEDPOWER)": [28.96, 28.21], "Godrej Consumer Products Ltd": [828.8, 833.15], "Vedant Fashions (Manyavar) Ltd": [476.9, 481.5], "Indian Railway Finance Corp Ltd": [74.56, 74.4], "RITES Ltd": [197.67, 189.38], "Indraprastha Gas Ltd": [139.52, 141.57], "Great Eastern Shipping Co Ltd": [1550.9, 1532.4], "HUDCO Ltd": [143.33, 145.25], "NTPC Green Energy Ltd": [83.13, 81.74], "Brigade Enterprises Ltd": [552.1, 545.15], "Sonata Software Ltd": [231.45, 235.9], "Syngene International Ltd": [366.2, 359.85], "Gujarat Energy": [212.68, 215.3], "Vinyl Chemicals (India) Ltd": [257.84, 240.07], "JK Tyre &amp; Industries Ltd": [303.65, 300.4], "REC Ltd": [286.5, 298.2], "Shakti Pumps (India) Ltd": [365.8, 367.0], "Ashoka Buildcon Ltd": [97.4, 98.56], "Cyient Ltd": [1182.3, 1242.9], "Utkarsh Small Finance Bank Ltd": [11.8, 11.72], "Orient Cement Ltd": [112.83, 118.79], "Container Corporation of India Ltd": [425.15, 411.6], "GSPL Transmission Ltd": [115.24, 114.13], "Mold-Tek Technologies Ltd": [86.14, 82.04], "Ambuja Cements Ltd": [348.8, 368.0], "Indian Energy Exchange Ltd": [103.49, 103.5], "VRL Logistics Ltd": [267.55, 267.9], "Page Industries Ltd": [34610.0, 33910.0], "Central Depository Services (India) Ltd": [1222.0, 1196.0], "Aarti Drugs Ltd": [402.25, 379.35], "Tanla Platforms Ltd": [579.15, 567.8], "Eureka Forbes Ltd": [316.0, 302.9], "Garware Technical Fibres Ltd": [775.55, 721.75], "Alkyl Amines Chemicals Ltd": [1646.3, 1637.0], "Jubilant FoodWorks Ltd": [429.5, 422.9], "Vaibhav Global Ltd": [185.98, 187.63], "Asian Paints Ltd": [2277.0, 2322.0], "ICICI Prudential Life Insurance Co Ltd": [409.55, 413.35], "Eternal Ltd": [331.0, 325.55], "Kotak Mahindra Bank Ltd": [442.5, 440.75], "Clean Science and Technology Ltd": [744.0, 737.25], "Waaree Renewable Technologies Ltd": [679.45, 655.75], "Pfizer Ltd": [3709.8, 3687.2], "Infosys Ltd": [1163.0, 1166.0], "Abbott India Ltd": [25515.0, 25225.0], "Dr Lal PathLabs Ltd": [1901.8, 1855.6], "Deepak Nitrite Ltd": [1431.5, 1442.5]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Gautam refreshed from HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448 reconciles to ₹55,01,448.50). Changes vs the 05.10 statement are derived: 16 buys and 1 exit (International Gemmological Institute, 80 sh, valued at the 05.10 statement price).", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced to the 27.10.2026 close."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC statement prices 23.10.2026", "stmt_invested": 5501448.5, "stmt_mv": 5224564.0, "basis_label": "Gautam stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 1901, 1912279, 1783138, ""], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1132, 527172, 489024, ""], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "HDFC Securities", 325, 325000, 325000, ""], ["HDFC Bank Ltd", "HDFC Securities", 447, 320122, 310218, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 47, 223898, 204450, ""], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 41, 140474, 157727, ""], ["Eicher Motors Ltd", "HDFC Securities", 20, 147414, 141680, ""], ["Bajaj Housing Finance Ltd", "HDFC Securities", 1600, 132930, 129920, ""], ["L&amp;T Technology Services Ltd", "HDFC Securities", 30, 104531, 119880, ""], ["Persistent Systems Ltd", "HDFC Securities", 19, 105436, 109060, ""], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 66, 106115, 89958, ""], ["Trent Ltd", "HDFC Securities", 31, 86006, 86056, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 24, 89946, 75984, ""], ["Waaree Energies Ltd", "HDFC Securities", 27, 68363, 63990, ""], ["Rategain Travel Technologies Ltd", "HDFC Securities", 72, 59636, 56808, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 830, 46702, 43575, ""], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 10, 11941, 10970, ""], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 27, 3672, 3429, ""], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["05.10–23.10.2026", "BUY", "Affle 3i Ltd", 8, 1364.62, 10917], ["05.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3179.0, 9537], ["05.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 237, 932.3, 220956], ["05.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 274, 81.1, 22222], ["05.10–23.10.2026", "BUY", "Eicher Motors Ltd", 3, 7055.0, 21165], ["05.10–23.10.2026", "BUY", "Fineotex Chemical Ltd", 138, 52.29, 7216], ["05.10–23.10.2026", "BUY", "HDFC Bank Ltd", 57, 693.96, 39556], ["05.10–23.10.2026", "SELL", "International Gemmological Institute (India) Ltd", 80, 314.0, 25120], ["05.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 5, 3954.0, 19770], ["05.10–23.10.2026", "BUY", "Nippon India ETF Nifty 1D Rate Liquid BeES", 25, 1000.0, 25000], ["05.10–23.10.2026", "BUY", "Persistent Systems Ltd", 3, 5806.0, 17418], ["05.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 131, 432.84, 56702], ["05.10–23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 9, 789.22, 7103], ["05.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3852.57, 26968], ["05.10–23.10.2026", "BUY", "Titan Company Ltd", 6, 4349.0, 26094], ["05.10–23.10.2026", "BUY", "Trent Ltd", 3, 2787.33, 8362], ["05.10–23.10.2026", "BUY", "Waaree Energies Ltd", 3, 2367.33, 7102]], "trades_title": "Changes between 05.10 and 23.10 statements (derived; buys at implied avg cost, sells at 05.10 statement price)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base", "amount": 4184195, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems L</t>
   </si>
   <si>
-    <t xml:space="preserve">td", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 452955, "cash": [["Cash added", 436000]]}}]}</t>
+    <t xml:space="preserve">td", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
   </si>
 </sst>
 </file>
@@ -2545,15 +2545,15 @@
       </c>
       <c r="N11" s="8" t="n">
         <f aca="false">'Dr Umesh Choudhry'!E33</f>
-        <v>888955</v>
+        <v>4965555</v>
       </c>
       <c r="O11" s="8" t="n">
         <f aca="false">G11-N11</f>
-        <v>4402087.62</v>
+        <v>325487.62</v>
       </c>
       <c r="P11" s="9" t="n">
         <f aca="false">IF(N11&gt;0,O11/N11,"")</f>
-        <v>4.9519802689675</v>
+        <v>0.0655490916926708</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2603,15 +2603,15 @@
       </c>
       <c r="N12" s="18" t="n">
         <f aca="false">SUM(N6:N11)</f>
-        <v>36422107</v>
+        <v>40498707</v>
       </c>
       <c r="O12" s="18" t="n">
         <f aca="false">SUM(O6:O11)</f>
-        <v>1484237.30292115</v>
+        <v>-2592362.69707885</v>
       </c>
       <c r="P12" s="19" t="n">
         <f aca="false">IF(N12&gt;0,O12/N12,"")</f>
-        <v>0.0407510005646062</v>
+        <v>-0.064010999093844</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40741,7 +40741,7 @@
         <v>282</v>
       </c>
       <c r="E31" s="83" t="n">
-        <v>452955</v>
+        <v>4529555</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40760,7 +40760,7 @@
       <c r="D33" s="121"/>
       <c r="E33" s="122" t="n">
         <f aca="false">SUM(E31:E32)</f>
-        <v>888955</v>
+        <v>4965555</v>
       </c>
       <c r="F33" s="121"/>
     </row>
@@ -40790,11 +40790,11 @@
       <c r="D36" s="121"/>
       <c r="E36" s="122" t="n">
         <f aca="false">E35-E33</f>
-        <v>4402087.62</v>
+        <v>325487.62</v>
       </c>
       <c r="F36" s="123" t="n">
         <f aca="false">IF(E33&gt;0,E36/E33,"")</f>
-        <v>4.9519802689675</v>
+        <v>0.0655490916926708</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Base block: remove current-invested line
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1351" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1345" uniqueCount="297">
   <si>
     <t xml:space="preserve">CONSOLIDATED PORTFOLIO SUMMARY – ALL MANAGED ACCOUNTS</t>
   </si>
@@ -730,9 +730,6 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL BASE (base + cash added)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current invested (from holdings above)</t>
   </si>
   <si>
     <t xml:space="preserve">Market value</t>
@@ -3206,12 +3203,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
   </sheetData>
@@ -27468,7 +27465,7 @@
     <tabColor rgb="FF1E8449"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V46"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -29615,31 +29612,22 @@
         <v>218</v>
       </c>
       <c r="E44" s="87" t="n">
-        <f aca="false">E38</f>
-        <v>5501448</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="82" t="s">
-        <v>219</v>
-      </c>
-      <c r="E45" s="87" t="n">
         <f aca="false">H38</f>
         <v>5106852.5</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="84" t="s">
-        <v>220</v>
-      </c>
-      <c r="C46" s="85"/>
-      <c r="D46" s="85"/>
-      <c r="E46" s="86" t="n">
-        <f aca="false">E45-E43</f>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="84" t="s">
+        <v>219</v>
+      </c>
+      <c r="C45" s="85"/>
+      <c r="D45" s="85"/>
+      <c r="E45" s="86" t="n">
+        <f aca="false">E44-E43</f>
         <v>-407591.5</v>
       </c>
-      <c r="F46" s="88" t="n">
-        <f aca="false">IF(E43&gt;0,E46/E43,"")</f>
+      <c r="F45" s="88" t="n">
+        <f aca="false">IF(E43&gt;0,E45/E43,"")</f>
         <v>-0.0739134353345505</v>
       </c>
     </row>
@@ -29665,7 +29653,7 @@
     <tabColor rgb="FF2874A6"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V67"/>
+  <dimension ref="A1:V66"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -29693,12 +29681,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29708,7 +29696,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -29784,7 +29772,7 @@
         <v>82</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D7" s="66" t="n">
         <v>919</v>
@@ -29829,7 +29817,7 @@
       </c>
       <c r="O7" s="67"/>
       <c r="Q7" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R7" s="68" t="s">
         <v>206</v>
@@ -29855,7 +29843,7 @@
         <v>86</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D8" s="66" t="n">
         <v>798</v>
@@ -29900,13 +29888,13 @@
       </c>
       <c r="O8" s="67"/>
       <c r="Q8" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R8" s="68" t="s">
         <v>208</v>
       </c>
       <c r="S8" s="68" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="T8" s="68" t="n">
         <v>33</v>
@@ -29926,7 +29914,7 @@
         <v>85</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D9" s="66" t="n">
         <v>379</v>
@@ -29971,7 +29959,7 @@
       </c>
       <c r="O9" s="67"/>
       <c r="Q9" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R9" s="68" t="s">
         <v>206</v>
@@ -29997,7 +29985,7 @@
         <v>83</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D10" s="66" t="n">
         <v>59</v>
@@ -30042,7 +30030,7 @@
       </c>
       <c r="O10" s="67"/>
       <c r="Q10" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R10" s="68" t="s">
         <v>206</v>
@@ -30068,7 +30056,7 @@
         <v>92</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D11" s="66" t="n">
         <v>800</v>
@@ -30113,7 +30101,7 @@
       </c>
       <c r="O11" s="67"/>
       <c r="Q11" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R11" s="68" t="s">
         <v>206</v>
@@ -30184,7 +30172,7 @@
       </c>
       <c r="O12" s="67"/>
       <c r="Q12" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R12" s="68" t="s">
         <v>206</v>
@@ -30210,7 +30198,7 @@
         <v>87</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D13" s="66" t="n">
         <v>120</v>
@@ -30254,10 +30242,10 @@
         <v>-108</v>
       </c>
       <c r="O13" s="67" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="Q13" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R13" s="68" t="s">
         <v>206</v>
@@ -30283,7 +30271,7 @@
         <v>89</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D14" s="66" t="n">
         <v>1881</v>
@@ -30328,7 +30316,7 @@
       </c>
       <c r="O14" s="67"/>
       <c r="Q14" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R14" s="68" t="s">
         <v>206</v>
@@ -30354,7 +30342,7 @@
         <v>91</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D15" s="66" t="n">
         <v>27</v>
@@ -30399,13 +30387,13 @@
       </c>
       <c r="O15" s="67"/>
       <c r="Q15" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R15" s="68" t="s">
         <v>208</v>
       </c>
       <c r="S15" s="68" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="T15" s="68" t="n">
         <v>380</v>
@@ -30425,7 +30413,7 @@
         <v>96</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D16" s="66" t="n">
         <v>18</v>
@@ -30470,7 +30458,7 @@
       </c>
       <c r="O16" s="67"/>
       <c r="Q16" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R16" s="68" t="s">
         <v>206</v>
@@ -30541,7 +30529,7 @@
       </c>
       <c r="O17" s="67"/>
       <c r="Q17" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R17" s="68" t="s">
         <v>206</v>
@@ -30612,7 +30600,7 @@
       </c>
       <c r="O18" s="67"/>
       <c r="Q18" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R18" s="68" t="s">
         <v>206</v>
@@ -30638,7 +30626,7 @@
         <v>94</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D19" s="66" t="n">
         <v>23</v>
@@ -30683,7 +30671,7 @@
       </c>
       <c r="O19" s="67"/>
       <c r="Q19" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R19" s="68" t="s">
         <v>206</v>
@@ -30709,7 +30697,7 @@
         <v>112</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D20" s="66" t="n">
         <v>50</v>
@@ -30754,7 +30742,7 @@
       </c>
       <c r="O20" s="67"/>
       <c r="Q20" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R20" s="68" t="s">
         <v>206</v>
@@ -30780,7 +30768,7 @@
         <v>88</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D21" s="66" t="n">
         <v>26</v>
@@ -30825,7 +30813,7 @@
       </c>
       <c r="O21" s="67"/>
       <c r="Q21" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R21" s="68" t="s">
         <v>206</v>
@@ -30851,7 +30839,7 @@
         <v>98</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D22" s="66" t="n">
         <v>9</v>
@@ -30896,7 +30884,7 @@
       </c>
       <c r="O22" s="67"/>
       <c r="Q22" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R22" s="68" t="s">
         <v>206</v>
@@ -30922,7 +30910,7 @@
         <v>109</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D23" s="66" t="n">
         <v>53</v>
@@ -30967,7 +30955,7 @@
       </c>
       <c r="O23" s="67"/>
       <c r="Q23" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R23" s="68" t="s">
         <v>206</v>
@@ -30993,7 +30981,7 @@
         <v>97</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D24" s="66" t="n">
         <v>46</v>
@@ -31038,7 +31026,7 @@
       </c>
       <c r="O24" s="67"/>
       <c r="Q24" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R24" s="68" t="s">
         <v>206</v>
@@ -31109,13 +31097,13 @@
       </c>
       <c r="O25" s="67"/>
       <c r="Q25" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R25" s="68" t="s">
         <v>208</v>
       </c>
       <c r="S25" s="68" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="T25" s="68" t="n">
         <v>187</v>
@@ -31135,7 +31123,7 @@
         <v>103</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D26" s="66" t="n">
         <v>20</v>
@@ -31180,7 +31168,7 @@
       </c>
       <c r="O26" s="67"/>
       <c r="Q26" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R26" s="68" t="s">
         <v>206</v>
@@ -31206,7 +31194,7 @@
         <v>90</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D27" s="66" t="n">
         <v>12</v>
@@ -31251,7 +31239,7 @@
       </c>
       <c r="O27" s="67"/>
       <c r="Q27" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R27" s="68" t="s">
         <v>206</v>
@@ -31322,7 +31310,7 @@
       </c>
       <c r="O28" s="67"/>
       <c r="Q28" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R28" s="68" t="s">
         <v>206</v>
@@ -31348,7 +31336,7 @@
         <v>105</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D29" s="66" t="n">
         <v>14</v>
@@ -31393,7 +31381,7 @@
       </c>
       <c r="O29" s="67"/>
       <c r="Q29" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R29" s="68" t="s">
         <v>206</v>
@@ -31419,7 +31407,7 @@
         <v>122</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D30" s="66" t="n">
         <v>80</v>
@@ -31464,7 +31452,7 @@
       </c>
       <c r="O30" s="67"/>
       <c r="Q30" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R30" s="68" t="s">
         <v>206</v>
@@ -31490,7 +31478,7 @@
         <v>123</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D31" s="66" t="n">
         <v>111</v>
@@ -31535,7 +31523,7 @@
       </c>
       <c r="O31" s="67"/>
       <c r="Q31" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R31" s="68" t="s">
         <v>206</v>
@@ -31606,7 +31594,7 @@
       </c>
       <c r="O32" s="67"/>
       <c r="Q32" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R32" s="68" t="s">
         <v>206</v>
@@ -31677,7 +31665,7 @@
       </c>
       <c r="O33" s="67"/>
       <c r="Q33" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R33" s="68" t="s">
         <v>206</v>
@@ -31748,7 +31736,7 @@
       </c>
       <c r="O34" s="67"/>
       <c r="Q34" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R34" s="68" t="s">
         <v>206</v>
@@ -31819,7 +31807,7 @@
       </c>
       <c r="O35" s="67"/>
       <c r="Q35" s="68" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="R35" s="68" t="s">
         <v>206</v>
@@ -31845,7 +31833,7 @@
         <v>128</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D36" s="66" t="n">
         <v>1072</v>
@@ -31905,7 +31893,7 @@
         <v>130</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D37" s="66" t="n">
         <v>110</v>
@@ -31949,7 +31937,7 @@
         <v>-176.200000000001</v>
       </c>
       <c r="O37" s="67" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31960,7 +31948,7 @@
         <v>131</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D38" s="66" t="n">
         <v>166</v>
@@ -32013,7 +32001,7 @@
         <v>132</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D39" s="66" t="n">
         <v>116</v>
@@ -32066,7 +32054,7 @@
         <v>133</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D40" s="66" t="n">
         <v>302</v>
@@ -32119,7 +32107,7 @@
         <v>134</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D41" s="66" t="n">
         <v>245</v>
@@ -32225,7 +32213,7 @@
         <v>137</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D43" s="66" t="n">
         <v>51</v>
@@ -32331,7 +32319,7 @@
         <v>138</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D45" s="66" t="n">
         <v>124</v>
@@ -32384,7 +32372,7 @@
         <v>139</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D46" s="66" t="n">
         <v>76</v>
@@ -32437,7 +32425,7 @@
         <v>140</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D47" s="66" t="n">
         <v>49</v>
@@ -32490,7 +32478,7 @@
         <v>141</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D48" s="66" t="n">
         <v>150</v>
@@ -32543,7 +32531,7 @@
         <v>144</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D49" s="66" t="n">
         <v>54</v>
@@ -32596,7 +32584,7 @@
         <v>146</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D50" s="66" t="n">
         <v>48</v>
@@ -32649,7 +32637,7 @@
         <v>148</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D51" s="66" t="n">
         <v>132</v>
@@ -32702,7 +32690,7 @@
         <v>149</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D52" s="66" t="n">
         <v>35</v>
@@ -32755,7 +32743,7 @@
         <v>152</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D53" s="66" t="n">
         <v>9</v>
@@ -32861,7 +32849,7 @@
         <v>159</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D55" s="66" t="n">
         <v>36</v>
@@ -32914,7 +32902,7 @@
         <v>163</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D56" s="66" t="n">
         <v>20</v>
@@ -33011,7 +32999,7 @@
         <v>0</v>
       </c>
       <c r="O57" s="67" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33022,7 +33010,7 @@
         <v>167</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D58" s="66" t="n">
         <v>6</v>
@@ -33075,7 +33063,7 @@
         <v>168</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D59" s="66" t="n">
         <v>1</v>
@@ -33190,31 +33178,22 @@
         <v>218</v>
       </c>
       <c r="E65" s="87" t="n">
-        <f aca="false">E60</f>
-        <v>4574421</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B66" s="82" t="s">
-        <v>219</v>
-      </c>
-      <c r="E66" s="87" t="n">
         <f aca="false">H60</f>
         <v>4003092.54</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B67" s="92" t="s">
-        <v>220</v>
-      </c>
-      <c r="C67" s="93"/>
-      <c r="D67" s="93"/>
-      <c r="E67" s="94" t="n">
-        <f aca="false">E66-E64</f>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B66" s="92" t="s">
+        <v>219</v>
+      </c>
+      <c r="C66" s="93"/>
+      <c r="D66" s="93"/>
+      <c r="E66" s="94" t="n">
+        <f aca="false">E65-E64</f>
         <v>-181102.46</v>
       </c>
-      <c r="F67" s="95" t="n">
-        <f aca="false">IF(E64&gt;0,E67/E64,"")</f>
+      <c r="F66" s="95" t="n">
+        <f aca="false">IF(E64&gt;0,E66/E64,"")</f>
         <v>-0.0432825095388719</v>
       </c>
     </row>
@@ -33240,7 +33219,7 @@
     <tabColor rgb="FF27AE60"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:O62"/>
+  <dimension ref="A1:O61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -33262,12 +33241,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33330,7 +33309,7 @@
         <v>82</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D7" s="66" t="n">
         <v>3895</v>
@@ -33374,7 +33353,7 @@
         <v>-73660</v>
       </c>
       <c r="O7" s="67" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33385,7 +33364,7 @@
         <v>84</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D8" s="66" t="n">
         <v>11160</v>
@@ -33429,7 +33408,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="67" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33440,7 +33419,7 @@
         <v>83</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D9" s="66" t="n">
         <v>165</v>
@@ -33484,7 +33463,7 @@
         <v>19648.4999999999</v>
       </c>
       <c r="O9" s="67" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33495,7 +33474,7 @@
         <v>85</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D10" s="66" t="n">
         <v>1013</v>
@@ -33539,7 +33518,7 @@
         <v>-8900.39999999991</v>
       </c>
       <c r="O10" s="67" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33550,7 +33529,7 @@
         <v>86</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D11" s="66" t="n">
         <v>1394</v>
@@ -33594,7 +33573,7 @@
         <v>-16554.7999999999</v>
       </c>
       <c r="O11" s="67" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33605,7 +33584,7 @@
         <v>87</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D12" s="66" t="n">
         <v>360</v>
@@ -33658,7 +33637,7 @@
         <v>100</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D13" s="66" t="n">
         <v>2004.589</v>
@@ -33702,7 +33681,7 @@
         <v>0</v>
       </c>
       <c r="O13" s="67" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33713,7 +33692,7 @@
         <v>91</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D14" s="66" t="n">
         <v>72</v>
@@ -33757,7 +33736,7 @@
         <v>17954.4</v>
       </c>
       <c r="O14" s="67" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33768,7 +33747,7 @@
         <v>89</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D15" s="66" t="n">
         <v>3762</v>
@@ -33812,7 +33791,7 @@
         <v>-2.32000000000699</v>
       </c>
       <c r="O15" s="67" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33823,7 +33802,7 @@
         <v>90</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D16" s="66" t="n">
         <v>66</v>
@@ -33867,7 +33846,7 @@
         <v>-8875.79999999999</v>
       </c>
       <c r="O16" s="67" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33878,7 +33857,7 @@
         <v>92</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D17" s="66" t="n">
         <v>800</v>
@@ -33931,7 +33910,7 @@
         <v>95</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D18" s="66" t="n">
         <v>3500</v>
@@ -33984,7 +33963,7 @@
         <v>106</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D19" s="66" t="n">
         <v>134</v>
@@ -34037,7 +34016,7 @@
         <v>94</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D20" s="66" t="n">
         <v>32</v>
@@ -34081,7 +34060,7 @@
         <v>-1321.2</v>
       </c>
       <c r="O20" s="67" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34092,7 +34071,7 @@
         <v>113</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D21" s="66" t="n">
         <v>44</v>
@@ -34145,7 +34124,7 @@
         <v>114</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D22" s="66" t="n">
         <v>3</v>
@@ -34198,7 +34177,7 @@
         <v>115</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D23" s="66" t="n">
         <v>64</v>
@@ -34251,7 +34230,7 @@
         <v>88</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D24" s="66" t="n">
         <v>29</v>
@@ -34304,7 +34283,7 @@
         <v>116</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D25" s="66" t="n">
         <v>160</v>
@@ -34348,7 +34327,7 @@
         <v>1502</v>
       </c>
       <c r="O25" s="67" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34359,7 +34338,7 @@
         <v>117</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D26" s="66" t="n">
         <v>2</v>
@@ -34412,7 +34391,7 @@
         <v>96</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D27" s="66" t="n">
         <v>11</v>
@@ -34456,7 +34435,7 @@
         <v>509.5</v>
       </c>
       <c r="O27" s="67" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34467,7 +34446,7 @@
         <v>97</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D28" s="66" t="n">
         <v>47</v>
@@ -34511,7 +34490,7 @@
         <v>1421.6</v>
       </c>
       <c r="O28" s="67" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34522,7 +34501,7 @@
         <v>120</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D29" s="66" t="n">
         <v>22</v>
@@ -34575,7 +34554,7 @@
         <v>98</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D30" s="66" t="n">
         <v>6</v>
@@ -34619,7 +34598,7 @@
         <v>1230</v>
       </c>
       <c r="O30" s="67" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34630,7 +34609,7 @@
         <v>102</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D31" s="66" t="n">
         <v>32</v>
@@ -34683,7 +34662,7 @@
         <v>129</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D32" s="66" t="n">
         <v>34</v>
@@ -34736,7 +34715,7 @@
         <v>103</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D33" s="66" t="n">
         <v>10</v>
@@ -34780,7 +34759,7 @@
         <v>1076</v>
       </c>
       <c r="O33" s="67" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34791,7 +34770,7 @@
         <v>118</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D34" s="66" t="n">
         <v>168</v>
@@ -34835,7 +34814,7 @@
         <v>1205</v>
       </c>
       <c r="O34" s="67" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34846,7 +34825,7 @@
         <v>105</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D35" s="66" t="n">
         <v>6</v>
@@ -34890,7 +34869,7 @@
         <v>442</v>
       </c>
       <c r="O35" s="67" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -34901,7 +34880,7 @@
         <v>136</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D36" s="66" t="n">
         <v>33</v>
@@ -34954,7 +34933,7 @@
         <v>104</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D37" s="66" t="n">
         <v>17</v>
@@ -34998,7 +34977,7 @@
         <v>478.099999999999</v>
       </c>
       <c r="O37" s="67" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35009,7 +34988,7 @@
         <v>108</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D38" s="66" t="n">
         <v>6</v>
@@ -35053,7 +35032,7 @@
         <v>-250</v>
       </c>
       <c r="O38" s="67" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35064,7 +35043,7 @@
         <v>147</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D39" s="66" t="n">
         <v>50</v>
@@ -35117,7 +35096,7 @@
         <v>150</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D40" s="66" t="n">
         <v>34</v>
@@ -35161,7 +35140,7 @@
         <v>843</v>
       </c>
       <c r="O40" s="67" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35172,7 +35151,7 @@
         <v>151</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D41" s="66" t="n">
         <v>35</v>
@@ -35225,7 +35204,7 @@
         <v>153</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D42" s="66" t="n">
         <v>14</v>
@@ -35278,7 +35257,7 @@
         <v>110</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D43" s="66" t="n">
         <v>32</v>
@@ -35331,7 +35310,7 @@
         <v>157</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D44" s="66" t="n">
         <v>3</v>
@@ -35384,7 +35363,7 @@
         <v>107</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D45" s="66" t="n">
         <v>5</v>
@@ -35437,7 +35416,7 @@
         <v>99</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D46" s="66" t="n">
         <v>4</v>
@@ -35481,7 +35460,7 @@
         <v>-1559</v>
       </c>
       <c r="O46" s="67" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35492,7 +35471,7 @@
         <v>160</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D47" s="66" t="n">
         <v>5</v>
@@ -35545,7 +35524,7 @@
         <v>161</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D48" s="66" t="n">
         <v>1</v>
@@ -35598,7 +35577,7 @@
         <v>155</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D49" s="66" t="n">
         <v>5</v>
@@ -35642,7 +35621,7 @@
         <v>-0.75</v>
       </c>
       <c r="O49" s="67" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35653,7 +35632,7 @@
         <v>162</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D50" s="66" t="n">
         <v>6</v>
@@ -35706,7 +35685,7 @@
         <v>164</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D51" s="66" t="n">
         <v>1</v>
@@ -35759,7 +35738,7 @@
         <v>141</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D52" s="66" t="n">
         <v>12</v>
@@ -35812,7 +35791,7 @@
         <v>166</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D53" s="66" t="n">
         <v>5</v>
@@ -35904,7 +35883,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="82" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E57" s="83" t="n">
         <v>12135171</v>
@@ -35935,31 +35914,22 @@
         <v>218</v>
       </c>
       <c r="E60" s="87" t="n">
-        <f aca="false">E54</f>
-        <v>9857778</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="82" t="s">
-        <v>219</v>
-      </c>
-      <c r="E61" s="87" t="n">
         <f aca="false">H54</f>
         <v>11617399.07</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B62" s="99" t="s">
-        <v>220</v>
-      </c>
-      <c r="C62" s="100"/>
-      <c r="D62" s="100"/>
-      <c r="E62" s="101" t="n">
-        <f aca="false">E61-E59</f>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="99" t="s">
+        <v>219</v>
+      </c>
+      <c r="C61" s="100"/>
+      <c r="D61" s="100"/>
+      <c r="E61" s="101" t="n">
+        <f aca="false">E60-E59</f>
         <v>-857771.93</v>
       </c>
-      <c r="F62" s="102" t="n">
-        <f aca="false">IF(E59&gt;0,E62/E59,"")</f>
+      <c r="F61" s="102" t="n">
+        <f aca="false">IF(E59&gt;0,E61/E59,"")</f>
         <v>-0.0687583304469333</v>
       </c>
     </row>
@@ -36013,12 +35983,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36028,7 +35998,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36146,10 +36116,10 @@
         <v/>
       </c>
       <c r="O7" s="67" t="s">
+        <v>266</v>
+      </c>
+      <c r="Q7" s="68" t="s">
         <v>267</v>
-      </c>
-      <c r="Q7" s="68" t="s">
-        <v>268</v>
       </c>
       <c r="R7" s="68" t="s">
         <v>208</v>
@@ -36217,10 +36187,10 @@
         <v/>
       </c>
       <c r="O8" s="67" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="Q8" s="68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R8" s="68" t="s">
         <v>206</v>
@@ -36291,7 +36261,7 @@
       </c>
       <c r="O9" s="67"/>
       <c r="Q9" s="68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R9" s="68" t="s">
         <v>206</v>
@@ -36359,10 +36329,10 @@
         <v/>
       </c>
       <c r="O10" s="67" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="Q10" s="68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R10" s="68" t="s">
         <v>206</v>
@@ -36430,10 +36400,10 @@
         <v/>
       </c>
       <c r="O11" s="67" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="Q11" s="68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R11" s="68" t="s">
         <v>206</v>
@@ -36504,13 +36474,13 @@
       </c>
       <c r="O12" s="67"/>
       <c r="Q12" s="68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R12" s="68" t="s">
         <v>208</v>
       </c>
       <c r="S12" s="68" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="T12" s="68" t="n">
         <v>700</v>
@@ -36575,7 +36545,7 @@
       </c>
       <c r="O13" s="67"/>
       <c r="Q13" s="68" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="R13" s="68" t="s">
         <v>206</v>
@@ -36646,7 +36616,7 @@
       </c>
       <c r="O14" s="67"/>
       <c r="Q14" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R14" s="68" t="s">
         <v>206</v>
@@ -36714,10 +36684,10 @@
         <v/>
       </c>
       <c r="O15" s="67" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="Q15" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R15" s="68" t="s">
         <v>206</v>
@@ -36785,10 +36755,10 @@
         <v/>
       </c>
       <c r="O16" s="67" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Q16" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R16" s="68" t="s">
         <v>206</v>
@@ -36859,7 +36829,7 @@
       </c>
       <c r="O17" s="67"/>
       <c r="Q17" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R17" s="68" t="s">
         <v>206</v>
@@ -36927,10 +36897,10 @@
         <v/>
       </c>
       <c r="O18" s="67" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q18" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R18" s="68" t="s">
         <v>206</v>
@@ -36998,10 +36968,10 @@
         <v/>
       </c>
       <c r="O19" s="67" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="Q19" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R19" s="68" t="s">
         <v>206</v>
@@ -37072,7 +37042,7 @@
       </c>
       <c r="O20" s="67"/>
       <c r="Q20" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R20" s="68" t="s">
         <v>206</v>
@@ -37140,10 +37110,10 @@
         <v/>
       </c>
       <c r="O21" s="67" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="Q21" s="68" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="R21" s="68" t="s">
         <v>206</v>
@@ -37211,7 +37181,7 @@
         <v/>
       </c>
       <c r="O22" s="67" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Q22" s="68" t="s">
         <v>20</v>
@@ -37282,7 +37252,7 @@
         <v/>
       </c>
       <c r="O23" s="67" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q23" s="68" t="s">
         <v>20</v>
@@ -37353,7 +37323,7 @@
         <v/>
       </c>
       <c r="O24" s="67" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="Q24" s="68" t="s">
         <v>20</v>
@@ -37424,7 +37394,7 @@
         <v/>
       </c>
       <c r="O25" s="67" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="Q25" s="68" t="s">
         <v>20</v>
@@ -37495,7 +37465,7 @@
         <v/>
       </c>
       <c r="O26" s="67" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="Q26" s="68" t="s">
         <v>20</v>
@@ -37566,7 +37536,7 @@
         <v/>
       </c>
       <c r="O27" s="67" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q27" s="68" t="s">
         <v>20</v>
@@ -37637,7 +37607,7 @@
         <v/>
       </c>
       <c r="O28" s="67" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="Q28" s="68" t="s">
         <v>20</v>
@@ -37708,7 +37678,7 @@
         <v/>
       </c>
       <c r="O29" s="67" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q29" s="68" t="s">
         <v>20</v>
@@ -37779,7 +37749,7 @@
         <v/>
       </c>
       <c r="O30" s="67" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="Q30" s="68" t="s">
         <v>20</v>
@@ -37974,7 +37944,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="82" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E35" s="83" t="n">
         <v>10914339</v>
@@ -38085,8 +38055,8 @@
         <v>218</v>
       </c>
       <c r="E39" s="87" t="n">
-        <f aca="false">E32</f>
-        <v>11739506</v>
+        <f aca="false">H32</f>
+        <v>11667394.24</v>
       </c>
       <c r="Q39" s="68" t="s">
         <v>20</v>
@@ -38108,12 +38078,18 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="82" t="s">
+      <c r="B40" s="106" t="s">
         <v>219</v>
       </c>
-      <c r="E40" s="87" t="n">
-        <f aca="false">H32</f>
-        <v>11667394.24</v>
+      <c r="C40" s="107"/>
+      <c r="D40" s="107"/>
+      <c r="E40" s="108" t="n">
+        <f aca="false">E39-E38</f>
+        <v>-1464425.76</v>
+      </c>
+      <c r="F40" s="109" t="n">
+        <f aca="false">IF(E38&gt;0,E40/E38,"")</f>
+        <v>-0.11151734946108</v>
       </c>
       <c r="Q40" s="68" t="s">
         <v>20</v>
@@ -38135,19 +38111,6 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="106" t="s">
-        <v>220</v>
-      </c>
-      <c r="C41" s="107"/>
-      <c r="D41" s="107"/>
-      <c r="E41" s="108" t="n">
-        <f aca="false">E40-E38</f>
-        <v>-1464425.76</v>
-      </c>
-      <c r="F41" s="109" t="n">
-        <f aca="false">IF(E38&gt;0,E41/E38,"")</f>
-        <v>-0.11151734946108</v>
-      </c>
       <c r="Q41" s="68" t="s">
         <v>20</v>
       </c>
@@ -38278,7 +38241,7 @@
     <tabColor rgb="FF52BE80"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V27"/>
+  <dimension ref="A1:V26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -38306,12 +38269,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -38321,7 +38284,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -38442,7 +38405,7 @@
       </c>
       <c r="O7" s="67"/>
       <c r="Q7" s="68" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="R7" s="68" t="s">
         <v>206</v>
@@ -38513,7 +38476,7 @@
       </c>
       <c r="O8" s="67"/>
       <c r="Q8" s="68" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="R8" s="68" t="s">
         <v>206</v>
@@ -38584,7 +38547,7 @@
       </c>
       <c r="O9" s="67"/>
       <c r="Q9" s="68" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="R9" s="68" t="s">
         <v>206</v>
@@ -39133,7 +39096,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="82" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E22" s="83" t="n">
         <v>167022</v>
@@ -39164,31 +39127,22 @@
         <v>218</v>
       </c>
       <c r="E25" s="87" t="n">
-        <f aca="false">E19</f>
-        <v>201361</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="82" t="s">
-        <v>219</v>
-      </c>
-      <c r="E26" s="87" t="n">
         <f aca="false">H19</f>
         <v>220563.332921147</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="113" t="s">
-        <v>220</v>
-      </c>
-      <c r="C27" s="114"/>
-      <c r="D27" s="114"/>
-      <c r="E27" s="115" t="n">
-        <f aca="false">E26-E24</f>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="113" t="s">
+        <v>219</v>
+      </c>
+      <c r="C26" s="114"/>
+      <c r="D26" s="114"/>
+      <c r="E26" s="115" t="n">
+        <f aca="false">E25-E24</f>
         <v>-6958.66707885306</v>
       </c>
-      <c r="F27" s="116" t="n">
-        <f aca="false">IF(E24&gt;0,E27/E24,"")</f>
+      <c r="F26" s="116" t="n">
+        <f aca="false">IF(E24&gt;0,E26/E24,"")</f>
         <v>-0.0305845899686758</v>
       </c>
     </row>
@@ -39214,7 +39168,7 @@
     <tabColor rgb="FF5DADE2"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V36"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -39242,12 +39196,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39257,7 +39211,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -39378,7 +39332,7 @@
       </c>
       <c r="O7" s="67"/>
       <c r="Q7" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R7" s="68" t="s">
         <v>206</v>
@@ -39449,7 +39403,7 @@
       </c>
       <c r="O8" s="67"/>
       <c r="Q8" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R8" s="68" t="s">
         <v>206</v>
@@ -39520,7 +39474,7 @@
       </c>
       <c r="O9" s="67"/>
       <c r="Q9" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R9" s="68" t="s">
         <v>206</v>
@@ -39590,10 +39544,10 @@
         <v>-26484</v>
       </c>
       <c r="O10" s="67" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="Q10" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R10" s="68" t="s">
         <v>206</v>
@@ -39664,7 +39618,7 @@
       </c>
       <c r="O11" s="67"/>
       <c r="Q11" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R11" s="68" t="s">
         <v>206</v>
@@ -39734,10 +39688,10 @@
         <v>-6560</v>
       </c>
       <c r="O12" s="67" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="Q12" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R12" s="68" t="s">
         <v>206</v>
@@ -39808,7 +39762,7 @@
       </c>
       <c r="O13" s="67"/>
       <c r="Q13" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R13" s="68" t="s">
         <v>206</v>
@@ -39881,7 +39835,7 @@
         <v>207</v>
       </c>
       <c r="Q14" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R14" s="68" t="s">
         <v>206</v>
@@ -39952,7 +39906,7 @@
       </c>
       <c r="O15" s="67"/>
       <c r="Q15" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R15" s="68" t="s">
         <v>206</v>
@@ -40023,7 +39977,7 @@
       </c>
       <c r="O16" s="67"/>
       <c r="Q16" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R16" s="68" t="s">
         <v>206</v>
@@ -40094,7 +40048,7 @@
       </c>
       <c r="O17" s="67"/>
       <c r="Q17" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R17" s="68" t="s">
         <v>206</v>
@@ -40165,7 +40119,7 @@
       </c>
       <c r="O18" s="67"/>
       <c r="Q18" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R18" s="68" t="s">
         <v>206</v>
@@ -40236,7 +40190,7 @@
       </c>
       <c r="O19" s="67"/>
       <c r="Q19" s="68" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R19" s="68" t="s">
         <v>206</v>
@@ -40419,7 +40373,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="67" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40474,7 +40428,7 @@
         <v>690</v>
       </c>
       <c r="O23" s="67" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40635,7 +40589,7 @@
         <v>-323.8</v>
       </c>
       <c r="O26" s="67" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -40738,7 +40692,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="82" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E31" s="83" t="n">
         <v>4529555</v>
@@ -40769,31 +40723,22 @@
         <v>218</v>
       </c>
       <c r="E34" s="87" t="n">
-        <f aca="false">E28</f>
-        <v>5222229</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="82" t="s">
-        <v>219</v>
-      </c>
-      <c r="E35" s="87" t="n">
         <f aca="false">H28</f>
         <v>5291042.62</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="120" t="s">
-        <v>220</v>
-      </c>
-      <c r="C36" s="121"/>
-      <c r="D36" s="121"/>
-      <c r="E36" s="122" t="n">
-        <f aca="false">E35-E33</f>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="120" t="s">
+        <v>219</v>
+      </c>
+      <c r="C35" s="121"/>
+      <c r="D35" s="121"/>
+      <c r="E35" s="122" t="n">
+        <f aca="false">E34-E33</f>
         <v>325487.62</v>
       </c>
-      <c r="F36" s="123" t="n">
-        <f aca="false">IF(E33&gt;0,E36/E33,"")</f>
+      <c r="F35" s="123" t="n">
+        <f aca="false">IF(E33&gt;0,E35/E33,"")</f>
         <v>0.0655490916926708</v>
       </c>
     </row>

</xml_diff>

<commit_message>
DA base 41,11,335 (14.08.2026)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1341" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1341" uniqueCount="292">
   <si>
     <t xml:space="preserve">CONSOLIDATED PORTFOLIO SUMMARY – ALL MANAGED ACCOUNTS</t>
   </si>
@@ -756,6 +756,9 @@
     <t xml:space="preserve">Rights entitlement – nil cost</t>
   </si>
   <si>
+    <t xml:space="preserve">Base – Year 0 base (as on 14.08.2026)</t>
+  </si>
+  <si>
     <t xml:space="preserve">MANISH SHILPA – Axis Direct + HDFC Securities – 23.10.2026 (live, ~11:23 IST)</t>
   </si>
   <si>
@@ -945,10 +948,10 @@
     <t xml:space="preserve">New position 09.10.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 5997629.63, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2294.0, 2269670.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1354.0, 616306.25, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:16", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:16", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:16", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:16", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:16", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:16", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:16", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:16", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:16", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:16", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:16", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:16", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:16", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:16", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:16", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:16", "BUY", "Poonawalla Fincorp Ltd", 222.0, 401.51, 89134.25], ["28.10.2026 11:03–11:16", "BUY", "Bajaj Finance Ltd", 393.0, 909.39, 357391.0], ["28.10.2026 11:03–11:16", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base", "amount": 4184195, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed price, charges no</t>
+    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 5997629.63, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2294.0, 2269670.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1354.0, 616306.25, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:16", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:16", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:16", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:16", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:16", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:16", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:16", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:16", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:16", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:16", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:16", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:16", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:16", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:16", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:16", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:16", "BUY", "Poonawalla Fincorp Ltd", 222.0, 401.51, 89134.25], ["28.10.2026 11:03–11:16", "BUY", "Bajaj Finance Ltd", 393.0, 909.39, 357391.0], ["28.10.2026 11:03–11:16", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at execute</t>
   </si>
   <si>
-    <t xml:space="preserve">t yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
+    <t xml:space="preserve">d price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
   </si>
 </sst>
 </file>
@@ -2215,15 +2218,15 @@
       </c>
       <c r="K7" s="8" t="n">
         <f aca="false">DA!E64</f>
-        <v>4184195</v>
+        <v>4111335</v>
       </c>
       <c r="L7" s="8" t="n">
         <f aca="false">G7-K7</f>
-        <v>-212434.11</v>
+        <v>-139574.11</v>
       </c>
       <c r="M7" s="9" t="n">
         <f aca="false">IF(K7&gt;0,L7/K7,"")</f>
-        <v>-0.0507706046204825</v>
+        <v>-0.0339486103662192</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2461,15 +2464,15 @@
       </c>
       <c r="K12" s="17" t="n">
         <f aca="false">SUM(K6:K11)</f>
-        <v>40498707</v>
+        <v>40425847</v>
       </c>
       <c r="L12" s="17" t="n">
         <f aca="false">SUM(L6:L11)</f>
-        <v>-2352189.25837137</v>
+        <v>-2279329.25837137</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(K12&gt;0,L12/K12,"")</f>
-        <v>-0.0580806013972586</v>
+        <v>-0.0563829685095125</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3059,12 +3062,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -30759,10 +30762,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="75" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="E63" s="76" t="n">
-        <v>4184195</v>
+        <v>4111335</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30773,7 +30776,7 @@
       <c r="D64" s="86"/>
       <c r="E64" s="87" t="n">
         <f aca="false">SUM(E63:E63)</f>
-        <v>4184195</v>
+        <v>4111335</v>
       </c>
       <c r="F64" s="86"/>
     </row>
@@ -30794,11 +30797,11 @@
       <c r="D66" s="86"/>
       <c r="E66" s="87" t="n">
         <f aca="false">E65-E64</f>
-        <v>-212434.11</v>
+        <v>-139574.11</v>
       </c>
       <c r="F66" s="88" t="n">
         <f aca="false">IF(E64&gt;0,E66/E64,"")</f>
-        <v>-0.0507706046204825</v>
+        <v>-0.0339486103662192</v>
       </c>
     </row>
   </sheetData>
@@ -30842,12 +30845,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30901,7 +30904,7 @@
         <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D7" s="60" t="n">
         <v>3895</v>
@@ -30934,7 +30937,7 @@
         <v>0.305628125337199</v>
       </c>
       <c r="L7" s="61" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30945,7 +30948,7 @@
         <v>81</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D8" s="60" t="n">
         <v>11160</v>
@@ -30978,7 +30981,7 @@
         <v>0.247667747990467</v>
       </c>
       <c r="L8" s="61" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30989,7 +30992,7 @@
         <v>80</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D9" s="60" t="n">
         <v>165</v>
@@ -31022,7 +31025,7 @@
         <v>0.0613913539222327</v>
       </c>
       <c r="L9" s="61" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31033,7 +31036,7 @@
         <v>82</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D10" s="60" t="n">
         <v>1013</v>
@@ -31066,7 +31069,7 @@
         <v>0.0591290750864015</v>
       </c>
       <c r="L10" s="61" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31077,7 +31080,7 @@
         <v>83</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D11" s="60" t="n">
         <v>1394</v>
@@ -31110,7 +31113,7 @@
         <v>0.048249628624683</v>
       </c>
       <c r="L11" s="61" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31121,7 +31124,7 @@
         <v>84</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D12" s="60" t="n">
         <v>360</v>
@@ -31163,7 +31166,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D13" s="60" t="n">
         <v>2004.589</v>
@@ -31196,7 +31199,7 @@
         <v>0.0272662721420509</v>
       </c>
       <c r="L13" s="61" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31207,7 +31210,7 @@
         <v>86</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D14" s="60" t="n">
         <v>3762</v>
@@ -31240,7 +31243,7 @@
         <v>0.0251381588851207</v>
       </c>
       <c r="L14" s="61" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31251,7 +31254,7 @@
         <v>88</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D15" s="60" t="n">
         <v>72</v>
@@ -31284,7 +31287,7 @@
         <v>0.0251350309341946</v>
       </c>
       <c r="L15" s="61" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31295,7 +31298,7 @@
         <v>87</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D16" s="60" t="n">
         <v>66</v>
@@ -31328,7 +31331,7 @@
         <v>0.0229480070702708</v>
       </c>
       <c r="L16" s="61" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31339,7 +31342,7 @@
         <v>89</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D17" s="60" t="n">
         <v>800</v>
@@ -31381,7 +31384,7 @@
         <v>92</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D18" s="60" t="n">
         <v>3500</v>
@@ -31423,7 +31426,7 @@
         <v>102</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D19" s="60" t="n">
         <v>134</v>
@@ -31465,7 +31468,7 @@
         <v>91</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D20" s="60" t="n">
         <v>32</v>
@@ -31498,7 +31501,7 @@
         <v>0.0102404513900704</v>
       </c>
       <c r="L20" s="61" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31509,7 +31512,7 @@
         <v>108</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D21" s="60" t="n">
         <v>44</v>
@@ -31551,7 +31554,7 @@
         <v>110</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D22" s="60" t="n">
         <v>3</v>
@@ -31593,7 +31596,7 @@
         <v>111</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D23" s="60" t="n">
         <v>64</v>
@@ -31635,7 +31638,7 @@
         <v>112</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D24" s="60" t="n">
         <v>160</v>
@@ -31668,7 +31671,7 @@
         <v>0.00608714120518771</v>
       </c>
       <c r="L24" s="61" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31679,7 +31682,7 @@
         <v>85</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D25" s="60" t="n">
         <v>29</v>
@@ -31721,7 +31724,7 @@
         <v>113</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D26" s="60" t="n">
         <v>2</v>
@@ -31763,7 +31766,7 @@
         <v>94</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D27" s="60" t="n">
         <v>47</v>
@@ -31796,7 +31799,7 @@
         <v>0.00557619932630266</v>
       </c>
       <c r="L27" s="61" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31807,7 +31810,7 @@
         <v>93</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D28" s="60" t="n">
         <v>11</v>
@@ -31840,7 +31843,7 @@
         <v>0.00547590259138421</v>
       </c>
       <c r="L28" s="61" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31851,7 +31854,7 @@
         <v>116</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D29" s="60" t="n">
         <v>22</v>
@@ -31893,7 +31896,7 @@
         <v>95</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D30" s="60" t="n">
         <v>6</v>
@@ -31926,7 +31929,7 @@
         <v>0.00370918956831849</v>
       </c>
       <c r="L30" s="61" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31937,7 +31940,7 @@
         <v>99</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D31" s="60" t="n">
         <v>32</v>
@@ -31979,7 +31982,7 @@
         <v>125</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D32" s="60" t="n">
         <v>34</v>
@@ -32021,7 +32024,7 @@
         <v>98</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D33" s="60" t="n">
         <v>10</v>
@@ -32054,7 +32057,7 @@
         <v>0.00245723110063977</v>
       </c>
       <c r="L33" s="61" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32065,7 +32068,7 @@
         <v>115</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D34" s="60" t="n">
         <v>168</v>
@@ -32098,7 +32101,7 @@
         <v>0.00173943021648071</v>
       </c>
       <c r="L34" s="61" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32109,7 +32112,7 @@
         <v>131</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D35" s="60" t="n">
         <v>33</v>
@@ -32151,7 +32154,7 @@
         <v>101</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D36" s="60" t="n">
         <v>6</v>
@@ -32184,7 +32187,7 @@
         <v>0.00162669010101251</v>
       </c>
       <c r="L36" s="61" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32195,7 +32198,7 @@
         <v>100</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D37" s="60" t="n">
         <v>17</v>
@@ -32228,7 +32231,7 @@
         <v>0.00158276218875317</v>
       </c>
       <c r="L37" s="61" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32239,7 +32242,7 @@
         <v>143</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D38" s="60" t="n">
         <v>50</v>
@@ -32281,7 +32284,7 @@
         <v>104</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D39" s="60" t="n">
         <v>6</v>
@@ -32314,7 +32317,7 @@
         <v>0.00113239085765181</v>
       </c>
       <c r="L39" s="61" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32325,7 +32328,7 @@
         <v>146</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D40" s="60" t="n">
         <v>35</v>
@@ -32367,7 +32370,7 @@
         <v>147</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D41" s="60" t="n">
         <v>34</v>
@@ -32400,7 +32403,7 @@
         <v>0.000957094193811925</v>
       </c>
       <c r="L41" s="61" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32411,7 +32414,7 @@
         <v>149</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D42" s="60" t="n">
         <v>14</v>
@@ -32453,7 +32456,7 @@
         <v>107</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D43" s="60" t="n">
         <v>32</v>
@@ -32495,7 +32498,7 @@
         <v>153</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D44" s="60" t="n">
         <v>4</v>
@@ -32528,7 +32531,7 @@
         <v>0.000480604731843519</v>
       </c>
       <c r="L44" s="61" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32539,7 +32542,7 @@
         <v>154</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D45" s="60" t="n">
         <v>3</v>
@@ -32581,7 +32584,7 @@
         <v>103</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D46" s="60" t="n">
         <v>5</v>
@@ -32623,7 +32626,7 @@
         <v>157</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D47" s="60" t="n">
         <v>5</v>
@@ -32665,7 +32668,7 @@
         <v>158</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D48" s="60" t="n">
         <v>1</v>
@@ -32707,7 +32710,7 @@
         <v>151</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D49" s="60" t="n">
         <v>5</v>
@@ -32740,7 +32743,7 @@
         <v>0.000287182724950748</v>
       </c>
       <c r="L49" s="61" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32751,7 +32754,7 @@
         <v>159</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D50" s="60" t="n">
         <v>6</v>
@@ -32793,7 +32796,7 @@
         <v>161</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D51" s="60" t="n">
         <v>1</v>
@@ -32835,7 +32838,7 @@
         <v>137</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D52" s="60" t="n">
         <v>12</v>
@@ -32877,7 +32880,7 @@
         <v>163</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D53" s="60" t="n">
         <v>5</v>
@@ -32949,7 +32952,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="75" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E57" s="76" t="n">
         <v>12135171</v>
@@ -33046,12 +33049,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33061,7 +33064,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33161,10 +33164,10 @@
         <v>0.387667709233293</v>
       </c>
       <c r="L7" s="61" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Q7" s="62" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>205</v>
@@ -33223,10 +33226,10 @@
         <v>0.0930272321101565</v>
       </c>
       <c r="L8" s="61" t="s">
+        <v>263</v>
+      </c>
+      <c r="Q8" s="62" t="s">
         <v>262</v>
-      </c>
-      <c r="Q8" s="62" t="s">
-        <v>261</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -33286,7 +33289,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -33345,10 +33348,10 @@
         <v>0.0665492729486535</v>
       </c>
       <c r="L10" s="61" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="Q10" s="62" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -33407,10 +33410,10 @@
         <v>0.0663936626599383</v>
       </c>
       <c r="L11" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q11" s="62" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -33470,13 +33473,13 @@
       </c>
       <c r="L12" s="61"/>
       <c r="Q12" s="62" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>205</v>
       </c>
       <c r="S12" s="62" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="T12" s="62" t="n">
         <v>700</v>
@@ -33530,7 +33533,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -33590,7 +33593,7 @@
       </c>
       <c r="L14" s="61"/>
       <c r="Q14" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -33649,10 +33652,10 @@
         <v>0.0282483930215812</v>
       </c>
       <c r="L15" s="61" t="s">
+        <v>268</v>
+      </c>
+      <c r="Q15" s="62" t="s">
         <v>267</v>
-      </c>
-      <c r="Q15" s="62" t="s">
-        <v>266</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -33711,10 +33714,10 @@
         <v>0.0272325527669234</v>
       </c>
       <c r="L16" s="61" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="Q16" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -33774,7 +33777,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -33833,10 +33836,10 @@
         <v>0.0222301631600693</v>
       </c>
       <c r="L18" s="61" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q18" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -33895,10 +33898,10 @@
         <v>0.0208031596594696</v>
       </c>
       <c r="L19" s="61" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q19" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -33958,7 +33961,7 @@
       </c>
       <c r="L20" s="61"/>
       <c r="Q20" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R20" s="62" t="s">
         <v>201</v>
@@ -34017,10 +34020,10 @@
         <v>0.00925511581813541</v>
       </c>
       <c r="L21" s="61" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q21" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="R21" s="62" t="s">
         <v>201</v>
@@ -34079,7 +34082,7 @@
         <v>0.0064722190095489</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="Q22" s="62" t="s">
         <v>21</v>
@@ -34141,7 +34144,7 @@
         <v>0.00633173137432947</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q23" s="62" t="s">
         <v>21</v>
@@ -34203,7 +34206,7 @@
         <v>0.00565045107879498</v>
       </c>
       <c r="L24" s="61" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q24" s="62" t="s">
         <v>21</v>
@@ -34265,7 +34268,7 @@
         <v>0.00494611932858946</v>
       </c>
       <c r="L25" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q25" s="62" t="s">
         <v>21</v>
@@ -34327,7 +34330,7 @@
         <v>0.00271144248698057</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q26" s="62" t="s">
         <v>21</v>
@@ -34389,7 +34392,7 @@
         <v>0.00207627374724527</v>
       </c>
       <c r="L27" s="61" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q27" s="62" t="s">
         <v>21</v>
@@ -34451,7 +34454,7 @@
         <v>0.00196599683318886</v>
       </c>
       <c r="L28" s="61" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q28" s="62" t="s">
         <v>21</v>
@@ -34513,7 +34516,7 @@
         <v>0.000701063389415708</v>
       </c>
       <c r="L29" s="61" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q29" s="62" t="s">
         <v>21</v>
@@ -34575,7 +34578,7 @@
         <v>0.00028721368924799</v>
       </c>
       <c r="L30" s="61" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q30" s="62" t="s">
         <v>21</v>
@@ -34750,7 +34753,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="75" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E35" s="76" t="n">
         <v>10914339</v>
@@ -35072,12 +35075,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35087,7 +35090,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35188,7 +35191,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -35248,7 +35251,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -35308,7 +35311,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -35749,7 +35752,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="75" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E22" s="76" t="n">
         <v>167022</v>
@@ -35846,12 +35849,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35861,7 +35864,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35962,7 +35965,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -36022,7 +36025,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -36082,7 +36085,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -36141,10 +36144,10 @@
         <v>0.060071305630396</v>
       </c>
       <c r="L10" s="61" t="s">
+        <v>287</v>
+      </c>
+      <c r="Q10" s="62" t="s">
         <v>286</v>
-      </c>
-      <c r="Q10" s="62" t="s">
-        <v>285</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -36204,7 +36207,7 @@
       </c>
       <c r="L11" s="61"/>
       <c r="Q11" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -36263,10 +36266,10 @@
         <v>0.0360333489709902</v>
       </c>
       <c r="L12" s="61" t="s">
+        <v>287</v>
+      </c>
+      <c r="Q12" s="62" t="s">
         <v>286</v>
-      </c>
-      <c r="Q12" s="62" t="s">
-        <v>285</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>201</v>
@@ -36326,7 +36329,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -36388,7 +36391,7 @@
         <v>202</v>
       </c>
       <c r="Q14" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -36448,7 +36451,7 @@
       </c>
       <c r="L15" s="61"/>
       <c r="Q15" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -36508,7 +36511,7 @@
       </c>
       <c r="L16" s="61"/>
       <c r="Q16" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -36568,7 +36571,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -36628,7 +36631,7 @@
       </c>
       <c r="L18" s="61"/>
       <c r="Q18" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -36688,7 +36691,7 @@
       </c>
       <c r="L19" s="61"/>
       <c r="Q19" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -36838,7 +36841,7 @@
         <v>0.00684755364735877</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36882,7 +36885,7 @@
         <v>0.00408028602961991</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37010,7 +37013,7 @@
         <v>0.00121270175094724</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37093,7 +37096,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="75" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E31" s="76" t="n">
         <v>4529555</v>

</xml_diff>

<commit_message>
Gautam: Invest Right tradebook 12 (2 further buys)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -678,7 +678,7 @@
     <t xml:space="preserve">28.10 buys at executed price (charges not yet shown)</t>
   </si>
   <si>
-    <t xml:space="preserve">28.10.2026 11:03–11:16</t>
+    <t xml:space="preserve">28.10.2026 11:03–11:25</t>
   </si>
   <si>
     <t xml:space="preserve">BUY</t>
@@ -948,10 +948,10 @@
     <t xml:space="preserve">New position 09.10.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 5997629.63, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2294.0, 2269670.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1354.0, 616306.25, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:16", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:16", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:16", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:16", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:16", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:16", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:16", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:16", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:16", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:16", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:16", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:16", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:16", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:16", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:16", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:16", "BUY", "Poonawalla Fincorp Ltd", 222.0, 401.51, 89134.25], ["28.10.2026 11:03–11:16", "BUY", "Bajaj Finance Ltd", 393.0, 909.39, 357391.0], ["28.10.2026 11:03–11:16", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at execute</t>
+    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed </t>
   </si>
   <si>
-    <t xml:space="preserve">d price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
+    <t xml:space="preserve">price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
   </si>
 </sst>
 </file>
@@ -2148,23 +2148,23 @@
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">Gautam!E37</f>
-        <v>5997629.63</v>
+        <v>6000656.23</v>
       </c>
       <c r="G6" s="7" t="n">
         <f aca="false">Gautam!H37</f>
-        <v>5566468.43659864</v>
+        <v>5569484.68659864</v>
       </c>
       <c r="H6" s="8" t="n">
         <f aca="false">G6-F6</f>
-        <v>-431161.19340136</v>
+        <v>-431171.543401361</v>
       </c>
       <c r="I6" s="9" t="n">
         <f aca="false">IF(F6&gt;0,H6/F6,"")</f>
-        <v>-0.0718885993300923</v>
+        <v>-0.0718540651013698</v>
       </c>
       <c r="J6" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G6/$G$12)</f>
-        <v>0.145923370366361</v>
+        <v>0.145990896974542</v>
       </c>
       <c r="K6" s="8" t="n">
         <f aca="false">Gautam!E42</f>
@@ -2172,11 +2172,11 @@
       </c>
       <c r="L6" s="8" t="n">
         <f aca="false">G6-K6</f>
-        <v>52024.4365986399</v>
+        <v>55040.6865986399</v>
       </c>
       <c r="M6" s="9" t="n">
         <f aca="false">IF(K6&gt;0,L6/K6,"")</f>
-        <v>0.00943421251510396</v>
+        <v>0.00998118515640742</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G7/$G$12)</f>
-        <v>0.104118570321445</v>
+        <v>0.10411033830378</v>
       </c>
       <c r="K7" s="8" t="n">
         <f aca="false">DA!E64</f>
@@ -2264,7 +2264,7 @@
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G8/$G$12)</f>
-        <v>0.303217129985863</v>
+        <v>0.303193156464495</v>
       </c>
       <c r="K8" s="8" t="n">
         <f aca="false">'Manish Shilpa'!E59</f>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="J9" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G9/$G$12)</f>
-        <v>0.303184440369409</v>
+        <v>0.303160469432609</v>
       </c>
       <c r="K9" s="8" t="n">
         <f aca="false">'Saloni Mehra'!E38</f>
@@ -2364,7 +2364,7 @@
       </c>
       <c r="J10" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G10/$G$12)</f>
-        <v>0.00573651661740919</v>
+        <v>0.00573606306617443</v>
       </c>
       <c r="K10" s="8" t="n">
         <f aca="false">'Vidushi Malhotra'!E24</f>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="J11" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G11/$G$12)</f>
-        <v>0.137819972339513</v>
+        <v>0.1378090757584</v>
       </c>
       <c r="K11" s="8" t="n">
         <f aca="false">'Dr Umesh Choudhry'!E33</f>
@@ -2444,19 +2444,19 @@
       </c>
       <c r="F12" s="17" t="n">
         <f aca="false">SUM(F6:F11)</f>
-        <v>37592924.63</v>
+        <v>37595951.23</v>
       </c>
       <c r="G12" s="17" t="n">
         <f aca="false">SUM(G6:G11)</f>
-        <v>38146517.7416286</v>
+        <v>38149533.9916286</v>
       </c>
       <c r="H12" s="17" t="n">
         <f aca="false">SUM(H6:H11)</f>
-        <v>553593.111628631</v>
+        <v>553582.761628631</v>
       </c>
       <c r="I12" s="18" t="n">
         <f aca="false">IF(F12&gt;0,H12/F12,"")</f>
-        <v>0.0147259921136025</v>
+        <v>0.0147245313263119</v>
       </c>
       <c r="J12" s="18" t="n">
         <f aca="false">SUM(J6:J11)</f>
@@ -2468,11 +2468,11 @@
       </c>
       <c r="L12" s="17" t="n">
         <f aca="false">SUM(L6:L11)</f>
-        <v>-2279329.25837137</v>
+        <v>-2276313.00837137</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(K12&gt;0,L12/K12,"")</f>
-        <v>-0.0563829685095125</v>
+        <v>-0.0563083565910535</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2525,15 +2525,15 @@
       </c>
       <c r="C17" s="7" t="n">
         <f aca="false">LARGE('Side by Side'!$I$7:$I$95,A17)</f>
-        <v>13233715.6</v>
+        <v>13235530.8</v>
       </c>
       <c r="D17" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C17,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.346918051331283</v>
+        <v>0.346938203829812</v>
       </c>
       <c r="E17" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C17,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.37403147502121</v>
+        <v>0.3741548306999</v>
       </c>
       <c r="F17" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C17,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2574,11 +2574,11 @@
       </c>
       <c r="D18" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C18,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.080326157704721</v>
+        <v>0.0803198068074013</v>
       </c>
       <c r="E18" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C18,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0440683716783801</v>
+        <v>0.0440445056955191</v>
       </c>
       <c r="F18" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C18,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2619,7 +2619,7 @@
       </c>
       <c r="D19" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C19,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0751038328668904</v>
+        <v>0.0750978948668107</v>
       </c>
       <c r="E19" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C19,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2664,11 +2664,11 @@
       </c>
       <c r="D20" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C20,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0665477257241153</v>
+        <v>0.0665424642030241</v>
       </c>
       <c r="E20" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C20,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0647681926353111</v>
+        <v>0.0647331163092183</v>
       </c>
       <c r="F20" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C20,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2705,15 +2705,15 @@
       </c>
       <c r="C21" s="7" t="n">
         <f aca="false">LARGE('Side by Side'!$I$7:$I$95,A21)</f>
-        <v>2510594.85</v>
+        <v>2511795.9</v>
       </c>
       <c r="D21" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C21,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0658145224946767</v>
+        <v>0.0658408016347245</v>
       </c>
       <c r="E21" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C21,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0973820127023358</v>
+        <v>0.0975449221194978</v>
       </c>
       <c r="F21" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C21,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2754,11 +2754,11 @@
       </c>
       <c r="D22" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C22,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0413951284018981</v>
+        <v>0.0413918555426262</v>
       </c>
       <c r="E22" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C22,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0283677167666631</v>
+        <v>0.0283523537428804</v>
       </c>
       <c r="F22" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C22,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2799,11 +2799,11 @@
       </c>
       <c r="D23" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C23,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0305295809145141</v>
+        <v>0.0305271671275344</v>
       </c>
       <c r="E23" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C23,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0400164669102319</v>
+        <v>0.0399947953059256</v>
       </c>
       <c r="F23" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C23,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2844,11 +2844,11 @@
       </c>
       <c r="D24" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C24,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0288785041261532</v>
+        <v>0.0288762208797029</v>
       </c>
       <c r="E24" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C24,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0286584864024627</v>
+        <v>0.0286429659073944</v>
       </c>
       <c r="F24" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C24,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2889,11 +2889,11 @@
       </c>
       <c r="D25" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C25,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0274112045320171</v>
+        <v>0.0274090372959589</v>
       </c>
       <c r="E25" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C25,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0433492083442849</v>
+        <v>0.0433257318366677</v>
       </c>
       <c r="F25" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C25,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2934,11 +2934,11 @@
       </c>
       <c r="D26" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C26,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0263572446326545</v>
+        <v>0.0263551607267504</v>
       </c>
       <c r="E26" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C26,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0282904864715673</v>
+        <v>0.0282751652731761</v>
       </c>
       <c r="F26" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$Z$7:$Z$95,MATCH(C26,'Side by Side'!$I$7:$I$95,0))</f>
@@ -3393,19 +3393,19 @@
       <c r="G6" s="43"/>
       <c r="H6" s="43" t="n">
         <f aca="false">SUM(H7:H95)</f>
-        <v>37592924.63</v>
+        <v>37595951.23</v>
       </c>
       <c r="I6" s="43" t="n">
         <f aca="false">SUM(I7:I95)</f>
-        <v>38146517.7416286</v>
+        <v>38149533.9916286</v>
       </c>
       <c r="J6" s="43" t="n">
         <f aca="false">I6-H6</f>
-        <v>553593.111628629</v>
+        <v>553582.761628628</v>
       </c>
       <c r="K6" s="44" t="n">
         <f aca="false">IF(H6&gt;0,J6/H6,"")</f>
-        <v>0.0147259921136024</v>
+        <v>0.0147245313263119</v>
       </c>
       <c r="L6" s="44" t="n">
         <f aca="false">SUM(L7:L95)</f>
@@ -3418,19 +3418,19 @@
       <c r="N6" s="43"/>
       <c r="O6" s="43" t="n">
         <f aca="false">SUM(O7:O95)</f>
-        <v>5997629.63</v>
+        <v>6000656.23</v>
       </c>
       <c r="P6" s="43" t="n">
         <f aca="false">SUM(P7:P95)</f>
-        <v>5566468.43659864</v>
+        <v>5569484.68659864</v>
       </c>
       <c r="Q6" s="43" t="n">
         <f aca="false">P6-O6</f>
-        <v>-431161.19340136</v>
+        <v>-431171.543401361</v>
       </c>
       <c r="R6" s="44" t="n">
         <f aca="false">IF(O6&gt;0,Q6/O6,"")</f>
-        <v>-0.0718885993300923</v>
+        <v>-0.0718540651013698</v>
       </c>
       <c r="S6" s="44" t="n">
         <f aca="false">SUM(S7:S95)</f>
@@ -3583,59 +3583,59 @@
       </c>
       <c r="F7" s="47" t="n">
         <f aca="false">M7+T7+AA7+AH7+AO7+AV7</f>
-        <v>14581</v>
+        <v>14583</v>
       </c>
       <c r="G7" s="48" t="n">
         <f aca="false">IF(AND(F7&gt;0,H7&gt;0),H7/F7,"")</f>
-        <v>879.706124408477</v>
+        <v>879.710464239183</v>
       </c>
       <c r="H7" s="48" t="n">
         <f aca="false">O7+V7+AC7+AJ7+AQ7+AX7</f>
-        <v>12826995</v>
+        <v>12828817.7</v>
       </c>
       <c r="I7" s="49" t="n">
         <f aca="false">P7+W7+AD7+AK7+AR7+AY7</f>
-        <v>13233715.6</v>
+        <v>13235530.8</v>
       </c>
       <c r="J7" s="48" t="n">
         <f aca="false">I7-H7</f>
-        <v>406720.600000002</v>
+        <v>406713.100000002</v>
       </c>
       <c r="K7" s="50" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>0.0317081748297245</v>
+        <v>0.0317030851564756</v>
       </c>
       <c r="L7" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I7/I$6)</f>
-        <v>0.346918051331283</v>
+        <v>0.346938203829812</v>
       </c>
       <c r="M7" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B7)</f>
-        <v>2294</v>
+        <v>2296</v>
       </c>
       <c r="N7" s="8" t="n">
         <f aca="false">IF(AND(M7&gt;0,O7&gt;0),O7/M7,"")</f>
-        <v>989.394071490846</v>
+        <v>989.326088850174</v>
       </c>
       <c r="O7" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$E$7:$E$300,Gautam!$B$7:$B$300,$B7)</f>
-        <v>2269670</v>
+        <v>2271492.7</v>
       </c>
       <c r="P7" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$H$7:$H$300,Gautam!$B$7:$B$300,$B7)</f>
-        <v>2082034.4</v>
+        <v>2083849.6</v>
       </c>
       <c r="Q7" s="8" t="n">
         <f aca="false">P7-O7</f>
-        <v>-187635.6</v>
+        <v>-187643.1</v>
       </c>
       <c r="R7" s="9" t="n">
         <f aca="false">IF(O7&gt;0,Q7/O7,"")</f>
-        <v>-0.0826708728581688</v>
+        <v>-0.0826078375686614</v>
       </c>
       <c r="S7" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P7/P$6)</f>
-        <v>0.37403147502121</v>
+        <v>0.3741548306999</v>
       </c>
       <c r="T7" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B7)</f>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="L8" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I8/I$6)</f>
-        <v>0.080326157704721</v>
+        <v>0.0803198068074013</v>
       </c>
       <c r="M8" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B8)</f>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="S8" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P8/P$6)</f>
-        <v>0.0440683716783801</v>
+        <v>0.0440445056955191</v>
       </c>
       <c r="T8" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B8)</f>
@@ -4039,7 +4039,7 @@
       </c>
       <c r="L9" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I9/I$6)</f>
-        <v>0.0751038328668904</v>
+        <v>0.0750978948668107</v>
       </c>
       <c r="M9" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B9)</f>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="L10" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I10/I$6)</f>
-        <v>0.0665477257241153</v>
+        <v>0.0665424642030241</v>
       </c>
       <c r="M10" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B10)</f>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="S10" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P10/P$6)</f>
-        <v>0.0647681926353111</v>
+        <v>0.0647331163092183</v>
       </c>
       <c r="T10" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B10)</f>
@@ -4447,59 +4447,59 @@
       </c>
       <c r="F11" s="47" t="n">
         <f aca="false">M11+T11+AA11+AH11+AO11+AV11</f>
-        <v>6271</v>
+        <v>6274</v>
       </c>
       <c r="G11" s="48" t="n">
         <f aca="false">IF(AND(F11&gt;0,H11&gt;0),H11/F11,"")</f>
-        <v>447.799114973688</v>
+        <v>447.776880777813</v>
       </c>
       <c r="H11" s="48" t="n">
         <f aca="false">O11+V11+AC11+AJ11+AQ11+AX11</f>
-        <v>2808148.25</v>
+        <v>2809352.15</v>
       </c>
       <c r="I11" s="49" t="n">
         <f aca="false">P11+W11+AD11+AK11+AR11+AY11</f>
-        <v>2510594.85</v>
+        <v>2511795.9</v>
       </c>
       <c r="J11" s="48" t="n">
         <f aca="false">I11-H11</f>
-        <v>-297553.4</v>
+        <v>-297556.25</v>
       </c>
       <c r="K11" s="50" t="n">
         <f aca="false">IF(H11&gt;0,J11/H11,"")</f>
-        <v>-0.105960716283408</v>
+        <v>-0.105916323092497</v>
       </c>
       <c r="L11" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I11/I$6)</f>
-        <v>0.0658145224946767</v>
+        <v>0.0658408016347245</v>
       </c>
       <c r="M11" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B11)</f>
-        <v>1354</v>
+        <v>1357</v>
       </c>
       <c r="N11" s="8" t="n">
         <f aca="false">IF(AND(M11&gt;0,O11&gt;0),O11/M11,"")</f>
-        <v>455.174483013294</v>
+        <v>455.055379513633</v>
       </c>
       <c r="O11" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$E$7:$E$300,Gautam!$B$7:$B$300,$B11)</f>
-        <v>616306.25</v>
+        <v>617510.15</v>
       </c>
       <c r="P11" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$H$7:$H$300,Gautam!$B$7:$B$300,$B11)</f>
-        <v>542073.9</v>
+        <v>543274.95</v>
       </c>
       <c r="Q11" s="8" t="n">
         <f aca="false">P11-O11</f>
-        <v>-74232.35</v>
+        <v>-74235.2</v>
       </c>
       <c r="R11" s="9" t="n">
         <f aca="false">IF(O11&gt;0,Q11/O11,"")</f>
-        <v>-0.120447180277662</v>
+        <v>-0.120216971332374</v>
       </c>
       <c r="S11" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P11/P$6)</f>
-        <v>0.0973820127023358</v>
+        <v>0.0975449221194978</v>
       </c>
       <c r="T11" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B11)</f>
@@ -4687,7 +4687,7 @@
       </c>
       <c r="L12" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I12/I$6)</f>
-        <v>0.0413951284018981</v>
+        <v>0.0413918555426262</v>
       </c>
       <c r="M12" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B12)</f>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="S12" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P12/P$6)</f>
-        <v>0.0283677167666631</v>
+        <v>0.0283523537428804</v>
       </c>
       <c r="T12" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B12)</f>
@@ -4903,7 +4903,7 @@
       </c>
       <c r="L13" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I13/I$6)</f>
-        <v>0.0305295809145141</v>
+        <v>0.0305271671275344</v>
       </c>
       <c r="M13" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B13)</f>
@@ -4931,7 +4931,7 @@
       </c>
       <c r="S13" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P13/P$6)</f>
-        <v>0.0400164669102319</v>
+        <v>0.0399947953059256</v>
       </c>
       <c r="T13" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B13)</f>
@@ -5119,7 +5119,7 @@
       </c>
       <c r="L14" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I14/I$6)</f>
-        <v>0.0288785041261532</v>
+        <v>0.0288762208797029</v>
       </c>
       <c r="M14" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B14)</f>
@@ -5147,7 +5147,7 @@
       </c>
       <c r="S14" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P14/P$6)</f>
-        <v>0.0286584864024627</v>
+        <v>0.0286429659073944</v>
       </c>
       <c r="T14" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B14)</f>
@@ -5335,7 +5335,7 @@
       </c>
       <c r="L15" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I15/I$6)</f>
-        <v>0.0274112045320171</v>
+        <v>0.0274090372959589</v>
       </c>
       <c r="M15" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B15)</f>
@@ -5363,7 +5363,7 @@
       </c>
       <c r="S15" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P15/P$6)</f>
-        <v>0.0433492083442849</v>
+        <v>0.0433257318366677</v>
       </c>
       <c r="T15" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B15)</f>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="L16" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I16/I$6)</f>
-        <v>0.0263572446326545</v>
+        <v>0.0263551607267504</v>
       </c>
       <c r="M16" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B16)</f>
@@ -5579,7 +5579,7 @@
       </c>
       <c r="S16" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P16/P$6)</f>
-        <v>0.0282904864715673</v>
+        <v>0.0282751652731761</v>
       </c>
       <c r="T16" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B16)</f>
@@ -5767,7 +5767,7 @@
       </c>
       <c r="L17" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I17/I$6)</f>
-        <v>0.0248305757924094</v>
+        <v>0.0248286125908602</v>
       </c>
       <c r="M17" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B17)</f>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="S17" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P17/P$6)</f>
-        <v>0.0340323496230505</v>
+        <v>0.0340139188201438</v>
       </c>
       <c r="T17" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B17)</f>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="L18" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I18/I$6)</f>
-        <v>0.0220334659559967</v>
+        <v>0.022031723904791</v>
       </c>
       <c r="M18" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B18)</f>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="L19" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I19/I$6)</f>
-        <v>0.0190186167165733</v>
+        <v>0.019017113031032</v>
       </c>
       <c r="M19" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B19)</f>
@@ -6227,7 +6227,7 @@
       </c>
       <c r="S19" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P19/P$6)</f>
-        <v>0.0359080451594434</v>
+        <v>0.0358885985414335</v>
       </c>
       <c r="T19" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B19)</f>
@@ -6415,7 +6415,7 @@
       </c>
       <c r="L20" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I20/I$6)</f>
-        <v>0.018562417539551</v>
+        <v>0.0185609499228845</v>
       </c>
       <c r="M20" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B20)</f>
@@ -6443,7 +6443,7 @@
       </c>
       <c r="S20" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P20/P$6)</f>
-        <v>0.00959507461657976</v>
+        <v>0.00958987823927722</v>
       </c>
       <c r="T20" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B20)</f>
@@ -6631,7 +6631,7 @@
       </c>
       <c r="L21" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I21/I$6)</f>
-        <v>0.0123774338511833</v>
+        <v>0.0123764552432962</v>
       </c>
       <c r="M21" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B21)</f>
@@ -6659,7 +6659,7 @@
       </c>
       <c r="S21" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P21/P$6)</f>
-        <v>0.0237913861379807</v>
+        <v>0.0237785015045762</v>
       </c>
       <c r="T21" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B21)</f>
@@ -6847,7 +6847,7 @@
       </c>
       <c r="L22" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I22/I$6)</f>
-        <v>0.0107923350379825</v>
+        <v>0.0107914817541504</v>
       </c>
       <c r="M22" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B22)</f>
@@ -6875,7 +6875,7 @@
       </c>
       <c r="S22" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P22/P$6)</f>
-        <v>0.0194758492273504</v>
+        <v>0.0194653017470111</v>
       </c>
       <c r="T22" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B22)</f>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="L23" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I23/I$6)</f>
-        <v>0.00937241512899195</v>
+        <v>0.00937167410953051</v>
       </c>
       <c r="M23" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B23)</f>
@@ -7091,7 +7091,7 @@
       </c>
       <c r="S23" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P23/P$6)</f>
-        <v>0.030829600842013</v>
+        <v>0.0308129045426653</v>
       </c>
       <c r="T23" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B23)</f>
@@ -7279,7 +7279,7 @@
       </c>
       <c r="L24" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I24/I$6)</f>
-        <v>0.00826760078432614</v>
+        <v>0.00826694711576833</v>
       </c>
       <c r="M24" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B24)</f>
@@ -7495,7 +7495,7 @@
       </c>
       <c r="L25" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I25/I$6)</f>
-        <v>0.00746123150552741</v>
+        <v>0.00746064159164974</v>
       </c>
       <c r="M25" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B25)</f>
@@ -7711,7 +7711,7 @@
       </c>
       <c r="L26" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I26/I$6)</f>
-        <v>0.00588608904017916</v>
+        <v>0.00588562366316901</v>
       </c>
       <c r="M26" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B26)</f>
@@ -7739,7 +7739,7 @@
       </c>
       <c r="S26" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P26/P$6)</f>
-        <v>0.0183813491741492</v>
+        <v>0.0183713944390945</v>
       </c>
       <c r="T26" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B26)</f>
@@ -7927,7 +7927,7 @@
       </c>
       <c r="L27" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I27/I$6)</f>
-        <v>0.00570666768260316</v>
+        <v>0.00570621649134086</v>
       </c>
       <c r="M27" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B27)</f>
@@ -8143,7 +8143,7 @@
       </c>
       <c r="L28" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I28/I$6)</f>
-        <v>0.00539204918763886</v>
+        <v>0.00539162287133403</v>
       </c>
       <c r="M28" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B28)</f>
@@ -8171,7 +8171,7 @@
       </c>
       <c r="S28" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P28/P$6)</f>
-        <v>0.00464308749692522</v>
+        <v>0.00464057295321953</v>
       </c>
       <c r="T28" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B28)</f>
@@ -8359,7 +8359,7 @@
       </c>
       <c r="L29" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I29/I$6)</f>
-        <v>0.00517902318995698</v>
+        <v>0.00517861371631308</v>
       </c>
       <c r="M29" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B29)</f>
@@ -8387,7 +8387,7 @@
       </c>
       <c r="S29" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P29/P$6)</f>
-        <v>0.016337306325511</v>
+        <v>0.0163284585769351</v>
       </c>
       <c r="T29" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B29)</f>
@@ -8575,7 +8575,7 @@
       </c>
       <c r="L30" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I30/I$6)</f>
-        <v>0.00428593249605016</v>
+        <v>0.00428559363361755</v>
       </c>
       <c r="M30" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B30)</f>
@@ -8791,7 +8791,7 @@
       </c>
       <c r="L31" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I31/I$6)</f>
-        <v>0.00380231037030452</v>
+        <v>0.00380200974491138</v>
       </c>
       <c r="M31" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B31)</f>
@@ -8819,7 +8819,7 @@
       </c>
       <c r="S31" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P31/P$6)</f>
-        <v>0.0124557698996613</v>
+        <v>0.0124490242637409</v>
       </c>
       <c r="T31" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B31)</f>
@@ -9007,7 +9007,7 @@
       </c>
       <c r="L32" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I32/I$6)</f>
-        <v>0.00331914962350098</v>
+        <v>0.00331888719866889</v>
       </c>
       <c r="M32" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B32)</f>
@@ -9035,7 +9035,7 @@
       </c>
       <c r="S32" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P32/P$6)</f>
-        <v>0.0129415985773592</v>
+        <v>0.012934589832582</v>
       </c>
       <c r="T32" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B32)</f>
@@ -9223,7 +9223,7 @@
       </c>
       <c r="L33" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I33/I$6)</f>
-        <v>0.00252025363497558</v>
+        <v>0.00252005437395635</v>
       </c>
       <c r="M33" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B33)</f>
@@ -9251,7 +9251,7 @@
       </c>
       <c r="S33" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P33/P$6)</f>
-        <v>0.00457787559387851</v>
+        <v>0.00457539636679791</v>
       </c>
       <c r="T33" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B33)</f>
@@ -9439,7 +9439,7 @@
       </c>
       <c r="L34" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I34/I$6)</f>
-        <v>0.0024194082570028</v>
+        <v>0.00241921696920996</v>
       </c>
       <c r="M34" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B34)</f>
@@ -9467,7 +9467,7 @@
       </c>
       <c r="S34" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P34/P$6)</f>
-        <v>0.0165799916142872</v>
+        <v>0.0165710124353289</v>
       </c>
       <c r="T34" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B34)</f>
@@ -9655,7 +9655,7 @@
       </c>
       <c r="L35" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I35/I$6)</f>
-        <v>0.0024117871157503</v>
+        <v>0.00241159643051442</v>
       </c>
       <c r="M35" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B35)</f>
@@ -9871,7 +9871,7 @@
       </c>
       <c r="L36" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I36/I$6)</f>
-        <v>0.00222892166923045</v>
+        <v>0.00222874544204544</v>
       </c>
       <c r="M36" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B36)</f>
@@ -10087,7 +10087,7 @@
       </c>
       <c r="L37" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I37/I$6)</f>
-        <v>0.00214027923998166</v>
+        <v>0.00214011002121063</v>
       </c>
       <c r="M37" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B37)</f>
@@ -10303,7 +10303,7 @@
       </c>
       <c r="L38" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I38/I$6)</f>
-        <v>0.00204671368770309</v>
+        <v>0.00204655186658722</v>
       </c>
       <c r="M38" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B38)</f>
@@ -10519,7 +10519,7 @@
       </c>
       <c r="L39" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I39/I$6)</f>
-        <v>0.00185977657201931</v>
+        <v>0.00185962953087625</v>
       </c>
       <c r="M39" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B39)</f>
@@ -10735,7 +10735,7 @@
       </c>
       <c r="L40" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I40/I$6)</f>
-        <v>0.0018457254860557</v>
+        <v>0.00184557955584595</v>
       </c>
       <c r="M40" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B40)</f>
@@ -10951,7 +10951,7 @@
       </c>
       <c r="L41" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I41/I$6)</f>
-        <v>0.00176503660061542</v>
+        <v>0.00176489704998165</v>
       </c>
       <c r="M41" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B41)</f>
@@ -11167,7 +11167,7 @@
       </c>
       <c r="L42" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I42/I$6)</f>
-        <v>0.00157607570911748</v>
+        <v>0.00157595109846408</v>
       </c>
       <c r="M42" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B42)</f>
@@ -11383,7 +11383,7 @@
       </c>
       <c r="L43" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I43/I$6)</f>
-        <v>0.00157599624465529</v>
+        <v>0.00157587164028465</v>
       </c>
       <c r="M43" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B43)</f>
@@ -11411,7 +11411,7 @@
       </c>
       <c r="S43" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P43/P$6)</f>
-        <v>0.000623913822236924</v>
+        <v>0.000623575931000622</v>
       </c>
       <c r="T43" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B43)</f>
@@ -11599,7 +11599,7 @@
       </c>
       <c r="L44" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I44/I$6)</f>
-        <v>0.00130310714956174</v>
+        <v>0.0013030041208605</v>
       </c>
       <c r="M44" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B44)</f>
@@ -11815,7 +11815,7 @@
       </c>
       <c r="L45" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I45/I$6)</f>
-        <v>0.00124473327609098</v>
+        <v>0.0012446348626544</v>
       </c>
       <c r="M45" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B45)</f>
@@ -12031,7 +12031,7 @@
       </c>
       <c r="L46" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I46/I$6)</f>
-        <v>0.00112503060674308</v>
+        <v>0.00112494165746343</v>
       </c>
       <c r="M46" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B46)</f>
@@ -12247,7 +12247,7 @@
       </c>
       <c r="L47" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I47/I$6)</f>
-        <v>0.00110239027018996</v>
+        <v>0.00110230311094305</v>
       </c>
       <c r="M47" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B47)</f>
@@ -12463,7 +12463,7 @@
       </c>
       <c r="L48" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I48/I$6)</f>
-        <v>0.00100304044157207</v>
+        <v>0.00100296113730763</v>
       </c>
       <c r="M48" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B48)</f>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="L49" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I49/I$6)</f>
-        <v>0.000943729654272317</v>
+        <v>0.000943655039348572</v>
       </c>
       <c r="M49" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B49)</f>
@@ -12895,7 +12895,7 @@
       </c>
       <c r="L50" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I50/I$6)</f>
-        <v>0.000897956144568848</v>
+        <v>0.000897885148676168</v>
       </c>
       <c r="M50" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B50)</f>
@@ -13111,7 +13111,7 @@
       </c>
       <c r="L51" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I51/I$6)</f>
-        <v>0.000857430820331637</v>
+        <v>0.000857363028528142</v>
       </c>
       <c r="M51" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B51)</f>
@@ -13327,7 +13327,7 @@
       </c>
       <c r="L52" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I52/I$6)</f>
-        <v>0.000807094377749762</v>
+        <v>0.000807030565740487</v>
       </c>
       <c r="M52" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B52)</f>
@@ -13543,7 +13543,7 @@
       </c>
       <c r="L53" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I53/I$6)</f>
-        <v>0.000781696515576284</v>
+        <v>0.000781634711620419</v>
       </c>
       <c r="M53" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B53)</f>
@@ -13759,7 +13759,7 @@
       </c>
       <c r="L54" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I54/I$6)</f>
-        <v>0.000614234309896923</v>
+        <v>0.000614185746152013</v>
       </c>
       <c r="M54" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B54)</f>
@@ -13975,7 +13975,7 @@
       </c>
       <c r="L55" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I55/I$6)</f>
-        <v>0.000613028433116464</v>
+        <v>0.000612979964712845</v>
       </c>
       <c r="M55" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B55)</f>
@@ -14191,7 +14191,7 @@
       </c>
       <c r="L56" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I56/I$6)</f>
-        <v>0.000589692620237572</v>
+        <v>0.000589645996853753</v>
       </c>
       <c r="M56" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B56)</f>
@@ -14407,7 +14407,7 @@
       </c>
       <c r="L57" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I57/I$6)</f>
-        <v>0.000583946355231558</v>
+        <v>0.00058390018616972</v>
       </c>
       <c r="M57" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B57)</f>
@@ -14623,7 +14623,7 @@
       </c>
       <c r="L58" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I58/I$6)</f>
-        <v>0.00053256237273344</v>
+        <v>0.000532520266288389</v>
       </c>
       <c r="M58" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B58)</f>
@@ -14839,7 +14839,7 @@
       </c>
       <c r="L59" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I59/I$6)</f>
-        <v>0.00051351476254471</v>
+        <v>0.000513474162077536</v>
       </c>
       <c r="M59" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B59)</f>
@@ -15055,7 +15055,7 @@
       </c>
       <c r="L60" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I60/I$6)</f>
-        <v>0.000510648183719858</v>
+        <v>0.000510607809895515</v>
       </c>
       <c r="M60" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B60)</f>
@@ -15271,7 +15271,7 @@
       </c>
       <c r="L61" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I61/I$6)</f>
-        <v>0.000501167632901314</v>
+        <v>0.000501128008646059</v>
       </c>
       <c r="M61" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B61)</f>
@@ -15487,7 +15487,7 @@
       </c>
       <c r="L62" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I62/I$6)</f>
-        <v>0.000469747726945074</v>
+        <v>0.000469710586869347</v>
       </c>
       <c r="M62" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B62)</f>
@@ -15703,7 +15703,7 @@
       </c>
       <c r="L63" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I63/I$6)</f>
-        <v>0.000451894459063252</v>
+        <v>0.000451858730536071</v>
       </c>
       <c r="M63" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B63)</f>
@@ -15919,7 +15919,7 @@
       </c>
       <c r="L64" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I64/I$6)</f>
-        <v>0.000449865440306566</v>
+        <v>0.000449829872201472</v>
       </c>
       <c r="M64" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B64)</f>
@@ -16135,7 +16135,7 @@
       </c>
       <c r="L65" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I65/I$6)</f>
-        <v>0.000433002039973225</v>
+        <v>0.000432967805153912</v>
       </c>
       <c r="M65" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B65)</f>
@@ -16351,7 +16351,7 @@
       </c>
       <c r="L66" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I66/I$6)</f>
-        <v>0.000412881723744139</v>
+        <v>0.000412849079715</v>
       </c>
       <c r="M66" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B66)</f>
@@ -16379,7 +16379,7 @@
       </c>
       <c r="S66" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P66/P$6)</f>
-        <v>0.0028294420743404</v>
+        <v>0.00282790974143404</v>
       </c>
       <c r="T66" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B66)</f>
@@ -16567,7 +16567,7 @@
       </c>
       <c r="L67" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I67/I$6)</f>
-        <v>0.000410239280712176</v>
+        <v>0.000410206845604824</v>
       </c>
       <c r="M67" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B67)</f>
@@ -16783,7 +16783,7 @@
       </c>
       <c r="L68" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I68/I$6)</f>
-        <v>0.000409342737540618</v>
+        <v>0.000409310373317443</v>
       </c>
       <c r="M68" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B68)</f>
@@ -16811,7 +16811,7 @@
       </c>
       <c r="S68" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P68/P$6)</f>
-        <v>0.00280518971370319</v>
+        <v>0.00280367051507889</v>
       </c>
       <c r="T68" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B68)</f>
@@ -16999,7 +16999,7 @@
       </c>
       <c r="L69" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I69/I$6)</f>
-        <v>0.000393377977555844</v>
+        <v>0.000393346875568463</v>
       </c>
       <c r="M69" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B69)</f>
@@ -17027,7 +17027,7 @@
       </c>
       <c r="S69" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P69/P$6)</f>
-        <v>0.0026736880249148</v>
+        <v>0.00267224004328653</v>
       </c>
       <c r="T69" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B69)</f>
@@ -17215,7 +17215,7 @@
       </c>
       <c r="L70" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I70/I$6)</f>
-        <v>0.00037988264349975</v>
+        <v>0.000379852608505779</v>
       </c>
       <c r="M70" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B70)</f>
@@ -17431,7 +17431,7 @@
       </c>
       <c r="L71" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I71/I$6)</f>
-        <v>0.000351277149090251</v>
+        <v>0.000351249375757524</v>
       </c>
       <c r="M71" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B71)</f>
@@ -17647,7 +17647,7 @@
       </c>
       <c r="L72" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I72/I$6)</f>
-        <v>0.000336223350368977</v>
+        <v>0.000336196767247915</v>
       </c>
       <c r="M72" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B72)</f>
@@ -17863,7 +17863,7 @@
       </c>
       <c r="L73" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I73/I$6)</f>
-        <v>0.000333473164868152</v>
+        <v>0.000333446799187414</v>
       </c>
       <c r="M73" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B73)</f>
@@ -18079,7 +18079,7 @@
       </c>
       <c r="L74" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I74/I$6)</f>
-        <v>0.00029025585179213</v>
+        <v>0.000290232903039645</v>
       </c>
       <c r="M74" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B74)</f>
@@ -18295,7 +18295,7 @@
       </c>
       <c r="L75" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I75/I$6)</f>
-        <v>0.000290207354573785</v>
+        <v>0.000290184409655679</v>
       </c>
       <c r="M75" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B75)</f>
@@ -18511,7 +18511,7 @@
       </c>
       <c r="L76" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I76/I$6)</f>
-        <v>0.000273044582222338</v>
+        <v>0.000273022994259526</v>
       </c>
       <c r="M76" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B76)</f>
@@ -18727,7 +18727,7 @@
       </c>
       <c r="L77" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I77/I$6)</f>
-        <v>0.000270354952707662</v>
+        <v>0.000270333577397382</v>
       </c>
       <c r="M77" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B77)</f>
@@ -18943,7 +18943,7 @@
       </c>
       <c r="L78" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I78/I$6)</f>
-        <v>0.000255174012630187</v>
+        <v>0.000255153837583861</v>
       </c>
       <c r="M78" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B78)</f>
@@ -18971,7 +18971,7 @@
       </c>
       <c r="S78" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P78/P$6)</f>
-        <v>0.00174868502550028</v>
+        <v>0.00174773799511866</v>
       </c>
       <c r="T78" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B78)</f>
@@ -19159,7 +19159,7 @@
       </c>
       <c r="L79" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I79/I$6)</f>
-        <v>0.000174157443282171</v>
+        <v>0.000174143673719784</v>
       </c>
       <c r="M79" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B79)</f>
@@ -19375,7 +19375,7 @@
       </c>
       <c r="L80" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I80/I$6)</f>
-        <v>0.000173667228156201</v>
+        <v>0.000173653497352123</v>
       </c>
       <c r="M80" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B80)</f>
@@ -19591,7 +19591,7 @@
       </c>
       <c r="L81" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I81/I$6)</f>
-        <v>0.000145727587447217</v>
+        <v>0.000145716065659409</v>
       </c>
       <c r="M81" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B81)</f>
@@ -19807,7 +19807,7 @@
       </c>
       <c r="L82" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I82/I$6)</f>
-        <v>0.000130116726082796</v>
+        <v>0.000130106438550184</v>
       </c>
       <c r="M82" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B82)</f>
@@ -20023,7 +20023,7 @@
       </c>
       <c r="L83" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I83/I$6)</f>
-        <v>0.000122193329193801</v>
+        <v>0.000122183668115654</v>
       </c>
       <c r="M83" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B83)</f>
@@ -20051,7 +20051,7 @@
       </c>
       <c r="S83" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P83/P$6)</f>
-        <v>0.000837380118667884</v>
+        <v>0.000836926621095836</v>
       </c>
       <c r="T83" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B83)</f>
@@ -20239,7 +20239,7 @@
       </c>
       <c r="L84" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I84/I$6)</f>
-        <v>0.000113247558512678</v>
+        <v>0.000113238604721829</v>
       </c>
       <c r="M84" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B84)</f>
@@ -20455,7 +20455,7 @@
       </c>
       <c r="L85" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I85/I$6)</f>
-        <v>9.81544377224757E-005</v>
+        <v>9.8146677252247E-005</v>
       </c>
       <c r="M85" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B85)</f>
@@ -20671,7 +20671,7 @@
       </c>
       <c r="L86" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I86/I$6)</f>
-        <v>9.76550474470899E-005</v>
+        <v>9.76473264605917E-005</v>
       </c>
       <c r="M86" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B86)</f>
@@ -20887,7 +20887,7 @@
       </c>
       <c r="L87" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I87/I$6)</f>
-        <v>7.09370123461358E-005</v>
+        <v>7.09314037910343E-005</v>
       </c>
       <c r="M87" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B87)</f>
@@ -21103,7 +21103,7 @@
       </c>
       <c r="L88" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I88/I$6)</f>
-        <v>5.93238946560626E-005</v>
+        <v>5.93192042790505E-005</v>
       </c>
       <c r="M88" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B88)</f>
@@ -21319,7 +21319,7 @@
       </c>
       <c r="L89" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I89/I$6)</f>
-        <v>3.84989269517868E-005</v>
+        <v>3.84958830774254E-005</v>
       </c>
       <c r="M89" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B89)</f>
@@ -21535,7 +21535,7 @@
       </c>
       <c r="L90" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I90/I$6)</f>
-        <v>3.23751700840642E-005</v>
+        <v>3.23726103776524E-005</v>
       </c>
       <c r="M90" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B90)</f>
@@ -21751,7 +21751,7 @@
       </c>
       <c r="L91" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I91/I$6)</f>
-        <v>2.44727449651645E-005</v>
+        <v>2.44708100551072E-005</v>
       </c>
       <c r="M91" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B91)</f>
@@ -21967,7 +21967,7 @@
       </c>
       <c r="L92" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I92/I$6)</f>
-        <v>1.41229142761852E-005</v>
+        <v>1.41217976638514E-005</v>
       </c>
       <c r="M92" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B92)</f>
@@ -22183,7 +22183,7 @@
       </c>
       <c r="L93" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I93/I$6)</f>
-        <v>1.08607554379173E-005</v>
+        <v>1.08598967445032E-005</v>
       </c>
       <c r="M93" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B93)</f>
@@ -26134,14 +26134,14 @@
         <v>16</v>
       </c>
       <c r="D7" s="60" t="n">
-        <v>2294</v>
+        <v>2296</v>
       </c>
       <c r="E7" s="57" t="n">
-        <v>2269670</v>
+        <v>2271492.7</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">IF(AND(D7&gt;0,N(E7)&gt;0),E7/D7,"")</f>
-        <v>989.394071490846</v>
+        <v>989.326088850174</v>
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH(B7,Prices!$A$6:$A$300,0)),"")</f>
@@ -26149,19 +26149,19 @@
       </c>
       <c r="H7" s="8" t="n">
         <f aca="false">IF(ISNUMBER(G7),D7*G7,0)</f>
-        <v>2082034.4</v>
+        <v>2083849.6</v>
       </c>
       <c r="I7" s="8" t="n">
         <f aca="false">H7-N(E7)</f>
-        <v>-187635.6</v>
+        <v>-187643.1</v>
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">IF(N(E7)&gt;0,I7/E7,"")</f>
-        <v>-0.0826708728581688</v>
+        <v>-0.0826078375686614</v>
       </c>
       <c r="K7" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H7/$H$37)</f>
-        <v>0.37403147502121</v>
+        <v>0.3741548306999</v>
       </c>
       <c r="L7" s="61" t="s">
         <v>199</v>
@@ -26196,14 +26196,14 @@
         <v>16</v>
       </c>
       <c r="D8" s="60" t="n">
-        <v>1354</v>
+        <v>1357</v>
       </c>
       <c r="E8" s="57" t="n">
-        <v>616306.25</v>
+        <v>617510.15</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">IF(AND(D8&gt;0,N(E8)&gt;0),E8/D8,"")</f>
-        <v>455.174483013294</v>
+        <v>455.055379513633</v>
       </c>
       <c r="G8" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH(B8,Prices!$A$6:$A$300,0)),"")</f>
@@ -26211,19 +26211,19 @@
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">IF(ISNUMBER(G8),D8*G8,0)</f>
-        <v>542073.9</v>
+        <v>543274.95</v>
       </c>
       <c r="I8" s="8" t="n">
         <f aca="false">H8-N(E8)</f>
-        <v>-74232.35</v>
+        <v>-74235.2</v>
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">IF(N(E8)&gt;0,I8/E8,"")</f>
-        <v>-0.120447180277662</v>
+        <v>-0.120216971332374</v>
       </c>
       <c r="K8" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H8/$H$37)</f>
-        <v>0.0973820127023358</v>
+        <v>0.0975449221194978</v>
       </c>
       <c r="L8" s="61" t="s">
         <v>199</v>
@@ -26285,7 +26285,7 @@
       </c>
       <c r="K9" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H9/$H$37)</f>
-        <v>0.0647681926353111</v>
+        <v>0.0647331163092183</v>
       </c>
       <c r="L9" s="61" t="s">
         <v>199</v>
@@ -26347,7 +26347,7 @@
       </c>
       <c r="K10" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H10/$H$37)</f>
-        <v>0.0440683716783801</v>
+        <v>0.0440445056955191</v>
       </c>
       <c r="L10" s="61" t="s">
         <v>199</v>
@@ -26409,7 +26409,7 @@
       </c>
       <c r="K11" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H11/$H$37)</f>
-        <v>0.0433492083442849</v>
+        <v>0.0433257318366677</v>
       </c>
       <c r="L11" s="61" t="s">
         <v>202</v>
@@ -26471,7 +26471,7 @@
       </c>
       <c r="K12" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H12/$H$37)</f>
-        <v>0.0400164669102319</v>
+        <v>0.0399947953059256</v>
       </c>
       <c r="L12" s="61"/>
       <c r="Q12" s="62" t="s">
@@ -26531,7 +26531,7 @@
       </c>
       <c r="K13" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H13/$H$37)</f>
-        <v>0.0359080451594434</v>
+        <v>0.0358885985414335</v>
       </c>
       <c r="L13" s="61" t="s">
         <v>199</v>
@@ -26593,7 +26593,7 @@
       </c>
       <c r="K14" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H14/$H$37)</f>
-        <v>0.0340323496230505</v>
+        <v>0.0340139188201438</v>
       </c>
       <c r="L14" s="61"/>
       <c r="Q14" s="62" t="s">
@@ -26653,7 +26653,7 @@
       </c>
       <c r="K15" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H15/$H$37)</f>
-        <v>0.030829600842013</v>
+        <v>0.0308129045426653</v>
       </c>
       <c r="L15" s="61" t="s">
         <v>199</v>
@@ -26715,7 +26715,7 @@
       </c>
       <c r="K16" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H16/$H$37)</f>
-        <v>0.0286584864024627</v>
+        <v>0.0286429659073944</v>
       </c>
       <c r="L16" s="61" t="s">
         <v>199</v>
@@ -26777,7 +26777,7 @@
       </c>
       <c r="K17" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H17/$H$37)</f>
-        <v>0.0283677167666631</v>
+        <v>0.0283523537428804</v>
       </c>
       <c r="L17" s="61" t="s">
         <v>203</v>
@@ -26839,7 +26839,7 @@
       </c>
       <c r="K18" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H18/$H$37)</f>
-        <v>0.0282904864715673</v>
+        <v>0.0282751652731761</v>
       </c>
       <c r="L18" s="61" t="s">
         <v>199</v>
@@ -26901,7 +26901,7 @@
       </c>
       <c r="K19" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H19/$H$37)</f>
-        <v>0.0237913861379807</v>
+        <v>0.0237785015045762</v>
       </c>
       <c r="L19" s="61" t="s">
         <v>199</v>
@@ -26963,7 +26963,7 @@
       </c>
       <c r="K20" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H20/$H$37)</f>
-        <v>0.0194758492273504</v>
+        <v>0.0194653017470111</v>
       </c>
       <c r="L20" s="61" t="s">
         <v>199</v>
@@ -27025,7 +27025,7 @@
       </c>
       <c r="K21" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H21/$H$37)</f>
-        <v>0.0183813491741492</v>
+        <v>0.0183713944390945</v>
       </c>
       <c r="L21" s="61" t="s">
         <v>199</v>
@@ -27087,7 +27087,7 @@
       </c>
       <c r="K22" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H22/$H$37)</f>
-        <v>0.0165799916142872</v>
+        <v>0.0165710124353289</v>
       </c>
       <c r="L22" s="61" t="s">
         <v>204</v>
@@ -27102,13 +27102,13 @@
         <v>83</v>
       </c>
       <c r="T22" s="62" t="n">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="U22" s="57" t="n">
-        <v>401.51</v>
+        <v>401.5</v>
       </c>
       <c r="V22" s="57" t="n">
-        <v>89134.25</v>
+        <v>90338.15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27149,7 +27149,7 @@
       </c>
       <c r="K23" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H23/$H$37)</f>
-        <v>0.016337306325511</v>
+        <v>0.0163284585769351</v>
       </c>
       <c r="L23" s="61" t="s">
         <v>199</v>
@@ -27164,13 +27164,13 @@
         <v>79</v>
       </c>
       <c r="T23" s="62" t="n">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="U23" s="57" t="n">
-        <v>909.39</v>
+        <v>909.4</v>
       </c>
       <c r="V23" s="57" t="n">
-        <v>357391</v>
+        <v>359213.7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27211,7 +27211,7 @@
       </c>
       <c r="K24" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H24/$H$37)</f>
-        <v>0.0129415985773592</v>
+        <v>0.012934589832582</v>
       </c>
       <c r="L24" s="61" t="s">
         <v>199</v>
@@ -27273,7 +27273,7 @@
       </c>
       <c r="K25" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H25/$H$37)</f>
-        <v>0.0124557698996613</v>
+        <v>0.0124490242637409</v>
       </c>
       <c r="L25" s="61" t="s">
         <v>199</v>
@@ -27283,7 +27283,7 @@
       </c>
       <c r="V25" s="64" t="n">
         <f aca="false">SUMIFS(V7:V24,R7:R24,"BUY")-SUMIFS(V7:V24,R7:R24,"SELL")</f>
-        <v>496184.88</v>
+        <v>499211.48</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27324,7 +27324,7 @@
       </c>
       <c r="K26" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H26/$H$37)</f>
-        <v>0.00959507461657976</v>
+        <v>0.00958987823927722</v>
       </c>
       <c r="L26" s="61" t="s">
         <v>199</v>
@@ -27368,7 +27368,7 @@
       </c>
       <c r="K27" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H27/$H$37)</f>
-        <v>0.00464308749692522</v>
+        <v>0.00464057295321953</v>
       </c>
       <c r="L27" s="61" t="s">
         <v>199</v>
@@ -27412,7 +27412,7 @@
       </c>
       <c r="K28" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H28/$H$37)</f>
-        <v>0.00457787559387851</v>
+        <v>0.00457539636679791</v>
       </c>
       <c r="L28" s="61"/>
     </row>
@@ -27454,7 +27454,7 @@
       </c>
       <c r="K29" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H29/$H$37)</f>
-        <v>0.0028294420743404</v>
+        <v>0.00282790974143404</v>
       </c>
       <c r="L29" s="61"/>
     </row>
@@ -27496,7 +27496,7 @@
       </c>
       <c r="K30" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H30/$H$37)</f>
-        <v>0.00280518971370319</v>
+        <v>0.00280367051507889</v>
       </c>
       <c r="L30" s="61"/>
     </row>
@@ -27538,7 +27538,7 @@
       </c>
       <c r="K31" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H31/$H$37)</f>
-        <v>0.0026736880249148</v>
+        <v>0.00267224004328653</v>
       </c>
       <c r="L31" s="61"/>
     </row>
@@ -27580,7 +27580,7 @@
       </c>
       <c r="K32" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H32/$H$37)</f>
-        <v>0.00174868502550028</v>
+        <v>0.00174773799511866</v>
       </c>
       <c r="L32" s="61"/>
     </row>
@@ -27622,7 +27622,7 @@
       </c>
       <c r="K33" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H33/$H$37)</f>
-        <v>0.000837380118667884</v>
+        <v>0.000836926621095836</v>
       </c>
       <c r="L33" s="61"/>
     </row>
@@ -27664,7 +27664,7 @@
       </c>
       <c r="K34" s="9" t="n">
         <f aca="false">IF($H$37=0,"",H34/$H$37)</f>
-        <v>0.000623913822236924</v>
+        <v>0.000623575931000622</v>
       </c>
       <c r="L34" s="61" t="s">
         <v>199</v>
@@ -27763,21 +27763,21 @@
       <c r="D37" s="72"/>
       <c r="E37" s="73" t="n">
         <f aca="false">SUM(E7:E36)</f>
-        <v>5997629.63</v>
+        <v>6000656.23</v>
       </c>
       <c r="F37" s="72"/>
       <c r="G37" s="72"/>
       <c r="H37" s="73" t="n">
         <f aca="false">SUM(H7:H36)</f>
-        <v>5566468.43659864</v>
+        <v>5569484.68659864</v>
       </c>
       <c r="I37" s="73" t="n">
         <f aca="false">H37-E37</f>
-        <v>-431161.19340136</v>
+        <v>-431171.543401361</v>
       </c>
       <c r="J37" s="74" t="n">
         <f aca="false">IF(E37&gt;0,I37/E37,"")</f>
-        <v>-0.0718885993300923</v>
+        <v>-0.0718540651013698</v>
       </c>
       <c r="K37" s="74" t="n">
         <f aca="false">SUM(K7:K36)</f>
@@ -27824,7 +27824,7 @@
       </c>
       <c r="E43" s="80" t="n">
         <f aca="false">H37</f>
-        <v>5566468.43659864</v>
+        <v>5569484.68659864</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27835,11 +27835,11 @@
       <c r="D44" s="78"/>
       <c r="E44" s="79" t="n">
         <f aca="false">E43-E42</f>
-        <v>52024.4365986399</v>
+        <v>55040.6865986399</v>
       </c>
       <c r="F44" s="81" t="n">
         <f aca="false">IF(E42&gt;0,E44/E42,"")</f>
-        <v>0.00943421251510396</v>
+        <v>0.00998118515640742</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Gautam base: cash added 5,00,000 on 28.10.2026
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1341" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="293">
   <si>
     <t xml:space="preserve">CONSOLIDATED PORTFOLIO SUMMARY – ALL MANAGED ACCOUNTS</t>
   </si>
@@ -711,6 +711,9 @@
     <t xml:space="preserve">+ Cash added</t>
   </si>
   <si>
+    <t xml:space="preserve">+ Cash added 28.10.2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOTAL BASE (base + cash added)</t>
   </si>
   <si>
@@ -948,10 +951,10 @@
     <t xml:space="preserve">New position 09.10.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed </t>
+    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges include</t>
   </si>
   <si>
-    <t xml:space="preserve">price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
+    <t xml:space="preserve">d in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
   </si>
 </sst>
 </file>
@@ -2167,16 +2170,16 @@
         <v>0.145990896974542</v>
       </c>
       <c r="K6" s="8" t="n">
-        <f aca="false">Gautam!E42</f>
-        <v>5514444</v>
+        <f aca="false">Gautam!E43</f>
+        <v>6014444</v>
       </c>
       <c r="L6" s="8" t="n">
         <f aca="false">G6-K6</f>
-        <v>55040.6865986399</v>
+        <v>-444959.31340136</v>
       </c>
       <c r="M6" s="9" t="n">
         <f aca="false">IF(K6&gt;0,L6/K6,"")</f>
-        <v>0.00998118515640742</v>
+        <v>-0.0739817867456011</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2464,15 +2467,15 @@
       </c>
       <c r="K12" s="17" t="n">
         <f aca="false">SUM(K6:K11)</f>
-        <v>40425847</v>
+        <v>40925847</v>
       </c>
       <c r="L12" s="17" t="n">
         <f aca="false">SUM(L6:L11)</f>
-        <v>-2276313.00837137</v>
+        <v>-2776313.00837137</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(K12&gt;0,L12/K12,"")</f>
-        <v>-0.0563083565910535</v>
+        <v>-0.0678376432470993</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3062,12 +3065,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
   </sheetData>
@@ -26024,7 +26027,7 @@
     <tabColor rgb="FF1E8449"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V44"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -27807,39 +27810,47 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="77" t="s">
+      <c r="B42" s="75" t="s">
         <v>211</v>
       </c>
-      <c r="C42" s="78"/>
-      <c r="D42" s="78"/>
-      <c r="E42" s="79" t="n">
-        <f aca="false">SUM(E40:E41)</f>
-        <v>5514444</v>
-      </c>
-      <c r="F42" s="78"/>
+      <c r="E42" s="76" t="n">
+        <v>500000</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="75" t="s">
+      <c r="B43" s="77" t="s">
         <v>212</v>
       </c>
-      <c r="E43" s="80" t="n">
+      <c r="C43" s="78"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="79" t="n">
+        <f aca="false">SUM(E40:E42)</f>
+        <v>6014444</v>
+      </c>
+      <c r="F43" s="78"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B44" s="75" t="s">
+        <v>213</v>
+      </c>
+      <c r="E44" s="80" t="n">
         <f aca="false">H37</f>
         <v>5569484.68659864</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="77" t="s">
-        <v>213</v>
-      </c>
-      <c r="C44" s="78"/>
-      <c r="D44" s="78"/>
-      <c r="E44" s="79" t="n">
-        <f aca="false">E43-E42</f>
-        <v>55040.6865986399</v>
-      </c>
-      <c r="F44" s="81" t="n">
-        <f aca="false">IF(E42&gt;0,E44/E42,"")</f>
-        <v>0.00998118515640742</v>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="77" t="s">
+        <v>214</v>
+      </c>
+      <c r="C45" s="78"/>
+      <c r="D45" s="78"/>
+      <c r="E45" s="79" t="n">
+        <f aca="false">E44-E43</f>
+        <v>-444959.31340136</v>
+      </c>
+      <c r="F45" s="81" t="n">
+        <f aca="false">IF(E43&gt;0,E45/E43,"")</f>
+        <v>-0.0739817867456011</v>
       </c>
     </row>
   </sheetData>
@@ -27889,12 +27900,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27904,7 +27915,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -27971,7 +27982,7 @@
         <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D7" s="60" t="n">
         <v>919</v>
@@ -28005,7 +28016,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -28031,7 +28042,7 @@
         <v>83</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D8" s="60" t="n">
         <v>798</v>
@@ -28065,13 +28076,13 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>205</v>
       </c>
       <c r="S8" s="62" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="T8" s="62" t="n">
         <v>33</v>
@@ -28091,7 +28102,7 @@
         <v>82</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D9" s="60" t="n">
         <v>379</v>
@@ -28125,7 +28136,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -28151,7 +28162,7 @@
         <v>80</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D10" s="60" t="n">
         <v>59</v>
@@ -28185,7 +28196,7 @@
       </c>
       <c r="L10" s="61"/>
       <c r="Q10" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -28211,7 +28222,7 @@
         <v>89</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D11" s="60" t="n">
         <v>800</v>
@@ -28245,7 +28256,7 @@
       </c>
       <c r="L11" s="61"/>
       <c r="Q11" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -28305,7 +28316,7 @@
       </c>
       <c r="L12" s="61"/>
       <c r="Q12" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>201</v>
@@ -28331,7 +28342,7 @@
         <v>84</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D13" s="60" t="n">
         <v>120</v>
@@ -28364,10 +28375,10 @@
         <v>0.0397576803773804</v>
       </c>
       <c r="L13" s="61" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Q13" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -28393,7 +28404,7 @@
         <v>86</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D14" s="60" t="n">
         <v>1881</v>
@@ -28427,7 +28438,7 @@
       </c>
       <c r="L14" s="61"/>
       <c r="Q14" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -28453,7 +28464,7 @@
         <v>88</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D15" s="60" t="n">
         <v>27</v>
@@ -28487,13 +28498,13 @@
       </c>
       <c r="L15" s="61"/>
       <c r="Q15" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>205</v>
       </c>
       <c r="S15" s="62" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="T15" s="62" t="n">
         <v>380</v>
@@ -28513,7 +28524,7 @@
         <v>93</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D16" s="60" t="n">
         <v>18</v>
@@ -28547,7 +28558,7 @@
       </c>
       <c r="L16" s="61"/>
       <c r="Q16" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -28607,7 +28618,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -28667,7 +28678,7 @@
       </c>
       <c r="L18" s="61"/>
       <c r="Q18" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -28693,7 +28704,7 @@
         <v>91</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D19" s="60" t="n">
         <v>23</v>
@@ -28727,7 +28738,7 @@
       </c>
       <c r="L19" s="61"/>
       <c r="Q19" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -28753,7 +28764,7 @@
         <v>109</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D20" s="60" t="n">
         <v>50</v>
@@ -28787,7 +28798,7 @@
       </c>
       <c r="L20" s="61"/>
       <c r="Q20" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R20" s="62" t="s">
         <v>201</v>
@@ -28813,7 +28824,7 @@
         <v>95</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D21" s="60" t="n">
         <v>9</v>
@@ -28847,7 +28858,7 @@
       </c>
       <c r="L21" s="61"/>
       <c r="Q21" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R21" s="62" t="s">
         <v>201</v>
@@ -28873,7 +28884,7 @@
         <v>94</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D22" s="60" t="n">
         <v>46</v>
@@ -28907,7 +28918,7 @@
       </c>
       <c r="L22" s="61"/>
       <c r="Q22" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R22" s="62" t="s">
         <v>201</v>
@@ -28933,7 +28944,7 @@
         <v>85</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D23" s="60" t="n">
         <v>26</v>
@@ -28967,7 +28978,7 @@
       </c>
       <c r="L23" s="61"/>
       <c r="Q23" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R23" s="62" t="s">
         <v>201</v>
@@ -28993,7 +29004,7 @@
         <v>105</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D24" s="60" t="n">
         <v>53</v>
@@ -29027,7 +29038,7 @@
       </c>
       <c r="L24" s="61"/>
       <c r="Q24" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R24" s="62" t="s">
         <v>201</v>
@@ -29087,13 +29098,13 @@
       </c>
       <c r="L25" s="61"/>
       <c r="Q25" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R25" s="62" t="s">
         <v>205</v>
       </c>
       <c r="S25" s="62" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="T25" s="62" t="n">
         <v>187</v>
@@ -29113,7 +29124,7 @@
         <v>98</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D26" s="60" t="n">
         <v>20</v>
@@ -29147,7 +29158,7 @@
       </c>
       <c r="L26" s="61"/>
       <c r="Q26" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R26" s="62" t="s">
         <v>201</v>
@@ -29173,7 +29184,7 @@
         <v>87</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D27" s="60" t="n">
         <v>12</v>
@@ -29207,7 +29218,7 @@
       </c>
       <c r="L27" s="61"/>
       <c r="Q27" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R27" s="62" t="s">
         <v>201</v>
@@ -29267,7 +29278,7 @@
       </c>
       <c r="L28" s="61"/>
       <c r="Q28" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R28" s="62" t="s">
         <v>201</v>
@@ -29293,7 +29304,7 @@
         <v>101</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D29" s="60" t="n">
         <v>14</v>
@@ -29327,7 +29338,7 @@
       </c>
       <c r="L29" s="61"/>
       <c r="Q29" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R29" s="62" t="s">
         <v>201</v>
@@ -29353,7 +29364,7 @@
         <v>118</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D30" s="60" t="n">
         <v>80</v>
@@ -29387,7 +29398,7 @@
       </c>
       <c r="L30" s="61"/>
       <c r="Q30" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R30" s="62" t="s">
         <v>201</v>
@@ -29413,7 +29424,7 @@
         <v>119</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D31" s="60" t="n">
         <v>111</v>
@@ -29447,7 +29458,7 @@
       </c>
       <c r="L31" s="61"/>
       <c r="Q31" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R31" s="62" t="s">
         <v>201</v>
@@ -29507,7 +29518,7 @@
       </c>
       <c r="L32" s="61"/>
       <c r="Q32" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R32" s="62" t="s">
         <v>201</v>
@@ -29567,7 +29578,7 @@
       </c>
       <c r="L33" s="61"/>
       <c r="Q33" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R33" s="62" t="s">
         <v>201</v>
@@ -29627,7 +29638,7 @@
       </c>
       <c r="L34" s="61"/>
       <c r="Q34" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R34" s="62" t="s">
         <v>201</v>
@@ -29687,7 +29698,7 @@
       </c>
       <c r="L35" s="61"/>
       <c r="Q35" s="62" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="R35" s="62" t="s">
         <v>201</v>
@@ -29713,7 +29724,7 @@
         <v>124</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D36" s="60" t="n">
         <v>1072</v>
@@ -29762,7 +29773,7 @@
         <v>126</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D37" s="60" t="n">
         <v>166</v>
@@ -29804,7 +29815,7 @@
         <v>127</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D38" s="60" t="n">
         <v>110</v>
@@ -29837,7 +29848,7 @@
         <v>0.00588779149794186</v>
       </c>
       <c r="L38" s="61" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -29848,7 +29859,7 @@
         <v>128</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D39" s="60" t="n">
         <v>116</v>
@@ -29890,7 +29901,7 @@
         <v>129</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D40" s="60" t="n">
         <v>302</v>
@@ -29932,7 +29943,7 @@
         <v>130</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D41" s="60" t="n">
         <v>245</v>
@@ -29974,7 +29985,7 @@
         <v>132</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D42" s="60" t="n">
         <v>51</v>
@@ -30058,7 +30069,7 @@
         <v>134</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D44" s="60" t="n">
         <v>124</v>
@@ -30142,7 +30153,7 @@
         <v>135</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D46" s="60" t="n">
         <v>49</v>
@@ -30184,7 +30195,7 @@
         <v>136</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D47" s="60" t="n">
         <v>76</v>
@@ -30226,7 +30237,7 @@
         <v>139</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D48" s="60" t="n">
         <v>54</v>
@@ -30268,7 +30279,7 @@
         <v>137</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D49" s="60" t="n">
         <v>150</v>
@@ -30310,7 +30321,7 @@
         <v>142</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D50" s="60" t="n">
         <v>48</v>
@@ -30352,7 +30363,7 @@
         <v>144</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D51" s="60" t="n">
         <v>35</v>
@@ -30394,7 +30405,7 @@
         <v>145</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D52" s="60" t="n">
         <v>132</v>
@@ -30436,7 +30447,7 @@
         <v>148</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D53" s="60" t="n">
         <v>9</v>
@@ -30520,7 +30531,7 @@
         <v>156</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D55" s="60" t="n">
         <v>36</v>
@@ -30562,7 +30573,7 @@
         <v>160</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D56" s="60" t="n">
         <v>20</v>
@@ -30637,7 +30648,7 @@
         <v>0.000310945203954612</v>
       </c>
       <c r="L57" s="61" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30648,7 +30659,7 @@
         <v>164</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D58" s="60" t="n">
         <v>6</v>
@@ -30690,7 +30701,7 @@
         <v>165</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D59" s="60" t="n">
         <v>1</v>
@@ -30762,7 +30773,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B63" s="75" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E63" s="76" t="n">
         <v>4111335</v>
@@ -30770,7 +30781,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B64" s="85" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C64" s="86"/>
       <c r="D64" s="86"/>
@@ -30782,7 +30793,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="75" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E65" s="80" t="n">
         <f aca="false">H60</f>
@@ -30791,7 +30802,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="85" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C66" s="86"/>
       <c r="D66" s="86"/>
@@ -30845,12 +30856,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30904,7 +30915,7 @@
         <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D7" s="60" t="n">
         <v>3895</v>
@@ -30937,7 +30948,7 @@
         <v>0.305628125337199</v>
       </c>
       <c r="L7" s="61" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30948,7 +30959,7 @@
         <v>81</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D8" s="60" t="n">
         <v>11160</v>
@@ -30981,7 +30992,7 @@
         <v>0.247667747990467</v>
       </c>
       <c r="L8" s="61" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30992,7 +31003,7 @@
         <v>80</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D9" s="60" t="n">
         <v>165</v>
@@ -31025,7 +31036,7 @@
         <v>0.0613913539222327</v>
       </c>
       <c r="L9" s="61" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31036,7 +31047,7 @@
         <v>82</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D10" s="60" t="n">
         <v>1013</v>
@@ -31069,7 +31080,7 @@
         <v>0.0591290750864015</v>
       </c>
       <c r="L10" s="61" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31080,7 +31091,7 @@
         <v>83</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D11" s="60" t="n">
         <v>1394</v>
@@ -31113,7 +31124,7 @@
         <v>0.048249628624683</v>
       </c>
       <c r="L11" s="61" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31124,7 +31135,7 @@
         <v>84</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D12" s="60" t="n">
         <v>360</v>
@@ -31166,7 +31177,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D13" s="60" t="n">
         <v>2004.589</v>
@@ -31199,7 +31210,7 @@
         <v>0.0272662721420509</v>
       </c>
       <c r="L13" s="61" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31210,7 +31221,7 @@
         <v>86</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D14" s="60" t="n">
         <v>3762</v>
@@ -31243,7 +31254,7 @@
         <v>0.0251381588851207</v>
       </c>
       <c r="L14" s="61" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31254,7 +31265,7 @@
         <v>88</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D15" s="60" t="n">
         <v>72</v>
@@ -31287,7 +31298,7 @@
         <v>0.0251350309341946</v>
       </c>
       <c r="L15" s="61" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31298,7 +31309,7 @@
         <v>87</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D16" s="60" t="n">
         <v>66</v>
@@ -31331,7 +31342,7 @@
         <v>0.0229480070702708</v>
       </c>
       <c r="L16" s="61" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31342,7 +31353,7 @@
         <v>89</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D17" s="60" t="n">
         <v>800</v>
@@ -31384,7 +31395,7 @@
         <v>92</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D18" s="60" t="n">
         <v>3500</v>
@@ -31426,7 +31437,7 @@
         <v>102</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D19" s="60" t="n">
         <v>134</v>
@@ -31468,7 +31479,7 @@
         <v>91</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D20" s="60" t="n">
         <v>32</v>
@@ -31501,7 +31512,7 @@
         <v>0.0102404513900704</v>
       </c>
       <c r="L20" s="61" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31512,7 +31523,7 @@
         <v>108</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D21" s="60" t="n">
         <v>44</v>
@@ -31554,7 +31565,7 @@
         <v>110</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D22" s="60" t="n">
         <v>3</v>
@@ -31596,7 +31607,7 @@
         <v>111</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D23" s="60" t="n">
         <v>64</v>
@@ -31638,7 +31649,7 @@
         <v>112</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D24" s="60" t="n">
         <v>160</v>
@@ -31671,7 +31682,7 @@
         <v>0.00608714120518771</v>
       </c>
       <c r="L24" s="61" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31682,7 +31693,7 @@
         <v>85</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D25" s="60" t="n">
         <v>29</v>
@@ -31724,7 +31735,7 @@
         <v>113</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D26" s="60" t="n">
         <v>2</v>
@@ -31766,7 +31777,7 @@
         <v>94</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D27" s="60" t="n">
         <v>47</v>
@@ -31799,7 +31810,7 @@
         <v>0.00557619932630266</v>
       </c>
       <c r="L27" s="61" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31810,7 +31821,7 @@
         <v>93</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D28" s="60" t="n">
         <v>11</v>
@@ -31843,7 +31854,7 @@
         <v>0.00547590259138421</v>
       </c>
       <c r="L28" s="61" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31854,7 +31865,7 @@
         <v>116</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D29" s="60" t="n">
         <v>22</v>
@@ -31896,7 +31907,7 @@
         <v>95</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D30" s="60" t="n">
         <v>6</v>
@@ -31929,7 +31940,7 @@
         <v>0.00370918956831849</v>
       </c>
       <c r="L30" s="61" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31940,7 +31951,7 @@
         <v>99</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D31" s="60" t="n">
         <v>32</v>
@@ -31982,7 +31993,7 @@
         <v>125</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D32" s="60" t="n">
         <v>34</v>
@@ -32024,7 +32035,7 @@
         <v>98</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D33" s="60" t="n">
         <v>10</v>
@@ -32057,7 +32068,7 @@
         <v>0.00245723110063977</v>
       </c>
       <c r="L33" s="61" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32068,7 +32079,7 @@
         <v>115</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D34" s="60" t="n">
         <v>168</v>
@@ -32101,7 +32112,7 @@
         <v>0.00173943021648071</v>
       </c>
       <c r="L34" s="61" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32112,7 +32123,7 @@
         <v>131</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D35" s="60" t="n">
         <v>33</v>
@@ -32154,7 +32165,7 @@
         <v>101</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D36" s="60" t="n">
         <v>6</v>
@@ -32187,7 +32198,7 @@
         <v>0.00162669010101251</v>
       </c>
       <c r="L36" s="61" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32198,7 +32209,7 @@
         <v>100</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D37" s="60" t="n">
         <v>17</v>
@@ -32231,7 +32242,7 @@
         <v>0.00158276218875317</v>
       </c>
       <c r="L37" s="61" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32242,7 +32253,7 @@
         <v>143</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D38" s="60" t="n">
         <v>50</v>
@@ -32284,7 +32295,7 @@
         <v>104</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D39" s="60" t="n">
         <v>6</v>
@@ -32317,7 +32328,7 @@
         <v>0.00113239085765181</v>
       </c>
       <c r="L39" s="61" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32328,7 +32339,7 @@
         <v>146</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D40" s="60" t="n">
         <v>35</v>
@@ -32370,7 +32381,7 @@
         <v>147</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D41" s="60" t="n">
         <v>34</v>
@@ -32403,7 +32414,7 @@
         <v>0.000957094193811925</v>
       </c>
       <c r="L41" s="61" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32414,7 +32425,7 @@
         <v>149</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D42" s="60" t="n">
         <v>14</v>
@@ -32456,7 +32467,7 @@
         <v>107</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D43" s="60" t="n">
         <v>32</v>
@@ -32498,7 +32509,7 @@
         <v>153</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D44" s="60" t="n">
         <v>4</v>
@@ -32531,7 +32542,7 @@
         <v>0.000480604731843519</v>
       </c>
       <c r="L44" s="61" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32542,7 +32553,7 @@
         <v>154</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D45" s="60" t="n">
         <v>3</v>
@@ -32584,7 +32595,7 @@
         <v>103</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D46" s="60" t="n">
         <v>5</v>
@@ -32626,7 +32637,7 @@
         <v>157</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D47" s="60" t="n">
         <v>5</v>
@@ -32668,7 +32679,7 @@
         <v>158</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D48" s="60" t="n">
         <v>1</v>
@@ -32710,7 +32721,7 @@
         <v>151</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D49" s="60" t="n">
         <v>5</v>
@@ -32743,7 +32754,7 @@
         <v>0.000287182724950748</v>
       </c>
       <c r="L49" s="61" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32754,7 +32765,7 @@
         <v>159</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D50" s="60" t="n">
         <v>6</v>
@@ -32796,7 +32807,7 @@
         <v>161</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D51" s="60" t="n">
         <v>1</v>
@@ -32838,7 +32849,7 @@
         <v>137</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D52" s="60" t="n">
         <v>12</v>
@@ -32880,7 +32891,7 @@
         <v>163</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D53" s="60" t="n">
         <v>5</v>
@@ -32952,7 +32963,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E57" s="76" t="n">
         <v>12135171</v>
@@ -32968,7 +32979,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B59" s="92" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C59" s="93"/>
       <c r="D59" s="93"/>
@@ -32980,7 +32991,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B60" s="75" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E60" s="80" t="n">
         <f aca="false">H54</f>
@@ -32989,7 +33000,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B61" s="92" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C61" s="93"/>
       <c r="D61" s="93"/>
@@ -33049,12 +33060,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33064,7 +33075,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33164,10 +33175,10 @@
         <v>0.387667709233293</v>
       </c>
       <c r="L7" s="61" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Q7" s="62" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>205</v>
@@ -33226,10 +33237,10 @@
         <v>0.0930272321101565</v>
       </c>
       <c r="L8" s="61" t="s">
+        <v>264</v>
+      </c>
+      <c r="Q8" s="62" t="s">
         <v>263</v>
-      </c>
-      <c r="Q8" s="62" t="s">
-        <v>262</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -33289,7 +33300,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -33348,10 +33359,10 @@
         <v>0.0665492729486535</v>
       </c>
       <c r="L10" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q10" s="62" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -33410,10 +33421,10 @@
         <v>0.0663936626599383</v>
       </c>
       <c r="L11" s="61" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Q11" s="62" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -33473,13 +33484,13 @@
       </c>
       <c r="L12" s="61"/>
       <c r="Q12" s="62" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>205</v>
       </c>
       <c r="S12" s="62" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="T12" s="62" t="n">
         <v>700</v>
@@ -33533,7 +33544,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -33593,7 +33604,7 @@
       </c>
       <c r="L14" s="61"/>
       <c r="Q14" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -33652,10 +33663,10 @@
         <v>0.0282483930215812</v>
       </c>
       <c r="L15" s="61" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q15" s="62" t="s">
         <v>268</v>
-      </c>
-      <c r="Q15" s="62" t="s">
-        <v>267</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -33714,10 +33725,10 @@
         <v>0.0272325527669234</v>
       </c>
       <c r="L16" s="61" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q16" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -33777,7 +33788,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -33836,10 +33847,10 @@
         <v>0.0222301631600693</v>
       </c>
       <c r="L18" s="61" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q18" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -33898,10 +33909,10 @@
         <v>0.0208031596594696</v>
       </c>
       <c r="L19" s="61" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q19" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -33961,7 +33972,7 @@
       </c>
       <c r="L20" s="61"/>
       <c r="Q20" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R20" s="62" t="s">
         <v>201</v>
@@ -34020,10 +34031,10 @@
         <v>0.00925511581813541</v>
       </c>
       <c r="L21" s="61" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q21" s="62" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="R21" s="62" t="s">
         <v>201</v>
@@ -34082,7 +34093,7 @@
         <v>0.0064722190095489</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q22" s="62" t="s">
         <v>21</v>
@@ -34144,7 +34155,7 @@
         <v>0.00633173137432947</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q23" s="62" t="s">
         <v>21</v>
@@ -34206,7 +34217,7 @@
         <v>0.00565045107879498</v>
       </c>
       <c r="L24" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q24" s="62" t="s">
         <v>21</v>
@@ -34268,7 +34279,7 @@
         <v>0.00494611932858946</v>
       </c>
       <c r="L25" s="61" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q25" s="62" t="s">
         <v>21</v>
@@ -34330,7 +34341,7 @@
         <v>0.00271144248698057</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q26" s="62" t="s">
         <v>21</v>
@@ -34392,7 +34403,7 @@
         <v>0.00207627374724527</v>
       </c>
       <c r="L27" s="61" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q27" s="62" t="s">
         <v>21</v>
@@ -34454,7 +34465,7 @@
         <v>0.00196599683318886</v>
       </c>
       <c r="L28" s="61" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="Q28" s="62" t="s">
         <v>21</v>
@@ -34516,7 +34527,7 @@
         <v>0.000701063389415708</v>
       </c>
       <c r="L29" s="61" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q29" s="62" t="s">
         <v>21</v>
@@ -34578,7 +34589,7 @@
         <v>0.00028721368924799</v>
       </c>
       <c r="L30" s="61" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q30" s="62" t="s">
         <v>21</v>
@@ -34753,7 +34764,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="75" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E35" s="76" t="n">
         <v>10914339</v>
@@ -34831,7 +34842,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="99" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C38" s="100"/>
       <c r="D38" s="100"/>
@@ -34861,7 +34872,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="75" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E39" s="80" t="n">
         <f aca="false">H32</f>
@@ -34888,7 +34899,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="99" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C40" s="100"/>
       <c r="D40" s="100"/>
@@ -35075,12 +35086,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35090,7 +35101,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35191,7 +35202,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -35251,7 +35262,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -35311,7 +35322,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -35752,7 +35763,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="75" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E22" s="76" t="n">
         <v>167022</v>
@@ -35768,7 +35779,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="106" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C24" s="107"/>
       <c r="D24" s="107"/>
@@ -35780,7 +35791,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="75" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E25" s="80" t="n">
         <f aca="false">H19</f>
@@ -35789,7 +35800,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="106" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C26" s="107"/>
       <c r="D26" s="107"/>
@@ -35849,12 +35860,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35864,7 +35875,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35965,7 +35976,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -36025,7 +36036,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -36085,7 +36096,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -36144,10 +36155,10 @@
         <v>0.060071305630396</v>
       </c>
       <c r="L10" s="61" t="s">
+        <v>288</v>
+      </c>
+      <c r="Q10" s="62" t="s">
         <v>287</v>
-      </c>
-      <c r="Q10" s="62" t="s">
-        <v>286</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -36207,7 +36218,7 @@
       </c>
       <c r="L11" s="61"/>
       <c r="Q11" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -36266,10 +36277,10 @@
         <v>0.0360333489709902</v>
       </c>
       <c r="L12" s="61" t="s">
+        <v>288</v>
+      </c>
+      <c r="Q12" s="62" t="s">
         <v>287</v>
-      </c>
-      <c r="Q12" s="62" t="s">
-        <v>286</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>201</v>
@@ -36329,7 +36340,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -36391,7 +36402,7 @@
         <v>202</v>
       </c>
       <c r="Q14" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -36451,7 +36462,7 @@
       </c>
       <c r="L15" s="61"/>
       <c r="Q15" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -36511,7 +36522,7 @@
       </c>
       <c r="L16" s="61"/>
       <c r="Q16" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -36571,7 +36582,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -36631,7 +36642,7 @@
       </c>
       <c r="L18" s="61"/>
       <c r="Q18" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -36691,7 +36702,7 @@
       </c>
       <c r="L19" s="61"/>
       <c r="Q19" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -36841,7 +36852,7 @@
         <v>0.00684755364735877</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36885,7 +36896,7 @@
         <v>0.00408028602961991</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37013,7 +37024,7 @@
         <v>0.00121270175094724</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37096,7 +37107,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="75" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E31" s="76" t="n">
         <v>4529555</v>
@@ -37112,7 +37123,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="113" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C33" s="114"/>
       <c r="D33" s="114"/>
@@ -37124,7 +37135,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="75" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E34" s="80" t="n">
         <f aca="false">H28</f>
@@ -37133,7 +37144,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="113" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C35" s="114"/>
       <c r="D35" s="114"/>

</xml_diff>

<commit_message>
Manish base 11,949,395 + 850,000 cash; drop combined invested/gain totals in Summary
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -951,7 +951,7 @@
     <t xml:space="preserve">New position 09.10.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 12135171, "cash": [["Cash added", 340000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges include</t>
+    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 11949395, "cash": [["Cash added", 850000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges include</t>
   </si>
   <si>
     <t xml:space="preserve">d in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
@@ -2271,15 +2271,15 @@
       </c>
       <c r="K8" s="8" t="n">
         <f aca="false">'Manish Shilpa'!E59</f>
-        <v>12475171</v>
+        <v>12799395</v>
       </c>
       <c r="L8" s="8" t="n">
         <f aca="false">G8-K8</f>
-        <v>-908493.371428572</v>
+        <v>-1232717.37142857</v>
       </c>
       <c r="M8" s="9" t="n">
         <f aca="false">IF(K8&gt;0,L8/K8,"")</f>
-        <v>-0.0728241217237481</v>
+        <v>-0.0963105968234101</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2445,37 +2445,28 @@
         <f aca="false">'Side by Side'!E6</f>
         <v>88</v>
       </c>
-      <c r="F12" s="17" t="n">
-        <f aca="false">SUM(F6:F11)</f>
-        <v>37595951.23</v>
-      </c>
+      <c r="F12" s="17"/>
       <c r="G12" s="17" t="n">
         <f aca="false">SUM(G6:G11)</f>
         <v>38149533.9916286</v>
       </c>
-      <c r="H12" s="17" t="n">
-        <f aca="false">SUM(H6:H11)</f>
-        <v>553582.761628631</v>
-      </c>
-      <c r="I12" s="18" t="n">
-        <f aca="false">IF(F12&gt;0,H12/F12,"")</f>
-        <v>0.0147245313263119</v>
-      </c>
+      <c r="H12" s="17"/>
+      <c r="I12" s="18"/>
       <c r="J12" s="18" t="n">
         <f aca="false">SUM(J6:J11)</f>
         <v>1</v>
       </c>
       <c r="K12" s="17" t="n">
         <f aca="false">SUM(K6:K11)</f>
-        <v>40925847</v>
+        <v>41250071</v>
       </c>
       <c r="L12" s="17" t="n">
         <f aca="false">SUM(L6:L11)</f>
-        <v>-2776313.00837137</v>
+        <v>-3100537.00837137</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(K12&gt;0,L12/K12,"")</f>
-        <v>-0.0678376432470993</v>
+        <v>-0.0751644041623921</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32966,7 +32957,7 @@
         <v>258</v>
       </c>
       <c r="E57" s="76" t="n">
-        <v>12135171</v>
+        <v>11949395</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32974,7 +32965,7 @@
         <v>210</v>
       </c>
       <c r="E58" s="76" t="n">
-        <v>340000</v>
+        <v>850000</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32985,7 +32976,7 @@
       <c r="D59" s="93"/>
       <c r="E59" s="94" t="n">
         <f aca="false">SUM(E57:E58)</f>
-        <v>12475171</v>
+        <v>12799395</v>
       </c>
       <c r="F59" s="93"/>
     </row>
@@ -33006,11 +32997,11 @@
       <c r="D61" s="93"/>
       <c r="E61" s="94" t="n">
         <f aca="false">E60-E59</f>
-        <v>-908493.371428572</v>
+        <v>-1232717.37142857</v>
       </c>
       <c r="F61" s="95" t="n">
         <f aca="false">IF(E59&gt;0,E61/E59,"")</f>
-        <v>-0.0728241217237481</v>
+        <v>-0.0963105968234101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Account tabs: no total for Invested or P&L in TOTAL row
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -2150,7 +2150,7 @@
         <v>30</v>
       </c>
       <c r="F6" s="7" t="n">
-        <f aca="false">Gautam!E37</f>
+        <f aca="false">SUM(Gautam!E7:E36)</f>
         <v>6000656.23</v>
       </c>
       <c r="G6" s="7" t="n">
@@ -2200,7 +2200,7 @@
         <v>53</v>
       </c>
       <c r="F7" s="7" t="n">
-        <f aca="false">DA!E60</f>
+        <f aca="false">SUM(DA!E7:E59)</f>
         <v>4574421</v>
       </c>
       <c r="G7" s="7" t="n">
@@ -2250,7 +2250,7 @@
         <v>47</v>
       </c>
       <c r="F8" s="7" t="n">
-        <f aca="false">'Manish Shilpa'!E54</f>
+        <f aca="false">SUM('Manish Shilpa'!E7:E53)</f>
         <v>9857778</v>
       </c>
       <c r="G8" s="7" t="n">
@@ -2300,7 +2300,7 @@
         <v>25</v>
       </c>
       <c r="F9" s="7" t="n">
-        <f aca="false">'Saloni Mehra'!E32</f>
+        <f aca="false">SUM('Saloni Mehra'!E7:E31)</f>
         <v>11739506</v>
       </c>
       <c r="G9" s="7" t="n">
@@ -2350,7 +2350,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="7" t="n">
-        <f aca="false">'Vidushi Malhotra'!E19</f>
+        <f aca="false">SUM('Vidushi Malhotra'!E7:E18)</f>
         <v>201361</v>
       </c>
       <c r="G10" s="7" t="n">
@@ -2400,7 +2400,7 @@
         <v>20</v>
       </c>
       <c r="F11" s="7" t="n">
-        <f aca="false">'Dr Umesh Choudhry'!E28</f>
+        <f aca="false">SUM('Dr Umesh Choudhry'!E7:E27)</f>
         <v>5222229</v>
       </c>
       <c r="G11" s="7" t="n">
@@ -27755,24 +27755,15 @@
       </c>
       <c r="C37" s="72"/>
       <c r="D37" s="72"/>
-      <c r="E37" s="73" t="n">
-        <f aca="false">SUM(E7:E36)</f>
-        <v>6000656.23</v>
-      </c>
+      <c r="E37" s="73"/>
       <c r="F37" s="72"/>
       <c r="G37" s="72"/>
       <c r="H37" s="73" t="n">
         <f aca="false">SUM(H7:H36)</f>
         <v>5569484.68659864</v>
       </c>
-      <c r="I37" s="73" t="n">
-        <f aca="false">H37-E37</f>
-        <v>-431171.543401361</v>
-      </c>
-      <c r="J37" s="74" t="n">
-        <f aca="false">IF(E37&gt;0,I37/E37,"")</f>
-        <v>-0.0718540651013698</v>
-      </c>
+      <c r="I37" s="73"/>
+      <c r="J37" s="74"/>
       <c r="K37" s="74" t="n">
         <f aca="false">SUM(K7:K36)</f>
         <v>1</v>
@@ -30733,24 +30724,15 @@
       </c>
       <c r="C60" s="82"/>
       <c r="D60" s="82"/>
-      <c r="E60" s="83" t="n">
-        <f aca="false">SUM(E7:E59)</f>
-        <v>4574421</v>
-      </c>
+      <c r="E60" s="83"/>
       <c r="F60" s="82"/>
       <c r="G60" s="82"/>
       <c r="H60" s="83" t="n">
         <f aca="false">SUM(H7:H59)</f>
         <v>3971760.89</v>
       </c>
-      <c r="I60" s="83" t="n">
-        <f aca="false">H60-E60</f>
-        <v>-602660.11</v>
-      </c>
-      <c r="J60" s="84" t="n">
-        <f aca="false">IF(E60&gt;0,I60/E60,"")</f>
-        <v>-0.131745659177413</v>
-      </c>
+      <c r="I60" s="83"/>
+      <c r="J60" s="84"/>
       <c r="K60" s="84" t="n">
         <f aca="false">SUM(K7:K59)</f>
         <v>1</v>
@@ -32923,24 +32905,15 @@
       </c>
       <c r="C54" s="89"/>
       <c r="D54" s="89"/>
-      <c r="E54" s="90" t="n">
-        <f aca="false">SUM(E7:E53)</f>
-        <v>9857778</v>
-      </c>
+      <c r="E54" s="90"/>
       <c r="F54" s="89"/>
       <c r="G54" s="89"/>
       <c r="H54" s="90" t="n">
         <f aca="false">SUM(H7:H53)</f>
         <v>11566677.6285714</v>
       </c>
-      <c r="I54" s="90" t="n">
-        <f aca="false">H54-E54</f>
-        <v>1708899.62857143</v>
-      </c>
-      <c r="J54" s="91" t="n">
-        <f aca="false">IF(E54&gt;0,I54/E54,"")</f>
-        <v>0.173355458864201</v>
-      </c>
+      <c r="I54" s="90"/>
+      <c r="J54" s="91"/>
       <c r="K54" s="91" t="n">
         <f aca="false">SUM(K7:K53)</f>
         <v>1</v>
@@ -34668,24 +34641,15 @@
       </c>
       <c r="C32" s="96"/>
       <c r="D32" s="96"/>
-      <c r="E32" s="97" t="n">
-        <f aca="false">SUM(E7:E31)</f>
-        <v>11739506</v>
-      </c>
+      <c r="E32" s="97"/>
       <c r="F32" s="96"/>
       <c r="G32" s="96"/>
       <c r="H32" s="97" t="n">
         <f aca="false">SUM(H7:H31)</f>
         <v>11565430.6335374</v>
       </c>
-      <c r="I32" s="97" t="n">
-        <f aca="false">H32-E32</f>
-        <v>-174075.366462585</v>
-      </c>
-      <c r="J32" s="98" t="n">
-        <f aca="false">IF(E32&gt;0,I32/E32,"")</f>
-        <v>-0.0148281679367585</v>
-      </c>
+      <c r="I32" s="97"/>
+      <c r="J32" s="98"/>
       <c r="K32" s="98" t="n">
         <f aca="false">SUM(K7:K31)</f>
         <v>1</v>
@@ -35723,24 +35687,15 @@
       </c>
       <c r="C19" s="103"/>
       <c r="D19" s="103"/>
-      <c r="E19" s="104" t="n">
-        <f aca="false">SUM(E7:E18)</f>
-        <v>201361</v>
-      </c>
+      <c r="E19" s="104"/>
       <c r="F19" s="103"/>
       <c r="G19" s="103"/>
       <c r="H19" s="104" t="n">
         <f aca="false">SUM(H7:H18)</f>
         <v>218828.132921147</v>
       </c>
-      <c r="I19" s="104" t="n">
-        <f aca="false">H19-E19</f>
-        <v>17467.132921147</v>
-      </c>
-      <c r="J19" s="105" t="n">
-        <f aca="false">IF(E19&gt;0,I19/E19,"")</f>
-        <v>0.0867453624145041</v>
-      </c>
+      <c r="I19" s="104"/>
+      <c r="J19" s="105"/>
       <c r="K19" s="105" t="n">
         <f aca="false">SUM(K7:K18)</f>
         <v>1</v>
@@ -37067,24 +37022,15 @@
       </c>
       <c r="C28" s="110"/>
       <c r="D28" s="110"/>
-      <c r="E28" s="111" t="n">
-        <f aca="false">SUM(E7:E27)</f>
-        <v>5222229</v>
-      </c>
+      <c r="E28" s="111"/>
       <c r="F28" s="110"/>
       <c r="G28" s="110"/>
       <c r="H28" s="111" t="n">
         <f aca="false">SUM(H7:H27)</f>
         <v>5257352.02</v>
       </c>
-      <c r="I28" s="111" t="n">
-        <f aca="false">H28-E28</f>
-        <v>35123.0200000005</v>
-      </c>
-      <c r="J28" s="112" t="n">
-        <f aca="false">IF(E28&gt;0,I28/E28,"")</f>
-        <v>0.00672567595178237</v>
-      </c>
+      <c r="I28" s="111"/>
+      <c r="J28" s="112"/>
       <c r="K28" s="112" t="n">
         <f aca="false">SUM(K7:K27)</f>
         <v>1</v>

</xml_diff>

<commit_message>
Manish: 29.10.2026 HDFC order book (5 buys)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1365" uniqueCount="295">
   <si>
     <t xml:space="preserve">CONSOLIDATED PORTFOLIO SUMMARY – ALL MANAGED ACCOUNTS</t>
   </si>
@@ -418,10 +418,10 @@
     <t xml:space="preserve">Page Industries Ltd</t>
   </si>
   <si>
-    <t xml:space="preserve">Vedant Fashions (Manyavar) Ltd</t>
+    <t xml:space="preserve">HDFC Gold ETF</t>
   </si>
   <si>
-    <t xml:space="preserve">HDFC Gold ETF</t>
+    <t xml:space="preserve">Vedant Fashions (Manyavar) Ltd</t>
   </si>
   <si>
     <t xml:space="preserve">Asian Paints Ltd</t>
@@ -768,10 +768,16 @@
     <t xml:space="preserve">Holdings as of 23.10.2026 (live, ~11:23 IST). Statement prices: Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged). Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
   </si>
   <si>
+    <t xml:space="preserve">HDFC Securities (Manish) order book of 29.10.2026 – 5 executed buys; order book carries no fill price, so cost uses its Close Price column (previous close) until the tradebook is supplied</t>
+  </si>
+  <si>
     <t xml:space="preserve">Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504</t>
+    <t xml:space="preserve">Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504; 29.10 buy 40 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29.10.2026 10:31–10:42</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101</t>
@@ -780,10 +786,10 @@
     <t xml:space="preserve">Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56</t>
+    <t xml:space="preserve">Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56; 29.10 buy 14 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8</t>
+    <t xml:space="preserve">Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8; 29.10 buy 21 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct (Manish)</t>
@@ -795,7 +801,7 @@
     <t xml:space="preserve">Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99</t>
+    <t xml:space="preserve">Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99; 29.10 buy 48 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6</t>
@@ -831,7 +837,7 @@
     <t xml:space="preserve">Axis Direct Shilpa 3; Axis Direct Manish 7</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 93; Axis Direct Manish 75</t>
+    <t xml:space="preserve">Axis Direct Shilpa 93; Axis Direct Manish 75; 29.10 buy 1 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct Shilpa 2; Axis Direct Manish 4</t>
@@ -951,10 +957,10 @@
     <t xml:space="preserve">New position 09.10.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3762.0, 432693, 292084, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 168.0, 15354, 20131, "Axis Direct Shilpa 93; Axis Direct Manish 75"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3895.0, 2912389, 3625900, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1013.0, 812683, 697943, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1394.0, 622513, 578058, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "", "trades": [], "base": {"label": "Year 3 base", "amount": 11949395, "cash": [["Cash added", 850000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges include</t>
+    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3810.0, 436419.72, null, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99; 29.10 buy 48 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 169.0, 15473.53, null, "Axis Direct Shilpa 93; Axis Direct Manish 75; 29.10 buy 1 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3935.0, 2948869.0, null, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504; 29.10 buy 40 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1027.0, 822205.8, null, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56; 29.10 buy 14 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1415.0, 630971.8, null, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8; 29.10 buy 21 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "HDFC Securities (Manish) order book of 29.10.2026 – 5 executed buys; order book carries no fill price, so cost uses its Close Price column (previous close) until the tradebook is supplied", "trades": [["29.10.2026 10:31–10:42", "BUY", "HDFC Gold ETF", 1.0, 119.53, 119.53], ["29.10.2026 10:31–10:42", "BUY", "HDFC Bank Ltd", 14.0, 680.2, 9522.8], ["29.10.2026 10:31–10:42", "BUY", "Poonawalla Fincorp Ltd", 21.0, 402.8, 8458.8], ["29.10.2026 10:31–10:42", "BUY", "Bajaj Housing Finance Ltd", 48.0, 77.64, 3726.72], ["29.1</t>
   </si>
   <si>
-    <t xml:space="preserve">d in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
+    <t xml:space="preserve">0.2026 10:31–10:42", "BUY", "Bajaj Finance Ltd", 40.0, 912.0, 36480.0]], "base": {"label": "Year 3 base", "amount": 11949395, "cash": [["Cash added", 850000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
   </si>
 </sst>
 </file>
@@ -2167,7 +2173,7 @@
       </c>
       <c r="J6" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G6/$G$12)</f>
-        <v>0.145990896974542</v>
+        <v>0.145769305327902</v>
       </c>
       <c r="K6" s="8" t="n">
         <f aca="false">Gautam!E43</f>
@@ -2217,7 +2223,7 @@
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G7/$G$12)</f>
-        <v>0.10411033830378</v>
+        <v>0.103952314880573</v>
       </c>
       <c r="K7" s="8" t="n">
         <f aca="false">DA!E64</f>
@@ -2251,23 +2257,23 @@
       </c>
       <c r="F8" s="7" t="n">
         <f aca="false">SUM('Manish Shilpa'!E7:E53)</f>
-        <v>9857778</v>
+        <v>9916085.85</v>
       </c>
       <c r="G8" s="7" t="n">
         <f aca="false">'Manish Shilpa'!H54</f>
-        <v>11566677.6285714</v>
+        <v>11624670.7570748</v>
       </c>
       <c r="H8" s="8" t="n">
         <f aca="false">G8-F8</f>
-        <v>1708899.62857143</v>
+        <v>1708584.90707483</v>
       </c>
       <c r="I8" s="9" t="n">
         <f aca="false">IF(F8&gt;0,H8/F8,"")</f>
-        <v>0.173355458864201</v>
+        <v>0.172304368167086</v>
       </c>
       <c r="J8" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G8/$G$12)</f>
-        <v>0.303193156464495</v>
+        <v>0.30425080169477</v>
       </c>
       <c r="K8" s="8" t="n">
         <f aca="false">'Manish Shilpa'!E59</f>
@@ -2275,11 +2281,11 @@
       </c>
       <c r="L8" s="8" t="n">
         <f aca="false">G8-K8</f>
-        <v>-1232717.37142857</v>
+        <v>-1174724.24292517</v>
       </c>
       <c r="M8" s="9" t="n">
         <f aca="false">IF(K8&gt;0,L8/K8,"")</f>
-        <v>-0.0963105968234101</v>
+        <v>-0.0917796695019701</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2317,7 +2323,7 @@
       </c>
       <c r="J9" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G9/$G$12)</f>
-        <v>0.303160469432609</v>
+        <v>0.302700318635472</v>
       </c>
       <c r="K9" s="8" t="n">
         <f aca="false">'Saloni Mehra'!E38</f>
@@ -2367,7 +2373,7 @@
       </c>
       <c r="J10" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G10/$G$12)</f>
-        <v>0.00573606306617443</v>
+        <v>0.00572735660785133</v>
       </c>
       <c r="K10" s="8" t="n">
         <f aca="false">'Vidushi Malhotra'!E24</f>
@@ -2417,7 +2423,7 @@
       </c>
       <c r="J11" s="9" t="n">
         <f aca="false">IF($G$12=0,"",G11/$G$12)</f>
-        <v>0.1378090757584</v>
+        <v>0.137599902853431</v>
       </c>
       <c r="K11" s="8" t="n">
         <f aca="false">'Dr Umesh Choudhry'!E33</f>
@@ -2448,7 +2454,7 @@
       <c r="F12" s="17"/>
       <c r="G12" s="17" t="n">
         <f aca="false">SUM(G6:G11)</f>
-        <v>38149533.9916286</v>
+        <v>38207527.120132</v>
       </c>
       <c r="H12" s="17"/>
       <c r="I12" s="18"/>
@@ -2462,11 +2468,11 @@
       </c>
       <c r="L12" s="17" t="n">
         <f aca="false">SUM(L6:L11)</f>
-        <v>-3100537.00837137</v>
+        <v>-3042543.87986797</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(K12&gt;0,L12/K12,"")</f>
-        <v>-0.0751644041623921</v>
+        <v>-0.0737585125579048</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2519,11 +2525,11 @@
       </c>
       <c r="C17" s="7" t="n">
         <f aca="false">LARGE('Side by Side'!$I$7:$I$95,A17)</f>
-        <v>13235530.8</v>
+        <v>13271834.8</v>
       </c>
       <c r="D17" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C17,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.346938203829812</v>
+        <v>0.347361784453381</v>
       </c>
       <c r="E17" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C17,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2535,7 +2541,7 @@
       </c>
       <c r="G17" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C17,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.305628125337199</v>
+        <v>0.307226421688238</v>
       </c>
       <c r="H17" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C17,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2568,7 +2574,7 @@
       </c>
       <c r="D18" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C18,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0803198068074013</v>
+        <v>0.0801978937387302</v>
       </c>
       <c r="E18" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C18,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2580,7 +2586,7 @@
       </c>
       <c r="G18" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C18,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0613913539222327</v>
+        <v>0.061085084888777</v>
       </c>
       <c r="H18" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C18,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2613,7 +2619,7 @@
       </c>
       <c r="D19" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C19,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0750978948668107</v>
+        <v>0.0749839078544177</v>
       </c>
       <c r="E19" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C19,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2625,7 +2631,7 @@
       </c>
       <c r="G19" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C19,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.247667747990467</v>
+        <v>0.246432183746497</v>
       </c>
       <c r="H19" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C19,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2654,11 +2660,11 @@
       </c>
       <c r="C20" s="7" t="n">
         <f aca="false">LARGE('Side by Side'!$I$7:$I$95,A20)</f>
-        <v>2538564</v>
+        <v>2548016.1</v>
       </c>
       <c r="D20" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C20,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0665424642030241</v>
+        <v>0.0666888514398886</v>
       </c>
       <c r="E20" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C20,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2670,7 +2676,7 @@
       </c>
       <c r="G20" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C20,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0591290750864015</v>
+        <v>0.0596471990037228</v>
       </c>
       <c r="H20" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C20,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2699,11 +2705,11 @@
       </c>
       <c r="C21" s="7" t="n">
         <f aca="false">LARGE('Side by Side'!$I$7:$I$95,A21)</f>
-        <v>2511795.9</v>
+        <v>2520203.25</v>
       </c>
       <c r="D21" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C21,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0658408016347245</v>
+        <v>0.0659609097986368</v>
       </c>
       <c r="E21" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C21,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2715,7 +2721,7 @@
       </c>
       <c r="G21" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C21,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.048249628624683</v>
+        <v>0.0487321543842632</v>
       </c>
       <c r="H21" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C21,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2748,7 +2754,7 @@
       </c>
       <c r="D22" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C22,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0413918555426262</v>
+        <v>0.0413290290951063</v>
       </c>
       <c r="E22" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C22,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2760,7 +2766,7 @@
       </c>
       <c r="G22" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C22,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.040955926603317</v>
+        <v>0.0407516057787434</v>
       </c>
       <c r="H22" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C22,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2793,7 +2799,7 @@
       </c>
       <c r="D23" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C23,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0305271671275344</v>
+        <v>0.0304808315999692</v>
       </c>
       <c r="E23" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C23,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2805,7 +2811,7 @@
       </c>
       <c r="G23" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C23,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.00607043805098872</v>
+        <v>0.00604015386476791</v>
       </c>
       <c r="H23" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C23,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2834,11 +2840,11 @@
       </c>
       <c r="C24" s="7" t="n">
         <f aca="false">LARGE('Side by Side'!$I$7:$I$95,A24)</f>
-        <v>1101614.37</v>
+        <v>1105324.29</v>
       </c>
       <c r="D24" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C24,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0288762208797029</v>
+        <v>0.0289294904253982</v>
       </c>
       <c r="E24" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C24,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2850,7 +2856,7 @@
       </c>
       <c r="G24" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C24,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0251381588851207</v>
+        <v>0.0253318916426757</v>
       </c>
       <c r="H24" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C24,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2883,7 +2889,7 @@
       </c>
       <c r="D25" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C25,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0274090372959589</v>
+        <v>0.0273674346081675</v>
       </c>
       <c r="E25" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C25,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2895,7 +2901,7 @@
       </c>
       <c r="G25" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C25,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0229480070702708</v>
+        <v>0.0228335241097867</v>
       </c>
       <c r="H25" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C25,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2928,7 +2934,7 @@
       </c>
       <c r="D26" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$L$7:$L$95,MATCH(C26,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0263551607267504</v>
+        <v>0.026315157660916</v>
       </c>
       <c r="E26" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$S$7:$S$95,MATCH(C26,'Side by Side'!$I$7:$I$95,0))</f>
@@ -2940,7 +2946,7 @@
       </c>
       <c r="G26" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AG$7:$AG$95,MATCH(C26,'Side by Side'!$I$7:$I$95,0))</f>
-        <v>0.0251350309341946</v>
+        <v>0.0250096373545084</v>
       </c>
       <c r="H26" s="28" t="n">
         <f aca="false">INDEX('Side by Side'!$AN$7:$AN$95,MATCH(C26,'Side by Side'!$I$7:$I$95,0))</f>
@@ -3056,12 +3062,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -3387,19 +3393,19 @@
       <c r="G6" s="43"/>
       <c r="H6" s="43" t="n">
         <f aca="false">SUM(H7:H95)</f>
-        <v>37595951.23</v>
+        <v>37654259.08</v>
       </c>
       <c r="I6" s="43" t="n">
         <f aca="false">SUM(I7:I95)</f>
-        <v>38149533.9916286</v>
+        <v>38207527.120132</v>
       </c>
       <c r="J6" s="43" t="n">
         <f aca="false">I6-H6</f>
-        <v>553582.761628628</v>
+        <v>553268.040132031</v>
       </c>
       <c r="K6" s="44" t="n">
         <f aca="false">IF(H6&gt;0,J6/H6,"")</f>
-        <v>0.0147245313263119</v>
+        <v>0.0146933721084927</v>
       </c>
       <c r="L6" s="44" t="n">
         <f aca="false">SUM(L7:L95)</f>
@@ -3462,19 +3468,19 @@
       <c r="AB6" s="43"/>
       <c r="AC6" s="43" t="n">
         <f aca="false">SUM(AC7:AC95)</f>
-        <v>9857778</v>
+        <v>9916085.85</v>
       </c>
       <c r="AD6" s="43" t="n">
         <f aca="false">SUM(AD7:AD95)</f>
-        <v>11566677.6285714</v>
+        <v>11624670.7570748</v>
       </c>
       <c r="AE6" s="43" t="n">
         <f aca="false">AD6-AC6</f>
-        <v>1708899.62857143</v>
+        <v>1708584.90707483</v>
       </c>
       <c r="AF6" s="44" t="n">
         <f aca="false">IF(AC6&gt;0,AE6/AC6,"")</f>
-        <v>0.173355458864201</v>
+        <v>0.172304368167086</v>
       </c>
       <c r="AG6" s="44" t="n">
         <f aca="false">SUM(AG7:AG95)</f>
@@ -3577,31 +3583,31 @@
       </c>
       <c r="F7" s="47" t="n">
         <f aca="false">M7+T7+AA7+AH7+AO7+AV7</f>
-        <v>14583</v>
+        <v>14623</v>
       </c>
       <c r="G7" s="48" t="n">
         <f aca="false">IF(AND(F7&gt;0,H7&gt;0),H7/F7,"")</f>
-        <v>879.710464239183</v>
+        <v>879.798789578062</v>
       </c>
       <c r="H7" s="48" t="n">
         <f aca="false">O7+V7+AC7+AJ7+AQ7+AX7</f>
-        <v>12828817.7</v>
+        <v>12865297.7</v>
       </c>
       <c r="I7" s="49" t="n">
         <f aca="false">P7+W7+AD7+AK7+AR7+AY7</f>
-        <v>13235530.8</v>
+        <v>13271834.8</v>
       </c>
       <c r="J7" s="48" t="n">
         <f aca="false">I7-H7</f>
-        <v>406713.100000002</v>
+        <v>406537.100000002</v>
       </c>
       <c r="K7" s="50" t="n">
         <f aca="false">IF(H7&gt;0,J7/H7,"")</f>
-        <v>0.0317030851564756</v>
+        <v>0.0315995097416208</v>
       </c>
       <c r="L7" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I7/I$6)</f>
-        <v>0.346938203829812</v>
+        <v>0.347361784453381</v>
       </c>
       <c r="M7" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B7)</f>
@@ -3661,31 +3667,31 @@
       </c>
       <c r="AA7" s="52" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$D$7:$D$300,'Manish Shilpa'!$B$7:$B$300,$B7)</f>
-        <v>3895</v>
+        <v>3935</v>
       </c>
       <c r="AB7" s="8" t="n">
         <f aca="false">IF(AND(AA7&gt;0,AC7&gt;0),AC7/AA7,"")</f>
-        <v>747.725032092426</v>
+        <v>749.394917407878</v>
       </c>
       <c r="AC7" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$E$7:$E$300,'Manish Shilpa'!$B$7:$B$300,$B7)</f>
-        <v>2912389</v>
+        <v>2948869</v>
       </c>
       <c r="AD7" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$H$7:$H$300,'Manish Shilpa'!$B$7:$B$300,$B7)</f>
-        <v>3535102</v>
+        <v>3571406</v>
       </c>
       <c r="AE7" s="8" t="n">
         <f aca="false">AD7-AC7</f>
-        <v>622713</v>
+        <v>622537</v>
       </c>
       <c r="AF7" s="9" t="n">
         <f aca="false">IF(AC7&gt;0,AE7/AC7,"")</f>
-        <v>0.213815187462939</v>
+        <v>0.211110429117062</v>
       </c>
       <c r="AG7" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD7/AD$6)</f>
-        <v>0.305628125337199</v>
+        <v>0.307226421688238</v>
       </c>
       <c r="AH7" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B7)</f>
@@ -3817,7 +3823,7 @@
       </c>
       <c r="L8" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I8/I$6)</f>
-        <v>0.0803198068074013</v>
+        <v>0.0801978937387302</v>
       </c>
       <c r="M8" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B8)</f>
@@ -3901,7 +3907,7 @@
       </c>
       <c r="AG8" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD8/AD$6)</f>
-        <v>0.0613913539222327</v>
+        <v>0.061085084888777</v>
       </c>
       <c r="AH8" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B8)</f>
@@ -4033,7 +4039,7 @@
       </c>
       <c r="L9" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I9/I$6)</f>
-        <v>0.0750978948668107</v>
+        <v>0.0749839078544177</v>
       </c>
       <c r="M9" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B9)</f>
@@ -4117,7 +4123,7 @@
       </c>
       <c r="AG9" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD9/AD$6)</f>
-        <v>0.247667747990467</v>
+        <v>0.246432183746497</v>
       </c>
       <c r="AH9" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B9)</f>
@@ -4225,31 +4231,31 @@
       </c>
       <c r="F10" s="47" t="n">
         <f aca="false">M10+T10+AA10+AH10+AO10+AV10</f>
-        <v>3760</v>
+        <v>3774</v>
       </c>
       <c r="G10" s="48" t="n">
         <f aca="false">IF(AND(F10&gt;0,H10&gt;0),H10/F10,"")</f>
-        <v>788.801954787234</v>
+        <v>788.399085850556</v>
       </c>
       <c r="H10" s="48" t="n">
         <f aca="false">O10+V10+AC10+AJ10+AQ10+AX10</f>
-        <v>2965895.35</v>
+        <v>2975418.15</v>
       </c>
       <c r="I10" s="49" t="n">
         <f aca="false">P10+W10+AD10+AK10+AR10+AY10</f>
-        <v>2538564</v>
+        <v>2548016.1</v>
       </c>
       <c r="J10" s="48" t="n">
         <f aca="false">I10-H10</f>
-        <v>-427331.35</v>
+        <v>-427402.05</v>
       </c>
       <c r="K10" s="50" t="n">
         <f aca="false">IF(H10&gt;0,J10/H10,"")</f>
-        <v>-0.144081735722739</v>
+        <v>-0.143644364742482</v>
       </c>
       <c r="L10" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I10/I$6)</f>
-        <v>0.0665424642030241</v>
+        <v>0.0666888514398886</v>
       </c>
       <c r="M10" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B10)</f>
@@ -4309,31 +4315,31 @@
       </c>
       <c r="AA10" s="52" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$D$7:$D$300,'Manish Shilpa'!$B$7:$B$300,$B10)</f>
-        <v>1013</v>
+        <v>1027</v>
       </c>
       <c r="AB10" s="8" t="n">
         <f aca="false">IF(AND(AA10&gt;0,AC10&gt;0),AC10/AA10,"")</f>
-        <v>802.253701875617</v>
+        <v>800.589873417722</v>
       </c>
       <c r="AC10" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$E$7:$E$300,'Manish Shilpa'!$B$7:$B$300,$B10)</f>
-        <v>812683</v>
+        <v>822205.8</v>
       </c>
       <c r="AD10" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$H$7:$H$300,'Manish Shilpa'!$B$7:$B$300,$B10)</f>
-        <v>683926.95</v>
+        <v>693379.05</v>
       </c>
       <c r="AE10" s="8" t="n">
         <f aca="false">AD10-AC10</f>
-        <v>-128756.05</v>
+        <v>-128826.75</v>
       </c>
       <c r="AF10" s="9" t="n">
         <f aca="false">IF(AC10&gt;0,AE10/AC10,"")</f>
-        <v>-0.158433300561228</v>
+        <v>-0.156684311883959</v>
       </c>
       <c r="AG10" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD10/AD$6)</f>
-        <v>0.0591290750864015</v>
+        <v>0.0596471990037228</v>
       </c>
       <c r="AH10" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B10)</f>
@@ -4441,31 +4447,31 @@
       </c>
       <c r="F11" s="47" t="n">
         <f aca="false">M11+T11+AA11+AH11+AO11+AV11</f>
-        <v>6274</v>
+        <v>6295</v>
       </c>
       <c r="G11" s="48" t="n">
         <f aca="false">IF(AND(F11&gt;0,H11&gt;0),H11/F11,"")</f>
-        <v>447.776880777813</v>
+        <v>447.626838760921</v>
       </c>
       <c r="H11" s="48" t="n">
         <f aca="false">O11+V11+AC11+AJ11+AQ11+AX11</f>
-        <v>2809352.15</v>
+        <v>2817810.95</v>
       </c>
       <c r="I11" s="49" t="n">
         <f aca="false">P11+W11+AD11+AK11+AR11+AY11</f>
-        <v>2511795.9</v>
+        <v>2520203.25</v>
       </c>
       <c r="J11" s="48" t="n">
         <f aca="false">I11-H11</f>
-        <v>-297556.25</v>
+        <v>-297607.700000001</v>
       </c>
       <c r="K11" s="50" t="n">
         <f aca="false">IF(H11&gt;0,J11/H11,"")</f>
-        <v>-0.105916323092497</v>
+        <v>-0.105616631236386</v>
       </c>
       <c r="L11" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I11/I$6)</f>
-        <v>0.0658408016347245</v>
+        <v>0.0659609097986368</v>
       </c>
       <c r="M11" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B11)</f>
@@ -4525,31 +4531,31 @@
       </c>
       <c r="AA11" s="52" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$D$7:$D$300,'Manish Shilpa'!$B$7:$B$300,$B11)</f>
-        <v>1394</v>
+        <v>1415</v>
       </c>
       <c r="AB11" s="8" t="n">
         <f aca="false">IF(AND(AA11&gt;0,AC11&gt;0),AC11/AA11,"")</f>
-        <v>446.56599713056</v>
+        <v>445.916466431095</v>
       </c>
       <c r="AC11" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$E$7:$E$300,'Manish Shilpa'!$B$7:$B$300,$B11)</f>
-        <v>622513</v>
+        <v>630971.8</v>
       </c>
       <c r="AD11" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$H$7:$H$300,'Manish Shilpa'!$B$7:$B$300,$B11)</f>
-        <v>558087.9</v>
+        <v>566495.25</v>
       </c>
       <c r="AE11" s="8" t="n">
         <f aca="false">AD11-AC11</f>
-        <v>-64425.1</v>
+        <v>-64476.5500000001</v>
       </c>
       <c r="AF11" s="9" t="n">
         <f aca="false">IF(AC11&gt;0,AE11/AC11,"")</f>
-        <v>-0.103491975267986</v>
+        <v>-0.102186104038247</v>
       </c>
       <c r="AG11" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD11/AD$6)</f>
-        <v>0.048249628624683</v>
+        <v>0.0487321543842632</v>
       </c>
       <c r="AH11" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B11)</f>
@@ -4681,7 +4687,7 @@
       </c>
       <c r="L12" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I12/I$6)</f>
-        <v>0.0413918555426262</v>
+        <v>0.0413290290951063</v>
       </c>
       <c r="M12" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B12)</f>
@@ -4765,7 +4771,7 @@
       </c>
       <c r="AG12" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD12/AD$6)</f>
-        <v>0.040955926603317</v>
+        <v>0.0407516057787434</v>
       </c>
       <c r="AH12" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B12)</f>
@@ -4897,7 +4903,7 @@
       </c>
       <c r="L13" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I13/I$6)</f>
-        <v>0.0305271671275344</v>
+        <v>0.0304808315999692</v>
       </c>
       <c r="M13" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B13)</f>
@@ -4981,7 +4987,7 @@
       </c>
       <c r="AG13" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD13/AD$6)</f>
-        <v>0.00607043805098872</v>
+        <v>0.00604015386476791</v>
       </c>
       <c r="AH13" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B13)</f>
@@ -5089,31 +5095,31 @@
       </c>
       <c r="F14" s="47" t="n">
         <f aca="false">M14+T14+AA14+AH14+AO14+AV14</f>
-        <v>14253</v>
+        <v>14301</v>
       </c>
       <c r="G14" s="48" t="n">
         <f aca="false">IF(AND(F14&gt;0,H14&gt;0),H14/F14,"")</f>
-        <v>99.4292380551463</v>
+        <v>99.356104468219</v>
       </c>
       <c r="H14" s="48" t="n">
         <f aca="false">O14+V14+AC14+AJ14+AQ14+AX14</f>
-        <v>1417164.93</v>
+        <v>1420891.65</v>
       </c>
       <c r="I14" s="49" t="n">
         <f aca="false">P14+W14+AD14+AK14+AR14+AY14</f>
-        <v>1101614.37</v>
+        <v>1105324.29</v>
       </c>
       <c r="J14" s="48" t="n">
         <f aca="false">I14-H14</f>
-        <v>-315550.56</v>
+        <v>-315567.36</v>
       </c>
       <c r="K14" s="50" t="n">
         <f aca="false">IF(H14&gt;0,J14/H14,"")</f>
-        <v>-0.222663257691538</v>
+        <v>-0.222091079217757</v>
       </c>
       <c r="L14" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I14/I$6)</f>
-        <v>0.0288762208797029</v>
+        <v>0.0289294904253982</v>
       </c>
       <c r="M14" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B14)</f>
@@ -5173,31 +5179,31 @@
       </c>
       <c r="AA14" s="52" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$D$7:$D$300,'Manish Shilpa'!$B$7:$B$300,$B14)</f>
-        <v>3762</v>
+        <v>3810</v>
       </c>
       <c r="AB14" s="8" t="n">
         <f aca="false">IF(AND(AA14&gt;0,AC14&gt;0),AC14/AA14,"")</f>
-        <v>115.016746411483</v>
+        <v>114.545858267717</v>
       </c>
       <c r="AC14" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$E$7:$E$300,'Manish Shilpa'!$B$7:$B$300,$B14)</f>
-        <v>432693</v>
+        <v>436419.72</v>
       </c>
       <c r="AD14" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$H$7:$H$300,'Manish Shilpa'!$B$7:$B$300,$B14)</f>
-        <v>290764.98</v>
+        <v>294474.9</v>
       </c>
       <c r="AE14" s="8" t="n">
         <f aca="false">AD14-AC14</f>
-        <v>-141928.02</v>
+        <v>-141944.82</v>
       </c>
       <c r="AF14" s="9" t="n">
         <f aca="false">IF(AC14&gt;0,AE14/AC14,"")</f>
-        <v>-0.328010899182561</v>
+        <v>-0.325248409948111</v>
       </c>
       <c r="AG14" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD14/AD$6)</f>
-        <v>0.0251381588851207</v>
+        <v>0.0253318916426757</v>
       </c>
       <c r="AH14" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B14)</f>
@@ -5329,7 +5335,7 @@
       </c>
       <c r="L15" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I15/I$6)</f>
-        <v>0.0274090372959589</v>
+        <v>0.0273674346081675</v>
       </c>
       <c r="M15" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B15)</f>
@@ -5413,7 +5419,7 @@
       </c>
       <c r="AG15" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD15/AD$6)</f>
-        <v>0.0229480070702708</v>
+        <v>0.0228335241097867</v>
       </c>
       <c r="AH15" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B15)</f>
@@ -5545,7 +5551,7 @@
       </c>
       <c r="L16" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I16/I$6)</f>
-        <v>0.0263551607267504</v>
+        <v>0.026315157660916</v>
       </c>
       <c r="M16" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B16)</f>
@@ -5629,7 +5635,7 @@
       </c>
       <c r="AG16" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD16/AD$6)</f>
-        <v>0.0251350309341946</v>
+        <v>0.0250096373545084</v>
       </c>
       <c r="AH16" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B16)</f>
@@ -5761,7 +5767,7 @@
       </c>
       <c r="L17" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I17/I$6)</f>
-        <v>0.0248286125908602</v>
+        <v>0.0247909265894601</v>
       </c>
       <c r="M17" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B17)</f>
@@ -5845,7 +5851,7 @@
       </c>
       <c r="AG17" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD17/AD$6)</f>
-        <v>0.0163780824609527</v>
+        <v>0.0162963755239869</v>
       </c>
       <c r="AH17" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B17)</f>
@@ -5977,7 +5983,7 @@
       </c>
       <c r="L18" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I18/I$6)</f>
-        <v>0.022031723904791</v>
+        <v>0.0219982831486922</v>
       </c>
       <c r="M18" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B18)</f>
@@ -6193,7 +6199,7 @@
       </c>
       <c r="L19" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I19/I$6)</f>
-        <v>0.019017113031032</v>
+        <v>0.0189882479889081</v>
       </c>
       <c r="M19" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B19)</f>
@@ -6277,7 +6283,7 @@
       </c>
       <c r="AG19" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD19/AD$6)</f>
-        <v>0.0102404513900704</v>
+        <v>0.0101893638516955</v>
       </c>
       <c r="AH19" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B19)</f>
@@ -6409,7 +6415,7 @@
       </c>
       <c r="L20" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I20/I$6)</f>
-        <v>0.0185609499228845</v>
+        <v>0.0185327772659461</v>
       </c>
       <c r="M20" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B20)</f>
@@ -6493,7 +6499,7 @@
       </c>
       <c r="AG20" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD20/AD$6)</f>
-        <v>0.0151326945922343</v>
+        <v>0.0150572006431643</v>
       </c>
       <c r="AH20" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B20)</f>
@@ -6625,7 +6631,7 @@
       </c>
       <c r="L21" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I21/I$6)</f>
-        <v>0.0123764552432962</v>
+        <v>0.0123576696946507</v>
       </c>
       <c r="M21" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B21)</f>
@@ -6709,7 +6715,7 @@
       </c>
       <c r="AG21" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD21/AD$6)</f>
-        <v>0.00547590259138421</v>
+        <v>0.00544858442218264</v>
       </c>
       <c r="AH21" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B21)</f>
@@ -6841,7 +6847,7 @@
       </c>
       <c r="L22" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I22/I$6)</f>
-        <v>0.0107914817541504</v>
+        <v>0.0107751019506069</v>
       </c>
       <c r="M22" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B22)</f>
@@ -6925,7 +6931,7 @@
       </c>
       <c r="AG22" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD22/AD$6)</f>
-        <v>0.00557619932630266</v>
+        <v>0.00554838079699988</v>
       </c>
       <c r="AH22" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B22)</f>
@@ -7057,7 +7063,7 @@
       </c>
       <c r="L23" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I23/I$6)</f>
-        <v>0.00937167410953051</v>
+        <v>0.00935744935483185</v>
       </c>
       <c r="M23" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B23)</f>
@@ -7141,7 +7147,7 @@
       </c>
       <c r="AG23" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD23/AD$6)</f>
-        <v>0.00370918956831849</v>
+        <v>0.00369068517264362</v>
       </c>
       <c r="AH23" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B23)</f>
@@ -7273,7 +7279,7 @@
       </c>
       <c r="L24" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I24/I$6)</f>
-        <v>0.00826694711576833</v>
+        <v>0.00825439916612196</v>
       </c>
       <c r="M24" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B24)</f>
@@ -7357,7 +7363,7 @@
       </c>
       <c r="AG24" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD24/AD$6)</f>
-        <v>0.0272662721420509</v>
+        <v>0.0271302462315381</v>
       </c>
       <c r="AH24" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B24)</f>
@@ -7489,7 +7495,7 @@
       </c>
       <c r="L25" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I25/I$6)</f>
-        <v>0.00746064159164974</v>
+        <v>0.0074493174893287</v>
       </c>
       <c r="M25" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B25)</f>
@@ -7705,7 +7711,7 @@
       </c>
       <c r="L26" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I26/I$6)</f>
-        <v>0.00588562366316901</v>
+        <v>0.00587669019494565</v>
       </c>
       <c r="M26" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B26)</f>
@@ -7789,7 +7795,7 @@
       </c>
       <c r="AG26" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD26/AD$6)</f>
-        <v>0.00245723110063977</v>
+        <v>0.00244497247224849</v>
       </c>
       <c r="AH26" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B26)</f>
@@ -7921,7 +7927,7 @@
       </c>
       <c r="L27" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I27/I$6)</f>
-        <v>0.00570621649134086</v>
+        <v>0.00569755533551128</v>
       </c>
       <c r="M27" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B27)</f>
@@ -8005,7 +8011,7 @@
       </c>
       <c r="AG27" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD27/AD$6)</f>
-        <v>0.00325542054591268</v>
+        <v>0.00323917991200597</v>
       </c>
       <c r="AH27" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B27)</f>
@@ -8137,7 +8143,7 @@
       </c>
       <c r="L28" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I28/I$6)</f>
-        <v>0.00539162287133403</v>
+        <v>0.00538343922005935</v>
       </c>
       <c r="M28" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B28)</f>
@@ -8221,7 +8227,7 @@
       </c>
       <c r="AG28" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD28/AD$6)</f>
-        <v>0.00158276218875317</v>
+        <v>0.00157486610869027</v>
       </c>
       <c r="AH28" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B28)</f>
@@ -8353,7 +8359,7 @@
       </c>
       <c r="L29" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I29/I$6)</f>
-        <v>0.00517861371631308</v>
+        <v>0.0051707533800559</v>
       </c>
       <c r="M29" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B29)</f>
@@ -8437,7 +8443,7 @@
       </c>
       <c r="AG29" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD29/AD$6)</f>
-        <v>0.00162669010101251</v>
+        <v>0.0016185748734904</v>
       </c>
       <c r="AH29" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B29)</f>
@@ -8569,7 +8575,7 @@
       </c>
       <c r="L30" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I30/I$6)</f>
-        <v>0.00428559363361755</v>
+        <v>0.00427908876400047</v>
       </c>
       <c r="M30" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B30)</f>
@@ -8653,7 +8659,7 @@
       </c>
       <c r="AG30" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD30/AD$6)</f>
-        <v>0.0141348626848687</v>
+        <v>0.0140643467171315</v>
       </c>
       <c r="AH30" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B30)</f>
@@ -8785,7 +8791,7 @@
       </c>
       <c r="L31" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I31/I$6)</f>
-        <v>0.00380200974491138</v>
+        <v>0.00379623888099196</v>
       </c>
       <c r="M31" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B31)</f>
@@ -8869,7 +8875,7 @@
       </c>
       <c r="AG31" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD31/AD$6)</f>
-        <v>0.000344502555354104</v>
+        <v>0.000342783901864477</v>
       </c>
       <c r="AH31" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B31)</f>
@@ -9001,7 +9007,7 @@
       </c>
       <c r="L32" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I32/I$6)</f>
-        <v>0.00331888719866889</v>
+        <v>0.00331384964020049</v>
       </c>
       <c r="M32" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B32)</f>
@@ -9085,7 +9091,7 @@
       </c>
       <c r="AG32" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD32/AD$6)</f>
-        <v>0.00113239085765181</v>
+        <v>0.00112674158896315</v>
       </c>
       <c r="AH32" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B32)</f>
@@ -9217,7 +9223,7 @@
       </c>
       <c r="L33" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I33/I$6)</f>
-        <v>0.00252005437395635</v>
+        <v>0.00251622932040905</v>
       </c>
       <c r="M33" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B33)</f>
@@ -9433,7 +9439,7 @@
       </c>
       <c r="L34" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I34/I$6)</f>
-        <v>0.00241921696920996</v>
+        <v>0.00241554497127793</v>
       </c>
       <c r="M34" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B34)</f>
@@ -9649,7 +9655,7 @@
       </c>
       <c r="L35" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I35/I$6)</f>
-        <v>0.00241159643051442</v>
+        <v>0.00240793599938383</v>
       </c>
       <c r="M35" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B35)</f>
@@ -9733,7 +9739,7 @@
       </c>
       <c r="AG35" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD35/AD$6)</f>
-        <v>0.000568142401044131</v>
+        <v>0.000565308053649652</v>
       </c>
       <c r="AH35" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B35)</f>
@@ -9865,7 +9871,7 @@
       </c>
       <c r="L36" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I36/I$6)</f>
-        <v>0.00222874544204544</v>
+        <v>0.00222536255049071</v>
       </c>
       <c r="M36" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B36)</f>
@@ -9949,7 +9955,7 @@
       </c>
       <c r="AG36" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD36/AD$6)</f>
-        <v>0.00735090945994501</v>
+        <v>0.00731423726115022</v>
       </c>
       <c r="AH36" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B36)</f>
@@ -10081,7 +10087,7 @@
       </c>
       <c r="L37" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I37/I$6)</f>
-        <v>0.00214011002121063</v>
+        <v>0.00213686166454307</v>
       </c>
       <c r="M37" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B37)</f>
@@ -10297,7 +10303,7 @@
       </c>
       <c r="L38" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I38/I$6)</f>
-        <v>0.00204655186658722</v>
+        <v>0.00204344551675686</v>
       </c>
       <c r="M38" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B38)</f>
@@ -10381,7 +10387,7 @@
       </c>
       <c r="AG38" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD38/AD$6)</f>
-        <v>0.00674999360292908</v>
+        <v>0.00671631925166424</v>
       </c>
       <c r="AH38" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B38)</f>
@@ -10513,7 +10519,7 @@
       </c>
       <c r="L39" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I39/I$6)</f>
-        <v>0.00185962953087625</v>
+        <v>0.00185680690029842</v>
       </c>
       <c r="M39" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B39)</f>
@@ -10597,7 +10603,7 @@
       </c>
       <c r="AG39" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD39/AD$6)</f>
-        <v>0.00613348121890747</v>
+        <v>0.00610288252308764</v>
       </c>
       <c r="AH39" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B39)</f>
@@ -10729,7 +10735,7 @@
       </c>
       <c r="L40" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I40/I$6)</f>
-        <v>0.00184557955584595</v>
+        <v>0.00184277825096147</v>
       </c>
       <c r="M40" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B40)</f>
@@ -10813,7 +10819,7 @@
       </c>
       <c r="AG40" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD40/AD$6)</f>
-        <v>0.00608714120518771</v>
+        <v>0.00605677369031285</v>
       </c>
       <c r="AH40" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B40)</f>
@@ -10945,7 +10951,7 @@
       </c>
       <c r="L41" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I41/I$6)</f>
-        <v>0.00176489704998165</v>
+        <v>0.00176221820868703</v>
       </c>
       <c r="M41" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B41)</f>
@@ -11029,7 +11035,7 @@
       </c>
       <c r="AG41" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD41/AD$6)</f>
-        <v>0.00582103194729702</v>
+        <v>0.00579199199762476</v>
       </c>
       <c r="AH41" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B41)</f>
@@ -11125,155 +11131,155 @@
       </c>
       <c r="C42" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH($B42,Prices!$A$6:$A$300,0)),"")</f>
-        <v>473.4</v>
+        <v>119.758503401361</v>
       </c>
       <c r="D42" s="46" t="str">
         <f aca="false">IFERROR(INDEX(Prices!$D$6:$D$300,MATCH($B42,Prices!$A$6:$A$300,0)),"")</f>
-        <v>Close 28.10.2026 live (~11:35 IST) (Screener.in)</v>
+        <v>DA stmt – 23.10</v>
       </c>
       <c r="E42" s="6" t="n">
         <f aca="false">(M42&gt;0)+(T42&gt;0)+(AA42&gt;0)+(AH42&gt;0)+(AO42&gt;0)+(AV42&gt;0)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F42" s="47" t="n">
         <f aca="false">M42+T42+AA42+AH42+AO42+AV42</f>
-        <v>127</v>
+        <v>503</v>
       </c>
       <c r="G42" s="48" t="n">
         <f aca="false">IF(AND(F42&gt;0,H42&gt;0),H42/F42,"")</f>
-        <v>606.212598425197</v>
+        <v>115.741292246521</v>
       </c>
       <c r="H42" s="48" t="n">
         <f aca="false">O42+V42+AC42+AJ42+AQ42+AX42</f>
-        <v>76989</v>
+        <v>58217.87</v>
       </c>
       <c r="I42" s="49" t="n">
         <f aca="false">P42+W42+AD42+AK42+AR42+AY42</f>
-        <v>60121.8</v>
+        <v>60238.5272108843</v>
       </c>
       <c r="J42" s="48" t="n">
         <f aca="false">I42-H42</f>
-        <v>-16867.2</v>
+        <v>2020.65721088433</v>
       </c>
       <c r="K42" s="50" t="n">
         <f aca="false">IF(H42&gt;0,J42/H42,"")</f>
-        <v>-0.219085843432179</v>
+        <v>0.0347085389912811</v>
       </c>
       <c r="L42" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I42/I$6)</f>
-        <v>0.00157595109846408</v>
+        <v>0.00157661413211806</v>
       </c>
       <c r="M42" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B42)</f>
-        <v>0</v>
-      </c>
-      <c r="N42" s="8" t="str">
+        <v>29</v>
+      </c>
+      <c r="N42" s="8" t="n">
         <f aca="false">IF(AND(M42&gt;0,O42&gt;0),O42/M42,"")</f>
-        <v/>
+        <v>134.94275862069</v>
       </c>
       <c r="O42" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$E$7:$E$300,Gautam!$B$7:$B$300,$B42)</f>
-        <v>0</v>
+        <v>3913.34</v>
       </c>
       <c r="P42" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$H$7:$H$300,Gautam!$B$7:$B$300,$B42)</f>
-        <v>0</v>
+        <v>3472.99659863945</v>
       </c>
       <c r="Q42" s="8" t="n">
         <f aca="false">P42-O42</f>
-        <v>0</v>
-      </c>
-      <c r="R42" s="9" t="str">
+        <v>-440.343401360546</v>
+      </c>
+      <c r="R42" s="9" t="n">
         <f aca="false">IF(O42&gt;0,Q42/O42,"")</f>
-        <v/>
+        <v>-0.11252367577582</v>
       </c>
       <c r="S42" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P42/P$6)</f>
-        <v>0</v>
+        <v>0.000623575931000622</v>
       </c>
       <c r="T42" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B42)</f>
-        <v>127</v>
+        <v>294</v>
       </c>
       <c r="U42" s="8" t="n">
         <f aca="false">IF(AND(T42&gt;0,V42&gt;0),V42/T42,"")</f>
-        <v>606.212598425197</v>
+        <v>127.360544217687</v>
       </c>
       <c r="V42" s="8" t="n">
         <f aca="false">SUMIFS(DA!$E$7:$E$300,DA!$B$7:$B$300,$B42)</f>
-        <v>76989</v>
+        <v>37444</v>
       </c>
       <c r="W42" s="8" t="n">
         <f aca="false">SUMIFS(DA!$H$7:$H$300,DA!$B$7:$B$300,$B42)</f>
-        <v>60121.8</v>
+        <v>35209</v>
       </c>
       <c r="X42" s="8" t="n">
         <f aca="false">W42-V42</f>
-        <v>-16867.2</v>
+        <v>-2235.00000000001</v>
       </c>
       <c r="Y42" s="9" t="n">
         <f aca="false">IF(V42&gt;0,X42/V42,"")</f>
-        <v>-0.219085843432179</v>
+        <v>-0.0596891357760927</v>
       </c>
       <c r="Z42" s="9" t="n">
         <f aca="false">IF(W$6=0,"",W42/W$6)</f>
-        <v>0.0151373160834967</v>
+        <v>0.00886483375387686</v>
       </c>
       <c r="AA42" s="52" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$D$7:$D$300,'Manish Shilpa'!$B$7:$B$300,$B42)</f>
-        <v>0</v>
-      </c>
-      <c r="AB42" s="8" t="str">
+        <v>169</v>
+      </c>
+      <c r="AB42" s="8" t="n">
         <f aca="false">IF(AND(AA42&gt;0,AC42&gt;0),AC42/AA42,"")</f>
-        <v/>
+        <v>91.559349112426</v>
       </c>
       <c r="AC42" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$E$7:$E$300,'Manish Shilpa'!$B$7:$B$300,$B42)</f>
-        <v>0</v>
+        <v>15473.53</v>
       </c>
       <c r="AD42" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$H$7:$H$300,'Manish Shilpa'!$B$7:$B$300,$B42)</f>
-        <v>0</v>
+        <v>20239.1870748299</v>
       </c>
       <c r="AE42" s="8" t="n">
         <f aca="false">AD42-AC42</f>
-        <v>0</v>
-      </c>
-      <c r="AF42" s="9" t="str">
+        <v>4765.65707482993</v>
+      </c>
+      <c r="AF42" s="9" t="n">
         <f aca="false">IF(AC42&gt;0,AE42/AC42,"")</f>
-        <v/>
+        <v>0.3079877102917</v>
       </c>
       <c r="AG42" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD42/AD$6)</f>
-        <v>0</v>
+        <v>0.00174105464987146</v>
       </c>
       <c r="AH42" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B42)</f>
-        <v>0</v>
-      </c>
-      <c r="AI42" s="8" t="str">
+        <v>11</v>
+      </c>
+      <c r="AI42" s="8" t="n">
         <f aca="false">IF(AND(AH42&gt;0,AJ42&gt;0),AJ42/AH42,"")</f>
-        <v/>
+        <v>126.090909090909</v>
       </c>
       <c r="AJ42" s="8" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$E$7:$E$300,'Saloni Mehra'!$B$7:$B$300,$B42)</f>
-        <v>0</v>
+        <v>1387</v>
       </c>
       <c r="AK42" s="8" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$H$7:$H$300,'Saloni Mehra'!$B$7:$B$300,$B42)</f>
-        <v>0</v>
+        <v>1317.34353741497</v>
       </c>
       <c r="AL42" s="8" t="n">
         <f aca="false">AK42-AJ42</f>
-        <v>0</v>
-      </c>
-      <c r="AM42" s="9" t="str">
+        <v>-69.6564625850344</v>
+      </c>
+      <c r="AM42" s="9" t="n">
         <f aca="false">IF(AJ42&gt;0,AL42/AJ42,"")</f>
-        <v/>
+        <v>-0.0502209535580638</v>
       </c>
       <c r="AN42" s="9" t="n">
         <f aca="false">IF(AK$6=0,"",AK42/AK$6)</f>
-        <v>0</v>
+        <v>0.000113903544031896</v>
       </c>
       <c r="AO42" s="52" t="n">
         <f aca="false">SUMIFS('Vidushi Malhotra'!$D$7:$D$300,'Vidushi Malhotra'!$B$7:$B$300,$B42)</f>
@@ -11341,155 +11347,155 @@
       </c>
       <c r="C43" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH($B43,Prices!$A$6:$A$300,0)),"")</f>
-        <v>119.758503401361</v>
+        <v>473.4</v>
       </c>
       <c r="D43" s="46" t="str">
         <f aca="false">IFERROR(INDEX(Prices!$D$6:$D$300,MATCH($B43,Prices!$A$6:$A$300,0)),"")</f>
-        <v>DA stmt – 23.10</v>
+        <v>Close 28.10.2026 live (~11:35 IST) (Screener.in)</v>
       </c>
       <c r="E43" s="6" t="n">
         <f aca="false">(M43&gt;0)+(T43&gt;0)+(AA43&gt;0)+(AH43&gt;0)+(AO43&gt;0)+(AV43&gt;0)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43" s="47" t="n">
         <f aca="false">M43+T43+AA43+AH43+AO43+AV43</f>
-        <v>502</v>
+        <v>127</v>
       </c>
       <c r="G43" s="48" t="n">
         <f aca="false">IF(AND(F43&gt;0,H43&gt;0),H43/F43,"")</f>
-        <v>115.73374501992</v>
+        <v>606.212598425197</v>
       </c>
       <c r="H43" s="48" t="n">
         <f aca="false">O43+V43+AC43+AJ43+AQ43+AX43</f>
-        <v>58098.34</v>
+        <v>76989</v>
       </c>
       <c r="I43" s="49" t="n">
         <f aca="false">P43+W43+AD43+AK43+AR43+AY43</f>
-        <v>60118.768707483</v>
+        <v>60121.8</v>
       </c>
       <c r="J43" s="48" t="n">
         <f aca="false">I43-H43</f>
-        <v>2020.42870748297</v>
+        <v>-16867.2</v>
       </c>
       <c r="K43" s="50" t="n">
         <f aca="false">IF(H43&gt;0,J43/H43,"")</f>
-        <v>0.0347760143832504</v>
+        <v>-0.219085843432179</v>
       </c>
       <c r="L43" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I43/I$6)</f>
-        <v>0.00157587164028465</v>
+        <v>0.00157355904795841</v>
       </c>
       <c r="M43" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B43)</f>
-        <v>29</v>
-      </c>
-      <c r="N43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N43" s="8" t="str">
         <f aca="false">IF(AND(M43&gt;0,O43&gt;0),O43/M43,"")</f>
-        <v>134.94275862069</v>
+        <v/>
       </c>
       <c r="O43" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$E$7:$E$300,Gautam!$B$7:$B$300,$B43)</f>
-        <v>3913.34</v>
+        <v>0</v>
       </c>
       <c r="P43" s="8" t="n">
         <f aca="false">SUMIFS(Gautam!$H$7:$H$300,Gautam!$B$7:$B$300,$B43)</f>
-        <v>3472.99659863945</v>
+        <v>0</v>
       </c>
       <c r="Q43" s="8" t="n">
         <f aca="false">P43-O43</f>
-        <v>-440.343401360546</v>
-      </c>
-      <c r="R43" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" s="9" t="str">
         <f aca="false">IF(O43&gt;0,Q43/O43,"")</f>
-        <v>-0.11252367577582</v>
+        <v/>
       </c>
       <c r="S43" s="9" t="n">
         <f aca="false">IF(P$6=0,"",P43/P$6)</f>
-        <v>0.000623575931000622</v>
+        <v>0</v>
       </c>
       <c r="T43" s="52" t="n">
         <f aca="false">SUMIFS(DA!$D$7:$D$300,DA!$B$7:$B$300,$B43)</f>
-        <v>294</v>
+        <v>127</v>
       </c>
       <c r="U43" s="8" t="n">
         <f aca="false">IF(AND(T43&gt;0,V43&gt;0),V43/T43,"")</f>
-        <v>127.360544217687</v>
+        <v>606.212598425197</v>
       </c>
       <c r="V43" s="8" t="n">
         <f aca="false">SUMIFS(DA!$E$7:$E$300,DA!$B$7:$B$300,$B43)</f>
-        <v>37444</v>
+        <v>76989</v>
       </c>
       <c r="W43" s="8" t="n">
         <f aca="false">SUMIFS(DA!$H$7:$H$300,DA!$B$7:$B$300,$B43)</f>
-        <v>35209</v>
+        <v>60121.8</v>
       </c>
       <c r="X43" s="8" t="n">
         <f aca="false">W43-V43</f>
-        <v>-2235.00000000001</v>
+        <v>-16867.2</v>
       </c>
       <c r="Y43" s="9" t="n">
         <f aca="false">IF(V43&gt;0,X43/V43,"")</f>
-        <v>-0.0596891357760927</v>
+        <v>-0.219085843432179</v>
       </c>
       <c r="Z43" s="9" t="n">
         <f aca="false">IF(W$6=0,"",W43/W$6)</f>
-        <v>0.00886483375387686</v>
+        <v>0.0151373160834967</v>
       </c>
       <c r="AA43" s="52" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$D$7:$D$300,'Manish Shilpa'!$B$7:$B$300,$B43)</f>
-        <v>168</v>
-      </c>
-      <c r="AB43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB43" s="8" t="str">
         <f aca="false">IF(AND(AA43&gt;0,AC43&gt;0),AC43/AA43,"")</f>
-        <v>91.3928571428571</v>
+        <v/>
       </c>
       <c r="AC43" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$E$7:$E$300,'Manish Shilpa'!$B$7:$B$300,$B43)</f>
-        <v>15354</v>
+        <v>0</v>
       </c>
       <c r="AD43" s="8" t="n">
         <f aca="false">SUMIFS('Manish Shilpa'!$H$7:$H$300,'Manish Shilpa'!$B$7:$B$300,$B43)</f>
-        <v>20119.4285714286</v>
+        <v>0</v>
       </c>
       <c r="AE43" s="8" t="n">
         <f aca="false">AD43-AC43</f>
-        <v>4765.42857142857</v>
-      </c>
-      <c r="AF43" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF43" s="9" t="str">
         <f aca="false">IF(AC43&gt;0,AE43/AC43,"")</f>
-        <v>0.310370494426766</v>
+        <v/>
       </c>
       <c r="AG43" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD43/AD$6)</f>
-        <v>0.00173943021648071</v>
+        <v>0</v>
       </c>
       <c r="AH43" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B43)</f>
-        <v>11</v>
-      </c>
-      <c r="AI43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI43" s="8" t="str">
         <f aca="false">IF(AND(AH43&gt;0,AJ43&gt;0),AJ43/AH43,"")</f>
-        <v>126.090909090909</v>
+        <v/>
       </c>
       <c r="AJ43" s="8" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$E$7:$E$300,'Saloni Mehra'!$B$7:$B$300,$B43)</f>
-        <v>1387</v>
+        <v>0</v>
       </c>
       <c r="AK43" s="8" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$H$7:$H$300,'Saloni Mehra'!$B$7:$B$300,$B43)</f>
-        <v>1317.34353741497</v>
+        <v>0</v>
       </c>
       <c r="AL43" s="8" t="n">
         <f aca="false">AK43-AJ43</f>
-        <v>-69.6564625850344</v>
-      </c>
-      <c r="AM43" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM43" s="9" t="str">
         <f aca="false">IF(AJ43&gt;0,AL43/AJ43,"")</f>
-        <v>-0.0502209535580638</v>
+        <v/>
       </c>
       <c r="AN43" s="9" t="n">
         <f aca="false">IF(AK$6=0,"",AK43/AK$6)</f>
-        <v>0.000113903544031896</v>
+        <v>0</v>
       </c>
       <c r="AO43" s="52" t="n">
         <f aca="false">SUMIFS('Vidushi Malhotra'!$D$7:$D$300,'Vidushi Malhotra'!$B$7:$B$300,$B43)</f>
@@ -11593,7 +11599,7 @@
       </c>
       <c r="L44" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I44/I$6)</f>
-        <v>0.0013030041208605</v>
+        <v>0.00130102636173509</v>
       </c>
       <c r="M44" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B44)</f>
@@ -11677,7 +11683,7 @@
       </c>
       <c r="AG44" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD44/AD$6)</f>
-        <v>0.00429760399626003</v>
+        <v>0.00427616412015341</v>
       </c>
       <c r="AH44" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B44)</f>
@@ -11809,7 +11815,7 @@
       </c>
       <c r="L45" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I45/I$6)</f>
-        <v>0.0012446348626544</v>
+        <v>0.00124274569905313</v>
       </c>
       <c r="M45" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B45)</f>
@@ -12025,7 +12031,7 @@
       </c>
       <c r="L46" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I46/I$6)</f>
-        <v>0.00112494165746343</v>
+        <v>0.00112323416967195</v>
       </c>
       <c r="M46" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B46)</f>
@@ -12241,7 +12247,7 @@
       </c>
       <c r="L47" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I47/I$6)</f>
-        <v>0.00110230311094305</v>
+        <v>0.00110062998497074</v>
       </c>
       <c r="M47" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B47)</f>
@@ -12457,7 +12463,7 @@
       </c>
       <c r="L48" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I48/I$6)</f>
-        <v>0.00100296113730763</v>
+        <v>0.001001438797117</v>
       </c>
       <c r="M48" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B48)</f>
@@ -12673,7 +12679,7 @@
       </c>
       <c r="L49" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I49/I$6)</f>
-        <v>0.000943655039348572</v>
+        <v>0.000942222716660224</v>
       </c>
       <c r="M49" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B49)</f>
@@ -12889,7 +12895,7 @@
       </c>
       <c r="L50" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I50/I$6)</f>
-        <v>0.000897885148676168</v>
+        <v>0.00089652229761688</v>
       </c>
       <c r="M50" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B50)</f>
@@ -13105,7 +13111,7 @@
       </c>
       <c r="L51" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I51/I$6)</f>
-        <v>0.000857363028528142</v>
+        <v>0.000856061683792295</v>
       </c>
       <c r="M51" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B51)</f>
@@ -13321,7 +13327,7 @@
       </c>
       <c r="L52" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I52/I$6)</f>
-        <v>0.000807030565740487</v>
+        <v>0.000805805617913898</v>
       </c>
       <c r="M52" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B52)</f>
@@ -13537,7 +13543,7 @@
       </c>
       <c r="L53" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I53/I$6)</f>
-        <v>0.000781634711620419</v>
+        <v>0.000780448310780312</v>
       </c>
       <c r="M53" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B53)</f>
@@ -13621,7 +13627,7 @@
       </c>
       <c r="AG53" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD53/AD$6)</f>
-        <v>0.00257800908415936</v>
+        <v>0.00256514791886489</v>
       </c>
       <c r="AH53" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B53)</f>
@@ -13753,7 +13759,7 @@
       </c>
       <c r="L54" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I54/I$6)</f>
-        <v>0.000614185746152013</v>
+        <v>0.000613253506994279</v>
       </c>
       <c r="M54" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B54)</f>
@@ -13969,7 +13975,7 @@
       </c>
       <c r="L55" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I55/I$6)</f>
-        <v>0.000612979964712845</v>
+        <v>0.000612049555745213</v>
       </c>
       <c r="M55" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B55)</f>
@@ -14185,7 +14191,7 @@
       </c>
       <c r="L56" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I56/I$6)</f>
-        <v>0.000589645996853753</v>
+        <v>0.00058875100524753</v>
       </c>
       <c r="M56" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B56)</f>
@@ -14401,7 +14407,7 @@
       </c>
       <c r="L57" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I57/I$6)</f>
-        <v>0.00058390018616972</v>
+        <v>0.000583013915817199</v>
       </c>
       <c r="M57" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B57)</f>
@@ -14617,7 +14623,7 @@
       </c>
       <c r="L58" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I58/I$6)</f>
-        <v>0.000532520266288389</v>
+        <v>0.000531711982723309</v>
       </c>
       <c r="M58" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B58)</f>
@@ -14833,7 +14839,7 @@
       </c>
       <c r="L59" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I59/I$6)</f>
-        <v>0.000513474162077536</v>
+        <v>0.000512694787558717</v>
       </c>
       <c r="M59" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B59)</f>
@@ -14917,7 +14923,7 @@
       </c>
       <c r="AG59" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD59/AD$6)</f>
-        <v>0.00169355459095814</v>
+        <v>0.00168510579003523</v>
       </c>
       <c r="AH59" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B59)</f>
@@ -15049,7 +15055,7 @@
       </c>
       <c r="L60" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I60/I$6)</f>
-        <v>0.000510607809895515</v>
+        <v>0.000509832786056861</v>
       </c>
       <c r="M60" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B60)</f>
@@ -15265,7 +15271,7 @@
       </c>
       <c r="L61" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I61/I$6)</f>
-        <v>0.000501128008646059</v>
+        <v>0.000500367373682412</v>
       </c>
       <c r="M61" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B61)</f>
@@ -15481,7 +15487,7 @@
       </c>
       <c r="L62" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I62/I$6)</f>
-        <v>0.000469710586869347</v>
+        <v>0.000468997638702404</v>
       </c>
       <c r="M62" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B62)</f>
@@ -15697,7 +15703,7 @@
       </c>
       <c r="L63" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I63/I$6)</f>
-        <v>0.000451858730536071</v>
+        <v>0.000451172878731452</v>
       </c>
       <c r="M63" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B63)</f>
@@ -15913,7 +15919,7 @@
       </c>
       <c r="L64" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I64/I$6)</f>
-        <v>0.000449829872201472</v>
+        <v>0.000449147099890633</v>
       </c>
       <c r="M64" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B64)</f>
@@ -16129,7 +16135,7 @@
       </c>
       <c r="L65" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I65/I$6)</f>
-        <v>0.000432967805153912</v>
+        <v>0.000432310626858044</v>
       </c>
       <c r="M65" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B65)</f>
@@ -16213,7 +16219,7 @@
       </c>
       <c r="AG65" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD65/AD$6)</f>
-        <v>0.000105779726840292</v>
+        <v>0.000105252013202641</v>
       </c>
       <c r="AH65" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B65)</f>
@@ -16345,7 +16351,7 @@
       </c>
       <c r="L66" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I66/I$6)</f>
-        <v>0.000412849079715</v>
+        <v>0.000412222438538848</v>
       </c>
       <c r="M66" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B66)</f>
@@ -16561,7 +16567,7 @@
       </c>
       <c r="L67" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I67/I$6)</f>
-        <v>0.000410206845604824</v>
+        <v>0.0004095842149322</v>
       </c>
       <c r="M67" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B67)</f>
@@ -16777,7 +16783,7 @@
       </c>
       <c r="L68" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I68/I$6)</f>
-        <v>0.000409310373317443</v>
+        <v>0.000408689103351372</v>
       </c>
       <c r="M68" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B68)</f>
@@ -16993,7 +16999,7 @@
       </c>
       <c r="L69" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I69/I$6)</f>
-        <v>0.000393346875568463</v>
+        <v>0.00039274983572787</v>
       </c>
       <c r="M69" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B69)</f>
@@ -17209,7 +17215,7 @@
       </c>
       <c r="L70" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I70/I$6)</f>
-        <v>0.000379852608505779</v>
+        <v>0.000379276050879629</v>
       </c>
       <c r="M70" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B70)</f>
@@ -17425,7 +17431,7 @@
       </c>
       <c r="L71" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I71/I$6)</f>
-        <v>0.000351249375757524</v>
+        <v>0.000350716233423528</v>
       </c>
       <c r="M71" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B71)</f>
@@ -17509,7 +17515,7 @@
       </c>
       <c r="AG71" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD71/AD$6)</f>
-        <v>0.00115850034299391</v>
+        <v>0.00115272081936985</v>
       </c>
       <c r="AH71" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B71)</f>
@@ -17641,7 +17647,7 @@
       </c>
       <c r="L72" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I72/I$6)</f>
-        <v>0.000336196767247915</v>
+        <v>0.000335686472450135</v>
       </c>
       <c r="M72" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B72)</f>
@@ -17857,7 +17863,7 @@
       </c>
       <c r="L73" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I73/I$6)</f>
-        <v>0.000333446799187414</v>
+        <v>0.000332940678416668</v>
       </c>
       <c r="M73" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B73)</f>
@@ -18073,7 +18079,7 @@
       </c>
       <c r="L74" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I74/I$6)</f>
-        <v>0.000290232903039645</v>
+        <v>0.00028979237429281</v>
       </c>
       <c r="M74" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B74)</f>
@@ -18157,7 +18163,7 @@
       </c>
       <c r="AG74" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD74/AD$6)</f>
-        <v>0.000957254136023458</v>
+        <v>0.000952478588975208</v>
       </c>
       <c r="AH74" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B74)</f>
@@ -18289,7 +18295,7 @@
       </c>
       <c r="L75" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I75/I$6)</f>
-        <v>0.000290184409655679</v>
+        <v>0.000289743954514315</v>
       </c>
       <c r="M75" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B75)</f>
@@ -18373,7 +18379,7 @@
       </c>
       <c r="AG75" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD75/AD$6)</f>
-        <v>0.000957094193811925</v>
+        <v>0.000952319444682982</v>
       </c>
       <c r="AH75" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B75)</f>
@@ -18505,7 +18511,7 @@
       </c>
       <c r="L76" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I76/I$6)</f>
-        <v>0.000273022994259526</v>
+        <v>0.000272608587497719</v>
       </c>
       <c r="M76" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B76)</f>
@@ -18721,7 +18727,7 @@
       </c>
       <c r="L77" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I77/I$6)</f>
-        <v>0.000270333577397382</v>
+        <v>0.000269923252755238</v>
       </c>
       <c r="M77" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B77)</f>
@@ -18805,7 +18811,7 @@
       </c>
       <c r="AG77" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD77/AD$6)</f>
-        <v>0.000891621633382874</v>
+        <v>0.000887173513600237</v>
       </c>
       <c r="AH77" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B77)</f>
@@ -18937,7 +18943,7 @@
       </c>
       <c r="L78" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I78/I$6)</f>
-        <v>0.000255153837583861</v>
+        <v>0.000254766553443628</v>
       </c>
       <c r="M78" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B78)</f>
@@ -19153,7 +19159,7 @@
       </c>
       <c r="L79" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I79/I$6)</f>
-        <v>0.000174143673719784</v>
+        <v>0.000173879350503672</v>
       </c>
       <c r="M79" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B79)</f>
@@ -19237,7 +19243,7 @@
       </c>
       <c r="AG79" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD79/AD$6)</f>
-        <v>0.000287182724950748</v>
+        <v>0.000285750028488193</v>
       </c>
       <c r="AH79" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B79)</f>
@@ -19369,7 +19375,7 @@
       </c>
       <c r="L80" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I80/I$6)</f>
-        <v>0.000173653497352123</v>
+        <v>0.000173389918148074</v>
       </c>
       <c r="M80" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B80)</f>
@@ -19585,7 +19591,7 @@
       </c>
       <c r="L81" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I81/I$6)</f>
-        <v>0.000145716065659409</v>
+        <v>0.000145494891164283</v>
       </c>
       <c r="M81" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B81)</f>
@@ -19669,7 +19675,7 @@
       </c>
       <c r="AG81" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD81/AD$6)</f>
-        <v>0.000480604731843519</v>
+        <v>0.000478207092154999</v>
       </c>
       <c r="AH81" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B81)</f>
@@ -19801,7 +19807,7 @@
       </c>
       <c r="L82" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I82/I$6)</f>
-        <v>0.000130106438550184</v>
+        <v>0.000129908957059528</v>
       </c>
       <c r="M82" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B82)</f>
@@ -19885,7 +19891,7 @@
       </c>
       <c r="AG82" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD82/AD$6)</f>
-        <v>0.000429120630779872</v>
+        <v>0.000426979834846436</v>
       </c>
       <c r="AH82" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B82)</f>
@@ -20017,7 +20023,7 @@
       </c>
       <c r="L83" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I83/I$6)</f>
-        <v>0.000122183668115654</v>
+        <v>0.000121998212167569</v>
       </c>
       <c r="M83" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B83)</f>
@@ -20233,7 +20239,7 @@
       </c>
       <c r="L84" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I84/I$6)</f>
-        <v>0.000113238604721829</v>
+        <v>0.000113066725999227</v>
       </c>
       <c r="M84" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B84)</f>
@@ -20449,7 +20455,7 @@
       </c>
       <c r="L85" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I85/I$6)</f>
-        <v>9.8146677252247E-005</v>
+        <v>9.79977057459735E-005</v>
       </c>
       <c r="M85" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B85)</f>
@@ -20533,7 +20539,7 @@
       </c>
       <c r="AG85" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD85/AD$6)</f>
-        <v>0.000323710067854847</v>
+        <v>0.000322095143875041</v>
       </c>
       <c r="AH85" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B85)</f>
@@ -20665,7 +20671,7 @@
       </c>
       <c r="L86" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I86/I$6)</f>
-        <v>9.76473264605917E-005</v>
+        <v>9.74991128917408E-005</v>
       </c>
       <c r="M86" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B86)</f>
@@ -20749,7 +20755,7 @@
       </c>
       <c r="AG86" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD86/AD$6)</f>
-        <v>0.000322063095352307</v>
+        <v>0.000320456387784818</v>
       </c>
       <c r="AH86" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B86)</f>
@@ -20881,7 +20887,7 @@
       </c>
       <c r="L87" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I87/I$6)</f>
-        <v>7.09314037910343E-005</v>
+        <v>7.08237408689602E-005</v>
       </c>
       <c r="M87" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B87)</f>
@@ -20965,7 +20971,7 @@
       </c>
       <c r="AG87" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD87/AD$6)</f>
-        <v>0.000233947905085188</v>
+        <v>0.000232780786359314</v>
       </c>
       <c r="AH87" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B87)</f>
@@ -21097,7 +21103,7 @@
       </c>
       <c r="L88" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I88/I$6)</f>
-        <v>5.93192042790505E-005</v>
+        <v>5.92291668833913E-005</v>
       </c>
       <c r="M88" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B88)</f>
@@ -21313,7 +21319,7 @@
       </c>
       <c r="L89" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I89/I$6)</f>
-        <v>3.84958830774254E-005</v>
+        <v>3.8437452269089E-005</v>
       </c>
       <c r="M89" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B89)</f>
@@ -21397,7 +21403,7 @@
       </c>
       <c r="AG89" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD89/AD$6)</f>
-        <v>0.000126968179382154</v>
+        <v>0.000126334760845265</v>
       </c>
       <c r="AH89" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B89)</f>
@@ -21529,7 +21535,7 @@
       </c>
       <c r="L90" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I90/I$6)</f>
-        <v>3.23726103776524E-005</v>
+        <v>3.23234737520938E-005</v>
       </c>
       <c r="M90" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B90)</f>
@@ -21745,7 +21751,7 @@
       </c>
       <c r="L91" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I91/I$6)</f>
-        <v>2.44708100551072E-005</v>
+        <v>2.44336671427265E-005</v>
       </c>
       <c r="M91" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B91)</f>
@@ -21829,7 +21835,7 @@
       </c>
       <c r="AG91" s="9" t="n">
         <f aca="false">IF(AD$6=0,"",AD91/AD$6)</f>
-        <v>8.07102981494005E-005</v>
+        <v>8.03076508151284E-005</v>
       </c>
       <c r="AH91" s="52" t="n">
         <f aca="false">SUMIFS('Saloni Mehra'!$D$7:$D$300,'Saloni Mehra'!$B$7:$B$300,$B91)</f>
@@ -21961,7 +21967,7 @@
       </c>
       <c r="L92" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I92/I$6)</f>
-        <v>1.41217976638514E-005</v>
+        <v>1.41003629548203E-005</v>
       </c>
       <c r="M92" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B92)</f>
@@ -22177,7 +22183,7 @@
       </c>
       <c r="L93" s="51" t="n">
         <f aca="false">IF(I$6=0,"",I93/I$6)</f>
-        <v>1.08598967445032E-005</v>
+        <v>1.08434130975647E-005</v>
       </c>
       <c r="M93" s="52" t="n">
         <f aca="false">SUMIFS(Gautam!$D$7:$D$300,Gautam!$B$7:$B$300,$B93)</f>
@@ -23257,9 +23263,7 @@
       <c r="F16" s="57" t="n">
         <v>928.949945593036</v>
       </c>
-      <c r="G16" s="57" t="n">
-        <v>930.911424903723</v>
-      </c>
+      <c r="G16" s="57"/>
       <c r="H16" s="57"/>
       <c r="I16" s="57" t="n">
         <v>973.900826446281</v>
@@ -23297,9 +23301,7 @@
       <c r="F17" s="57" t="n">
         <v>77.4497607655502</v>
       </c>
-      <c r="G17" s="57" t="n">
-        <v>77.6406166932483</v>
-      </c>
+      <c r="G17" s="57"/>
       <c r="H17" s="57"/>
       <c r="I17" s="57" t="n">
         <v>81.801652892562</v>
@@ -24069,9 +24071,7 @@
       <c r="F39" s="57" t="n">
         <v>692.799472295515</v>
       </c>
-      <c r="G39" s="57" t="n">
-        <v>688.986179664363</v>
-      </c>
+      <c r="G39" s="57"/>
       <c r="H39" s="57"/>
       <c r="I39" s="57" t="n">
         <v>707.761904761905</v>
@@ -24092,7 +24092,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B40" s="54"/>
       <c r="C40" s="55" t="n">
@@ -24107,9 +24107,7 @@
       <c r="F40" s="57" t="n">
         <v>119.758503401361</v>
       </c>
-      <c r="G40" s="57" t="n">
-        <v>119.827380952381</v>
-      </c>
+      <c r="G40" s="57"/>
       <c r="H40" s="57" t="n">
         <v>123.909090909091</v>
       </c>
@@ -25105,9 +25103,7 @@
       <c r="F69" s="57" t="n">
         <v>413</v>
       </c>
-      <c r="G69" s="57" t="n">
-        <v>414.675753228121</v>
-      </c>
+      <c r="G69" s="57"/>
       <c r="H69" s="57"/>
       <c r="I69" s="57" t="n">
         <v>450.605263157895</v>
@@ -25752,7 +25748,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B88" s="54" t="n">
         <v>473.4</v>
@@ -26167,7 +26163,7 @@
         <v>201</v>
       </c>
       <c r="S7" s="62" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="T7" s="62" t="n">
         <v>2</v>
@@ -27625,7 +27621,7 @@
         <v>28</v>
       </c>
       <c r="B34" s="59" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>16</v>
@@ -28786,7 +28782,7 @@
         <v>201</v>
       </c>
       <c r="S20" s="62" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="T20" s="62" t="n">
         <v>195</v>
@@ -29043,7 +29039,7 @@
         <v>19</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>16</v>
@@ -29523,7 +29519,7 @@
         <v>27</v>
       </c>
       <c r="B33" s="59" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>16</v>
@@ -29686,7 +29682,7 @@
         <v>201</v>
       </c>
       <c r="S35" s="62" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="T35" s="62" t="n">
         <v>61</v>
@@ -30810,7 +30806,7 @@
     <tabColor rgb="FF27AE60"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:V61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -30825,6 +30821,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30842,6 +30844,11 @@
         <v>187</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q5" s="30" t="s">
+        <v>230</v>
+      </c>
+    </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
         <v>69</v>
@@ -30879,6 +30886,24 @@
       <c r="L6" s="23" t="s">
         <v>193</v>
       </c>
+      <c r="Q6" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="R6" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="S6" s="23" t="s">
+        <v>196</v>
+      </c>
+      <c r="T6" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="U6" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="V6" s="23" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="n">
@@ -30888,17 +30913,17 @@
         <v>79</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D7" s="60" t="n">
-        <v>3895</v>
+        <v>3935</v>
       </c>
       <c r="E7" s="57" t="n">
-        <v>2912389</v>
+        <v>2948869</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">IF(AND(D7&gt;0,N(E7)&gt;0),E7/D7,"")</f>
-        <v>747.725032092426</v>
+        <v>749.394917407878</v>
       </c>
       <c r="G7" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH(B7,Prices!$A$6:$A$300,0)),"")</f>
@@ -30906,22 +30931,40 @@
       </c>
       <c r="H7" s="8" t="n">
         <f aca="false">IF(ISNUMBER(G7),D7*G7,0)</f>
-        <v>3535102</v>
+        <v>3571406</v>
       </c>
       <c r="I7" s="8" t="n">
         <f aca="false">H7-N(E7)</f>
-        <v>622713</v>
+        <v>622537</v>
       </c>
       <c r="J7" s="9" t="n">
         <f aca="false">IF(N(E7)&gt;0,I7/E7,"")</f>
-        <v>0.213815187462939</v>
+        <v>0.211110429117062</v>
       </c>
       <c r="K7" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H7/$H$54)</f>
-        <v>0.305628125337199</v>
+        <v>0.307226421688238</v>
       </c>
       <c r="L7" s="61" t="s">
-        <v>231</v>
+        <v>232</v>
+      </c>
+      <c r="Q7" s="62" t="s">
+        <v>233</v>
+      </c>
+      <c r="R7" s="62" t="s">
+        <v>201</v>
+      </c>
+      <c r="S7" s="62" t="s">
+        <v>114</v>
+      </c>
+      <c r="T7" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="U7" s="57" t="n">
+        <v>119.53</v>
+      </c>
+      <c r="V7" s="57" t="n">
+        <v>119.53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30932,7 +30975,7 @@
         <v>81</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D8" s="60" t="n">
         <v>11160</v>
@@ -30962,10 +31005,28 @@
       </c>
       <c r="K8" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H8/$H$54)</f>
-        <v>0.247667747990467</v>
+        <v>0.246432183746497</v>
       </c>
       <c r="L8" s="61" t="s">
-        <v>232</v>
+        <v>234</v>
+      </c>
+      <c r="Q8" s="62" t="s">
+        <v>233</v>
+      </c>
+      <c r="R8" s="62" t="s">
+        <v>201</v>
+      </c>
+      <c r="S8" s="62" t="s">
+        <v>82</v>
+      </c>
+      <c r="T8" s="62" t="n">
+        <v>14</v>
+      </c>
+      <c r="U8" s="57" t="n">
+        <v>680.2</v>
+      </c>
+      <c r="V8" s="57" t="n">
+        <v>9522.8</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30976,7 +31037,7 @@
         <v>80</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D9" s="60" t="n">
         <v>165</v>
@@ -31006,10 +31067,28 @@
       </c>
       <c r="K9" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H9/$H$54)</f>
-        <v>0.0613913539222327</v>
+        <v>0.061085084888777</v>
       </c>
       <c r="L9" s="61" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q9" s="62" t="s">
         <v>233</v>
+      </c>
+      <c r="R9" s="62" t="s">
+        <v>201</v>
+      </c>
+      <c r="S9" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="T9" s="62" t="n">
+        <v>21</v>
+      </c>
+      <c r="U9" s="57" t="n">
+        <v>402.8</v>
+      </c>
+      <c r="V9" s="57" t="n">
+        <v>8458.8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31020,17 +31099,17 @@
         <v>82</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D10" s="60" t="n">
-        <v>1013</v>
+        <v>1027</v>
       </c>
       <c r="E10" s="57" t="n">
-        <v>812683</v>
+        <v>822205.8</v>
       </c>
       <c r="F10" s="8" t="n">
         <f aca="false">IF(AND(D10&gt;0,N(E10)&gt;0),E10/D10,"")</f>
-        <v>802.253701875617</v>
+        <v>800.589873417722</v>
       </c>
       <c r="G10" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH(B10,Prices!$A$6:$A$300,0)),"")</f>
@@ -31038,22 +31117,40 @@
       </c>
       <c r="H10" s="8" t="n">
         <f aca="false">IF(ISNUMBER(G10),D10*G10,0)</f>
-        <v>683926.95</v>
+        <v>693379.05</v>
       </c>
       <c r="I10" s="8" t="n">
         <f aca="false">H10-N(E10)</f>
-        <v>-128756.05</v>
+        <v>-128826.75</v>
       </c>
       <c r="J10" s="9" t="n">
         <f aca="false">IF(N(E10)&gt;0,I10/E10,"")</f>
-        <v>-0.158433300561228</v>
+        <v>-0.156684311883959</v>
       </c>
       <c r="K10" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H10/$H$54)</f>
-        <v>0.0591290750864015</v>
+        <v>0.0596471990037228</v>
       </c>
       <c r="L10" s="61" t="s">
-        <v>234</v>
+        <v>236</v>
+      </c>
+      <c r="Q10" s="62" t="s">
+        <v>233</v>
+      </c>
+      <c r="R10" s="62" t="s">
+        <v>201</v>
+      </c>
+      <c r="S10" s="62" t="s">
+        <v>86</v>
+      </c>
+      <c r="T10" s="62" t="n">
+        <v>48</v>
+      </c>
+      <c r="U10" s="57" t="n">
+        <v>77.64</v>
+      </c>
+      <c r="V10" s="57" t="n">
+        <v>3726.72</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31064,17 +31161,17 @@
         <v>83</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D11" s="60" t="n">
-        <v>1394</v>
+        <v>1415</v>
       </c>
       <c r="E11" s="57" t="n">
-        <v>622513</v>
+        <v>630971.8</v>
       </c>
       <c r="F11" s="8" t="n">
         <f aca="false">IF(AND(D11&gt;0,N(E11)&gt;0),E11/D11,"")</f>
-        <v>446.56599713056</v>
+        <v>445.916466431095</v>
       </c>
       <c r="G11" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH(B11,Prices!$A$6:$A$300,0)),"")</f>
@@ -31082,22 +31179,40 @@
       </c>
       <c r="H11" s="8" t="n">
         <f aca="false">IF(ISNUMBER(G11),D11*G11,0)</f>
-        <v>558087.9</v>
+        <v>566495.25</v>
       </c>
       <c r="I11" s="8" t="n">
         <f aca="false">H11-N(E11)</f>
-        <v>-64425.1</v>
+        <v>-64476.5500000001</v>
       </c>
       <c r="J11" s="9" t="n">
         <f aca="false">IF(N(E11)&gt;0,I11/E11,"")</f>
-        <v>-0.103491975267986</v>
+        <v>-0.102186104038247</v>
       </c>
       <c r="K11" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H11/$H$54)</f>
-        <v>0.048249628624683</v>
+        <v>0.0487321543842632</v>
       </c>
       <c r="L11" s="61" t="s">
-        <v>235</v>
+        <v>237</v>
+      </c>
+      <c r="Q11" s="62" t="s">
+        <v>233</v>
+      </c>
+      <c r="R11" s="62" t="s">
+        <v>201</v>
+      </c>
+      <c r="S11" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="T11" s="62" t="n">
+        <v>40</v>
+      </c>
+      <c r="U11" s="57" t="n">
+        <v>912</v>
+      </c>
+      <c r="V11" s="57" t="n">
+        <v>36480</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31108,7 +31223,7 @@
         <v>84</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D12" s="60" t="n">
         <v>360</v>
@@ -31138,9 +31253,16 @@
       </c>
       <c r="K12" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H12/$H$54)</f>
-        <v>0.040955926603317</v>
+        <v>0.0407516057787434</v>
       </c>
       <c r="L12" s="61"/>
+      <c r="S12" s="63" t="s">
+        <v>206</v>
+      </c>
+      <c r="V12" s="64" t="n">
+        <f aca="false">SUMIFS(V7:V11,R7:R11,"BUY")-SUMIFS(V7:V11,R7:R11,"SELL")</f>
+        <v>58307.85</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
@@ -31150,7 +31272,7 @@
         <v>96</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D13" s="60" t="n">
         <v>2004.589</v>
@@ -31180,10 +31302,10 @@
       </c>
       <c r="K13" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H13/$H$54)</f>
-        <v>0.0272662721420509</v>
+        <v>0.0271302462315381</v>
       </c>
       <c r="L13" s="61" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31194,17 +31316,17 @@
         <v>86</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D14" s="60" t="n">
-        <v>3762</v>
+        <v>3810</v>
       </c>
       <c r="E14" s="57" t="n">
-        <v>432693</v>
+        <v>436419.72</v>
       </c>
       <c r="F14" s="8" t="n">
         <f aca="false">IF(AND(D14&gt;0,N(E14)&gt;0),E14/D14,"")</f>
-        <v>115.016746411483</v>
+        <v>114.545858267717</v>
       </c>
       <c r="G14" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH(B14,Prices!$A$6:$A$300,0)),"")</f>
@@ -31212,22 +31334,22 @@
       </c>
       <c r="H14" s="8" t="n">
         <f aca="false">IF(ISNUMBER(G14),D14*G14,0)</f>
-        <v>290764.98</v>
+        <v>294474.9</v>
       </c>
       <c r="I14" s="8" t="n">
         <f aca="false">H14-N(E14)</f>
-        <v>-141928.02</v>
+        <v>-141944.82</v>
       </c>
       <c r="J14" s="9" t="n">
         <f aca="false">IF(N(E14)&gt;0,I14/E14,"")</f>
-        <v>-0.328010899182561</v>
+        <v>-0.325248409948111</v>
       </c>
       <c r="K14" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H14/$H$54)</f>
-        <v>0.0251381588851207</v>
+        <v>0.0253318916426757</v>
       </c>
       <c r="L14" s="61" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31238,7 +31360,7 @@
         <v>88</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D15" s="60" t="n">
         <v>72</v>
@@ -31268,10 +31390,10 @@
       </c>
       <c r="K15" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H15/$H$54)</f>
-        <v>0.0251350309341946</v>
+        <v>0.0250096373545084</v>
       </c>
       <c r="L15" s="61" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31282,7 +31404,7 @@
         <v>87</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D16" s="60" t="n">
         <v>66</v>
@@ -31312,10 +31434,10 @@
       </c>
       <c r="K16" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H16/$H$54)</f>
-        <v>0.0229480070702708</v>
+        <v>0.0228335241097867</v>
       </c>
       <c r="L16" s="61" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31326,7 +31448,7 @@
         <v>89</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D17" s="60" t="n">
         <v>800</v>
@@ -31356,7 +31478,7 @@
       </c>
       <c r="K17" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H17/$H$54)</f>
-        <v>0.0163780824609527</v>
+        <v>0.0162963755239869</v>
       </c>
       <c r="L17" s="61"/>
     </row>
@@ -31368,7 +31490,7 @@
         <v>92</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D18" s="60" t="n">
         <v>3500</v>
@@ -31398,7 +31520,7 @@
       </c>
       <c r="K18" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H18/$H$54)</f>
-        <v>0.0151326945922343</v>
+        <v>0.0150572006431643</v>
       </c>
       <c r="L18" s="61"/>
     </row>
@@ -31410,7 +31532,7 @@
         <v>102</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D19" s="60" t="n">
         <v>134</v>
@@ -31440,7 +31562,7 @@
       </c>
       <c r="K19" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H19/$H$54)</f>
-        <v>0.0141348626848687</v>
+        <v>0.0140643467171315</v>
       </c>
       <c r="L19" s="61"/>
     </row>
@@ -31452,7 +31574,7 @@
         <v>91</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D20" s="60" t="n">
         <v>32</v>
@@ -31482,10 +31604,10 @@
       </c>
       <c r="K20" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H20/$H$54)</f>
-        <v>0.0102404513900704</v>
+        <v>0.0101893638516955</v>
       </c>
       <c r="L20" s="61" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31496,7 +31618,7 @@
         <v>108</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D21" s="60" t="n">
         <v>44</v>
@@ -31526,7 +31648,7 @@
       </c>
       <c r="K21" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H21/$H$54)</f>
-        <v>0.00735090945994501</v>
+        <v>0.00731423726115022</v>
       </c>
       <c r="L21" s="61"/>
     </row>
@@ -31538,7 +31660,7 @@
         <v>110</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D22" s="60" t="n">
         <v>3</v>
@@ -31568,7 +31690,7 @@
       </c>
       <c r="K22" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H22/$H$54)</f>
-        <v>0.00674999360292908</v>
+        <v>0.00671631925166424</v>
       </c>
       <c r="L22" s="61"/>
     </row>
@@ -31580,7 +31702,7 @@
         <v>111</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D23" s="60" t="n">
         <v>64</v>
@@ -31610,7 +31732,7 @@
       </c>
       <c r="K23" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H23/$H$54)</f>
-        <v>0.00613348121890747</v>
+        <v>0.00610288252308764</v>
       </c>
       <c r="L23" s="61"/>
     </row>
@@ -31622,7 +31744,7 @@
         <v>112</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D24" s="60" t="n">
         <v>160</v>
@@ -31652,10 +31774,10 @@
       </c>
       <c r="K24" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H24/$H$54)</f>
-        <v>0.00608714120518771</v>
+        <v>0.00605677369031285</v>
       </c>
       <c r="L24" s="61" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31666,7 +31788,7 @@
         <v>85</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D25" s="60" t="n">
         <v>29</v>
@@ -31696,7 +31818,7 @@
       </c>
       <c r="K25" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H25/$H$54)</f>
-        <v>0.00607043805098872</v>
+        <v>0.00604015386476791</v>
       </c>
       <c r="L25" s="61"/>
     </row>
@@ -31708,7 +31830,7 @@
         <v>113</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D26" s="60" t="n">
         <v>2</v>
@@ -31738,7 +31860,7 @@
       </c>
       <c r="K26" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H26/$H$54)</f>
-        <v>0.00582103194729702</v>
+        <v>0.00579199199762476</v>
       </c>
       <c r="L26" s="61"/>
     </row>
@@ -31750,7 +31872,7 @@
         <v>94</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D27" s="60" t="n">
         <v>47</v>
@@ -31780,10 +31902,10 @@
       </c>
       <c r="K27" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H27/$H$54)</f>
-        <v>0.00557619932630266</v>
+        <v>0.00554838079699988</v>
       </c>
       <c r="L27" s="61" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31794,7 +31916,7 @@
         <v>93</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D28" s="60" t="n">
         <v>11</v>
@@ -31824,10 +31946,10 @@
       </c>
       <c r="K28" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H28/$H$54)</f>
-        <v>0.00547590259138421</v>
+        <v>0.00544858442218264</v>
       </c>
       <c r="L28" s="61" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31838,7 +31960,7 @@
         <v>116</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D29" s="60" t="n">
         <v>22</v>
@@ -31868,7 +31990,7 @@
       </c>
       <c r="K29" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H29/$H$54)</f>
-        <v>0.00429760399626003</v>
+        <v>0.00427616412015341</v>
       </c>
       <c r="L29" s="61"/>
     </row>
@@ -31880,7 +32002,7 @@
         <v>95</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D30" s="60" t="n">
         <v>6</v>
@@ -31910,10 +32032,10 @@
       </c>
       <c r="K30" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H30/$H$54)</f>
-        <v>0.00370918956831849</v>
+        <v>0.00369068517264362</v>
       </c>
       <c r="L30" s="61" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -31924,7 +32046,7 @@
         <v>99</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D31" s="60" t="n">
         <v>32</v>
@@ -31954,7 +32076,7 @@
       </c>
       <c r="K31" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H31/$H$54)</f>
-        <v>0.00325542054591268</v>
+        <v>0.00323917991200597</v>
       </c>
       <c r="L31" s="61"/>
     </row>
@@ -31966,7 +32088,7 @@
         <v>125</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D32" s="60" t="n">
         <v>34</v>
@@ -31996,7 +32118,7 @@
       </c>
       <c r="K32" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H32/$H$54)</f>
-        <v>0.00257800908415936</v>
+        <v>0.00256514791886489</v>
       </c>
       <c r="L32" s="61"/>
     </row>
@@ -32008,7 +32130,7 @@
         <v>98</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D33" s="60" t="n">
         <v>10</v>
@@ -32038,10 +32160,10 @@
       </c>
       <c r="K33" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H33/$H$54)</f>
-        <v>0.00245723110063977</v>
+        <v>0.00244497247224849</v>
       </c>
       <c r="L33" s="61" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32049,20 +32171,20 @@
         <v>28</v>
       </c>
       <c r="B34" s="59" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D34" s="60" t="n">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E34" s="57" t="n">
-        <v>15354</v>
+        <v>15473.53</v>
       </c>
       <c r="F34" s="8" t="n">
         <f aca="false">IF(AND(D34&gt;0,N(E34)&gt;0),E34/D34,"")</f>
-        <v>91.3928571428571</v>
+        <v>91.559349112426</v>
       </c>
       <c r="G34" s="7" t="n">
         <f aca="false">IFERROR(INDEX(Prices!$C$6:$C$300,MATCH(B34,Prices!$A$6:$A$300,0)),"")</f>
@@ -32070,22 +32192,22 @@
       </c>
       <c r="H34" s="8" t="n">
         <f aca="false">IF(ISNUMBER(G34),D34*G34,0)</f>
-        <v>20119.4285714286</v>
+        <v>20239.1870748299</v>
       </c>
       <c r="I34" s="8" t="n">
         <f aca="false">H34-N(E34)</f>
-        <v>4765.42857142857</v>
+        <v>4765.65707482993</v>
       </c>
       <c r="J34" s="9" t="n">
         <f aca="false">IF(N(E34)&gt;0,I34/E34,"")</f>
-        <v>0.310370494426766</v>
+        <v>0.3079877102917</v>
       </c>
       <c r="K34" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H34/$H$54)</f>
-        <v>0.00173943021648071</v>
+        <v>0.00174105464987146</v>
       </c>
       <c r="L34" s="61" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32096,7 +32218,7 @@
         <v>131</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D35" s="60" t="n">
         <v>33</v>
@@ -32126,7 +32248,7 @@
       </c>
       <c r="K35" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H35/$H$54)</f>
-        <v>0.00169355459095814</v>
+        <v>0.00168510579003523</v>
       </c>
       <c r="L35" s="61"/>
     </row>
@@ -32138,7 +32260,7 @@
         <v>101</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D36" s="60" t="n">
         <v>6</v>
@@ -32168,10 +32290,10 @@
       </c>
       <c r="K36" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H36/$H$54)</f>
-        <v>0.00162669010101251</v>
+        <v>0.0016185748734904</v>
       </c>
       <c r="L36" s="61" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32182,7 +32304,7 @@
         <v>100</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D37" s="60" t="n">
         <v>17</v>
@@ -32212,10 +32334,10 @@
       </c>
       <c r="K37" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H37/$H$54)</f>
-        <v>0.00158276218875317</v>
+        <v>0.00157486610869027</v>
       </c>
       <c r="L37" s="61" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32226,7 +32348,7 @@
         <v>143</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D38" s="60" t="n">
         <v>50</v>
@@ -32256,7 +32378,7 @@
       </c>
       <c r="K38" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H38/$H$54)</f>
-        <v>0.00115850034299391</v>
+        <v>0.00115272081936985</v>
       </c>
       <c r="L38" s="61"/>
     </row>
@@ -32268,7 +32390,7 @@
         <v>104</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D39" s="60" t="n">
         <v>6</v>
@@ -32298,10 +32420,10 @@
       </c>
       <c r="K39" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H39/$H$54)</f>
-        <v>0.00113239085765181</v>
+        <v>0.00112674158896315</v>
       </c>
       <c r="L39" s="61" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32312,7 +32434,7 @@
         <v>146</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D40" s="60" t="n">
         <v>35</v>
@@ -32342,7 +32464,7 @@
       </c>
       <c r="K40" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H40/$H$54)</f>
-        <v>0.000957254136023458</v>
+        <v>0.000952478588975208</v>
       </c>
       <c r="L40" s="61"/>
     </row>
@@ -32354,7 +32476,7 @@
         <v>147</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D41" s="60" t="n">
         <v>34</v>
@@ -32384,10 +32506,10 @@
       </c>
       <c r="K41" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H41/$H$54)</f>
-        <v>0.000957094193811925</v>
+        <v>0.000952319444682982</v>
       </c>
       <c r="L41" s="61" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32398,7 +32520,7 @@
         <v>149</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D42" s="60" t="n">
         <v>14</v>
@@ -32428,7 +32550,7 @@
       </c>
       <c r="K42" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H42/$H$54)</f>
-        <v>0.000891621633382874</v>
+        <v>0.000887173513600237</v>
       </c>
       <c r="L42" s="61"/>
     </row>
@@ -32440,7 +32562,7 @@
         <v>107</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D43" s="60" t="n">
         <v>32</v>
@@ -32470,7 +32592,7 @@
       </c>
       <c r="K43" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H43/$H$54)</f>
-        <v>0.000568142401044131</v>
+        <v>0.000565308053649652</v>
       </c>
       <c r="L43" s="61"/>
     </row>
@@ -32482,7 +32604,7 @@
         <v>153</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D44" s="60" t="n">
         <v>4</v>
@@ -32512,10 +32634,10 @@
       </c>
       <c r="K44" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H44/$H$54)</f>
-        <v>0.000480604731843519</v>
+        <v>0.000478207092154999</v>
       </c>
       <c r="L44" s="61" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32526,7 +32648,7 @@
         <v>154</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D45" s="60" t="n">
         <v>3</v>
@@ -32556,7 +32678,7 @@
       </c>
       <c r="K45" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H45/$H$54)</f>
-        <v>0.000429120630779872</v>
+        <v>0.000426979834846436</v>
       </c>
       <c r="L45" s="61"/>
     </row>
@@ -32568,7 +32690,7 @@
         <v>103</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D46" s="60" t="n">
         <v>5</v>
@@ -32598,7 +32720,7 @@
       </c>
       <c r="K46" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H46/$H$54)</f>
-        <v>0.000344502555354104</v>
+        <v>0.000342783901864477</v>
       </c>
       <c r="L46" s="61"/>
     </row>
@@ -32610,7 +32732,7 @@
         <v>157</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D47" s="60" t="n">
         <v>5</v>
@@ -32640,7 +32762,7 @@
       </c>
       <c r="K47" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H47/$H$54)</f>
-        <v>0.000323710067854847</v>
+        <v>0.000322095143875041</v>
       </c>
       <c r="L47" s="61"/>
     </row>
@@ -32652,7 +32774,7 @@
         <v>158</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D48" s="60" t="n">
         <v>1</v>
@@ -32682,7 +32804,7 @@
       </c>
       <c r="K48" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H48/$H$54)</f>
-        <v>0.000322063095352307</v>
+        <v>0.000320456387784818</v>
       </c>
       <c r="L48" s="61"/>
     </row>
@@ -32694,7 +32816,7 @@
         <v>151</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D49" s="60" t="n">
         <v>5</v>
@@ -32724,10 +32846,10 @@
       </c>
       <c r="K49" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H49/$H$54)</f>
-        <v>0.000287182724950748</v>
+        <v>0.000285750028488193</v>
       </c>
       <c r="L49" s="61" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32738,7 +32860,7 @@
         <v>159</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D50" s="60" t="n">
         <v>6</v>
@@ -32768,7 +32890,7 @@
       </c>
       <c r="K50" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H50/$H$54)</f>
-        <v>0.000233947905085188</v>
+        <v>0.000232780786359314</v>
       </c>
       <c r="L50" s="61"/>
     </row>
@@ -32780,7 +32902,7 @@
         <v>161</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D51" s="60" t="n">
         <v>1</v>
@@ -32810,7 +32932,7 @@
       </c>
       <c r="K51" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H51/$H$54)</f>
-        <v>0.000126968179382154</v>
+        <v>0.000126334760845265</v>
       </c>
       <c r="L51" s="61"/>
     </row>
@@ -32822,7 +32944,7 @@
         <v>137</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D52" s="60" t="n">
         <v>12</v>
@@ -32852,7 +32974,7 @@
       </c>
       <c r="K52" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H52/$H$54)</f>
-        <v>0.000105779726840292</v>
+        <v>0.000105252013202641</v>
       </c>
       <c r="L52" s="61"/>
     </row>
@@ -32864,7 +32986,7 @@
         <v>163</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D53" s="60" t="n">
         <v>5</v>
@@ -32894,7 +33016,7 @@
       </c>
       <c r="K53" s="9" t="n">
         <f aca="false">IF($H$54=0,"",H53/$H$54)</f>
-        <v>8.07102981494005E-005</v>
+        <v>8.03076508151284E-005</v>
       </c>
       <c r="L53" s="61"/>
     </row>
@@ -32910,7 +33032,7 @@
       <c r="G54" s="89"/>
       <c r="H54" s="90" t="n">
         <f aca="false">SUM(H7:H53)</f>
-        <v>11566677.6285714</v>
+        <v>11624670.7570748</v>
       </c>
       <c r="I54" s="90"/>
       <c r="J54" s="91"/>
@@ -32927,7 +33049,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B57" s="75" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E57" s="76" t="n">
         <v>11949395</v>
@@ -32959,7 +33081,7 @@
       </c>
       <c r="E60" s="80" t="n">
         <f aca="false">H54</f>
-        <v>11566677.6285714</v>
+        <v>11624670.7570748</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32970,11 +33092,11 @@
       <c r="D61" s="93"/>
       <c r="E61" s="94" t="n">
         <f aca="false">E60-E59</f>
-        <v>-1232717.37142857</v>
+        <v>-1174724.24292517</v>
       </c>
       <c r="F61" s="95" t="n">
         <f aca="false">IF(E59&gt;0,E61/E59,"")</f>
-        <v>-0.0963105968234101</v>
+        <v>-0.0917796695019701</v>
       </c>
     </row>
   </sheetData>
@@ -33024,12 +33146,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33039,7 +33161,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33139,10 +33261,10 @@
         <v>0.387667709233293</v>
       </c>
       <c r="L7" s="61" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="Q7" s="62" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>205</v>
@@ -33201,10 +33323,10 @@
         <v>0.0930272321101565</v>
       </c>
       <c r="L8" s="61" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="Q8" s="62" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -33264,7 +33386,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -33323,10 +33445,10 @@
         <v>0.0665492729486535</v>
       </c>
       <c r="L10" s="61" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q10" s="62" t="s">
         <v>265</v>
-      </c>
-      <c r="Q10" s="62" t="s">
-        <v>263</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -33385,10 +33507,10 @@
         <v>0.0663936626599383</v>
       </c>
       <c r="L11" s="61" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="Q11" s="62" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -33448,13 +33570,13 @@
       </c>
       <c r="L12" s="61"/>
       <c r="Q12" s="62" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>205</v>
       </c>
       <c r="S12" s="62" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="T12" s="62" t="n">
         <v>700</v>
@@ -33508,7 +33630,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -33568,7 +33690,7 @@
       </c>
       <c r="L14" s="61"/>
       <c r="Q14" s="62" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -33627,10 +33749,10 @@
         <v>0.0282483930215812</v>
       </c>
       <c r="L15" s="61" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="Q15" s="62" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -33689,10 +33811,10 @@
         <v>0.0272325527669234</v>
       </c>
       <c r="L16" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="Q16" s="62" t="s">
         <v>270</v>
-      </c>
-      <c r="Q16" s="62" t="s">
-        <v>268</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -33752,7 +33874,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -33811,10 +33933,10 @@
         <v>0.0222301631600693</v>
       </c>
       <c r="L18" s="61" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="Q18" s="62" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -33873,10 +33995,10 @@
         <v>0.0208031596594696</v>
       </c>
       <c r="L19" s="61" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="Q19" s="62" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -33936,7 +34058,7 @@
       </c>
       <c r="L20" s="61"/>
       <c r="Q20" s="62" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="R20" s="62" t="s">
         <v>201</v>
@@ -33995,10 +34117,10 @@
         <v>0.00925511581813541</v>
       </c>
       <c r="L21" s="61" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="Q21" s="62" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="R21" s="62" t="s">
         <v>201</v>
@@ -34057,7 +34179,7 @@
         <v>0.0064722190095489</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="Q22" s="62" t="s">
         <v>21</v>
@@ -34119,7 +34241,7 @@
         <v>0.00633173137432947</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="Q23" s="62" t="s">
         <v>21</v>
@@ -34181,7 +34303,7 @@
         <v>0.00565045107879498</v>
       </c>
       <c r="L24" s="61" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="Q24" s="62" t="s">
         <v>21</v>
@@ -34243,7 +34365,7 @@
         <v>0.00494611932858946</v>
       </c>
       <c r="L25" s="61" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="Q25" s="62" t="s">
         <v>21</v>
@@ -34305,7 +34427,7 @@
         <v>0.00271144248698057</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="Q26" s="62" t="s">
         <v>21</v>
@@ -34367,7 +34489,7 @@
         <v>0.00207627374724527</v>
       </c>
       <c r="L27" s="61" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="Q27" s="62" t="s">
         <v>21</v>
@@ -34429,7 +34551,7 @@
         <v>0.00196599683318886</v>
       </c>
       <c r="L28" s="61" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="Q28" s="62" t="s">
         <v>21</v>
@@ -34491,7 +34613,7 @@
         <v>0.000701063389415708</v>
       </c>
       <c r="L29" s="61" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="Q29" s="62" t="s">
         <v>21</v>
@@ -34553,7 +34675,7 @@
         <v>0.00028721368924799</v>
       </c>
       <c r="L30" s="61" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="Q30" s="62" t="s">
         <v>21</v>
@@ -34579,7 +34701,7 @@
         <v>25</v>
       </c>
       <c r="B31" s="59" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>28</v>
@@ -34719,7 +34841,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="75" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E35" s="76" t="n">
         <v>10914339</v>
@@ -35041,12 +35163,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35056,7 +35178,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35157,7 +35279,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -35217,7 +35339,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -35277,7 +35399,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -35709,7 +35831,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="75" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E22" s="76" t="n">
         <v>167022</v>
@@ -35806,12 +35928,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35821,7 +35943,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35922,7 +36044,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -35982,7 +36104,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -36042,7 +36164,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -36101,10 +36223,10 @@
         <v>0.060071305630396</v>
       </c>
       <c r="L10" s="61" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="Q10" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -36164,7 +36286,7 @@
       </c>
       <c r="L11" s="61"/>
       <c r="Q11" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -36223,10 +36345,10 @@
         <v>0.0360333489709902</v>
       </c>
       <c r="L12" s="61" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="Q12" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>201</v>
@@ -36286,7 +36408,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -36348,7 +36470,7 @@
         <v>202</v>
       </c>
       <c r="Q14" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -36408,7 +36530,7 @@
       </c>
       <c r="L15" s="61"/>
       <c r="Q15" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -36468,7 +36590,7 @@
       </c>
       <c r="L16" s="61"/>
       <c r="Q16" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -36528,7 +36650,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -36588,7 +36710,7 @@
       </c>
       <c r="L18" s="61"/>
       <c r="Q18" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -36648,7 +36770,7 @@
       </c>
       <c r="L19" s="61"/>
       <c r="Q19" s="62" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -36798,7 +36920,7 @@
         <v>0.00684755364735877</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36842,7 +36964,7 @@
         <v>0.00408028602961991</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36970,7 +37092,7 @@
         <v>0.00121270175094724</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37044,7 +37166,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="75" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E31" s="76" t="n">
         <v>4529555</v>

</xml_diff>

<commit_message>
Manish: cash added 60,000 on 29.10.2026
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1365" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1366" uniqueCount="296">
   <si>
     <t xml:space="preserve">CONSOLIDATED PORTFOLIO SUMMARY – ALL MANAGED ACCOUNTS</t>
   </si>
@@ -861,6 +861,9 @@
     <t xml:space="preserve">Base – Year 3 base</t>
   </si>
   <si>
+    <t xml:space="preserve">+ Cash added 29.10.2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">SALONI MEHRA – Angel One – 20.10.2026 + trades of 21–23.10.2026</t>
   </si>
   <si>
@@ -960,7 +963,7 @@
     <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3810.0, 436419.72, null, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99; 29.10 buy 48 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 169.0, 15473.53, null, "Axis Direct Shilpa 93; Axis Direct Manish 75; 29.10 buy 1 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3935.0, 2948869.0, null, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504; 29.10 buy 40 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1027.0, 822205.8, null, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56; 29.10 buy 14 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1415.0, 630971.8, null, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8; 29.10 buy 21 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "HDFC Securities (Manish) order book of 29.10.2026 – 5 executed buys; order book carries no fill price, so cost uses its Close Price column (previous close) until the tradebook is supplied", "trades": [["29.10.2026 10:31–10:42", "BUY", "HDFC Gold ETF", 1.0, 119.53, 119.53], ["29.10.2026 10:31–10:42", "BUY", "HDFC Bank Ltd", 14.0, 680.2, 9522.8], ["29.10.2026 10:31–10:42", "BUY", "Poonawalla Fincorp Ltd", 21.0, 402.8, 8458.8], ["29.10.2026 10:31–10:42", "BUY", "Bajaj Housing Finance Ltd", 48.0, 77.64, 3726.72], ["29.1</t>
   </si>
   <si>
-    <t xml:space="preserve">0.2026 10:31–10:42", "BUY", "Bajaj Finance Ltd", 40.0, 912.0, 36480.0]], "base": {"label": "Year 3 base", "amount": 11949395, "cash": [["Cash added", 850000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
+    <t xml:space="preserve">0.2026 10:31–10:42", "BUY", "Bajaj Finance Ltd", 40.0, 912.0, 36480.0]], "base": {"label": "Year 3 base", "amount": 11949395, "cash": [["Cash added", 850000], ["Cash added 29.10.2026", 60000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
   </si>
 </sst>
 </file>
@@ -2276,16 +2279,16 @@
         <v>0.30425080169477</v>
       </c>
       <c r="K8" s="8" t="n">
-        <f aca="false">'Manish Shilpa'!E59</f>
-        <v>12799395</v>
+        <f aca="false">'Manish Shilpa'!E60</f>
+        <v>12859395</v>
       </c>
       <c r="L8" s="8" t="n">
         <f aca="false">G8-K8</f>
-        <v>-1174724.24292517</v>
+        <v>-1234724.24292517</v>
       </c>
       <c r="M8" s="9" t="n">
         <f aca="false">IF(K8&gt;0,L8/K8,"")</f>
-        <v>-0.0917796695019701</v>
+        <v>-0.0960172887546552</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2464,15 +2467,15 @@
       </c>
       <c r="K12" s="17" t="n">
         <f aca="false">SUM(K6:K11)</f>
-        <v>41250071</v>
+        <v>41310071</v>
       </c>
       <c r="L12" s="17" t="n">
         <f aca="false">SUM(L6:L11)</f>
-        <v>-3042543.87986797</v>
+        <v>-3102543.87986797</v>
       </c>
       <c r="M12" s="18" t="n">
         <f aca="false">IF(K12&gt;0,L12/K12,"")</f>
-        <v>-0.0737585125579048</v>
+        <v>-0.0751038137859401</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3062,12 +3065,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -30806,7 +30809,7 @@
     <tabColor rgb="FF27AE60"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V61"/>
+  <dimension ref="A1:V62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -33064,39 +33067,47 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B59" s="92" t="s">
+      <c r="B59" s="75" t="s">
+        <v>261</v>
+      </c>
+      <c r="E59" s="76" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="92" t="s">
         <v>212</v>
       </c>
-      <c r="C59" s="93"/>
-      <c r="D59" s="93"/>
-      <c r="E59" s="94" t="n">
-        <f aca="false">SUM(E57:E58)</f>
-        <v>12799395</v>
-      </c>
-      <c r="F59" s="93"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B60" s="75" t="s">
+      <c r="C60" s="93"/>
+      <c r="D60" s="93"/>
+      <c r="E60" s="94" t="n">
+        <f aca="false">SUM(E57:E59)</f>
+        <v>12859395</v>
+      </c>
+      <c r="F60" s="93"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="75" t="s">
         <v>213</v>
       </c>
-      <c r="E60" s="80" t="n">
+      <c r="E61" s="80" t="n">
         <f aca="false">H54</f>
         <v>11624670.7570748</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B61" s="92" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="92" t="s">
         <v>214</v>
       </c>
-      <c r="C61" s="93"/>
-      <c r="D61" s="93"/>
-      <c r="E61" s="94" t="n">
-        <f aca="false">E60-E59</f>
-        <v>-1174724.24292517</v>
-      </c>
-      <c r="F61" s="95" t="n">
-        <f aca="false">IF(E59&gt;0,E61/E59,"")</f>
-        <v>-0.0917796695019701</v>
+      <c r="C62" s="93"/>
+      <c r="D62" s="93"/>
+      <c r="E62" s="94" t="n">
+        <f aca="false">E61-E60</f>
+        <v>-1234724.24292517</v>
+      </c>
+      <c r="F62" s="95" t="n">
+        <f aca="false">IF(E60&gt;0,E62/E60,"")</f>
+        <v>-0.0960172887546552</v>
       </c>
     </row>
   </sheetData>
@@ -33146,12 +33157,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33161,7 +33172,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -33261,10 +33272,10 @@
         <v>0.387667709233293</v>
       </c>
       <c r="L7" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q7" s="62" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>205</v>
@@ -33323,10 +33334,10 @@
         <v>0.0930272321101565</v>
       </c>
       <c r="L8" s="61" t="s">
+        <v>267</v>
+      </c>
+      <c r="Q8" s="62" t="s">
         <v>266</v>
-      </c>
-      <c r="Q8" s="62" t="s">
-        <v>265</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -33386,7 +33397,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -33445,10 +33456,10 @@
         <v>0.0665492729486535</v>
       </c>
       <c r="L10" s="61" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Q10" s="62" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -33507,10 +33518,10 @@
         <v>0.0663936626599383</v>
       </c>
       <c r="L11" s="61" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="Q11" s="62" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -33570,13 +33581,13 @@
       </c>
       <c r="L12" s="61"/>
       <c r="Q12" s="62" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>205</v>
       </c>
       <c r="S12" s="62" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="T12" s="62" t="n">
         <v>700</v>
@@ -33630,7 +33641,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -33690,7 +33701,7 @@
       </c>
       <c r="L14" s="61"/>
       <c r="Q14" s="62" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -33749,10 +33760,10 @@
         <v>0.0282483930215812</v>
       </c>
       <c r="L15" s="61" t="s">
+        <v>272</v>
+      </c>
+      <c r="Q15" s="62" t="s">
         <v>271</v>
-      </c>
-      <c r="Q15" s="62" t="s">
-        <v>270</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -33811,10 +33822,10 @@
         <v>0.0272325527669234</v>
       </c>
       <c r="L16" s="61" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q16" s="62" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -33874,7 +33885,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -33933,10 +33944,10 @@
         <v>0.0222301631600693</v>
       </c>
       <c r="L18" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q18" s="62" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -33995,10 +34006,10 @@
         <v>0.0208031596594696</v>
       </c>
       <c r="L19" s="61" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q19" s="62" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -34058,7 +34069,7 @@
       </c>
       <c r="L20" s="61"/>
       <c r="Q20" s="62" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R20" s="62" t="s">
         <v>201</v>
@@ -34117,10 +34128,10 @@
         <v>0.00925511581813541</v>
       </c>
       <c r="L21" s="61" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="Q21" s="62" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R21" s="62" t="s">
         <v>201</v>
@@ -34179,7 +34190,7 @@
         <v>0.0064722190095489</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q22" s="62" t="s">
         <v>21</v>
@@ -34241,7 +34252,7 @@
         <v>0.00633173137432947</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q23" s="62" t="s">
         <v>21</v>
@@ -34303,7 +34314,7 @@
         <v>0.00565045107879498</v>
       </c>
       <c r="L24" s="61" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="Q24" s="62" t="s">
         <v>21</v>
@@ -34365,7 +34376,7 @@
         <v>0.00494611932858946</v>
       </c>
       <c r="L25" s="61" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="Q25" s="62" t="s">
         <v>21</v>
@@ -34427,7 +34438,7 @@
         <v>0.00271144248698057</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="Q26" s="62" t="s">
         <v>21</v>
@@ -34489,7 +34500,7 @@
         <v>0.00207627374724527</v>
       </c>
       <c r="L27" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q27" s="62" t="s">
         <v>21</v>
@@ -34551,7 +34562,7 @@
         <v>0.00196599683318886</v>
       </c>
       <c r="L28" s="61" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="Q28" s="62" t="s">
         <v>21</v>
@@ -34613,7 +34624,7 @@
         <v>0.000701063389415708</v>
       </c>
       <c r="L29" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q29" s="62" t="s">
         <v>21</v>
@@ -34675,7 +34686,7 @@
         <v>0.00028721368924799</v>
       </c>
       <c r="L30" s="61" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Q30" s="62" t="s">
         <v>21</v>
@@ -34841,7 +34852,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="75" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E35" s="76" t="n">
         <v>10914339</v>
@@ -35163,12 +35174,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35178,7 +35189,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35279,7 +35290,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -35339,7 +35350,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -35399,7 +35410,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -35831,7 +35842,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="75" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E22" s="76" t="n">
         <v>167022</v>
@@ -35928,12 +35939,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35943,7 +35954,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q5" s="30" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -36044,7 +36055,7 @@
       </c>
       <c r="L7" s="61"/>
       <c r="Q7" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R7" s="62" t="s">
         <v>201</v>
@@ -36104,7 +36115,7 @@
       </c>
       <c r="L8" s="61"/>
       <c r="Q8" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R8" s="62" t="s">
         <v>201</v>
@@ -36164,7 +36175,7 @@
       </c>
       <c r="L9" s="61"/>
       <c r="Q9" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R9" s="62" t="s">
         <v>201</v>
@@ -36223,10 +36234,10 @@
         <v>0.060071305630396</v>
       </c>
       <c r="L10" s="61" t="s">
+        <v>291</v>
+      </c>
+      <c r="Q10" s="62" t="s">
         <v>290</v>
-      </c>
-      <c r="Q10" s="62" t="s">
-        <v>289</v>
       </c>
       <c r="R10" s="62" t="s">
         <v>201</v>
@@ -36286,7 +36297,7 @@
       </c>
       <c r="L11" s="61"/>
       <c r="Q11" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R11" s="62" t="s">
         <v>201</v>
@@ -36345,10 +36356,10 @@
         <v>0.0360333489709902</v>
       </c>
       <c r="L12" s="61" t="s">
+        <v>291</v>
+      </c>
+      <c r="Q12" s="62" t="s">
         <v>290</v>
-      </c>
-      <c r="Q12" s="62" t="s">
-        <v>289</v>
       </c>
       <c r="R12" s="62" t="s">
         <v>201</v>
@@ -36408,7 +36419,7 @@
       </c>
       <c r="L13" s="61"/>
       <c r="Q13" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R13" s="62" t="s">
         <v>201</v>
@@ -36470,7 +36481,7 @@
         <v>202</v>
       </c>
       <c r="Q14" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R14" s="62" t="s">
         <v>201</v>
@@ -36530,7 +36541,7 @@
       </c>
       <c r="L15" s="61"/>
       <c r="Q15" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R15" s="62" t="s">
         <v>201</v>
@@ -36590,7 +36601,7 @@
       </c>
       <c r="L16" s="61"/>
       <c r="Q16" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R16" s="62" t="s">
         <v>201</v>
@@ -36650,7 +36661,7 @@
       </c>
       <c r="L17" s="61"/>
       <c r="Q17" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R17" s="62" t="s">
         <v>201</v>
@@ -36710,7 +36721,7 @@
       </c>
       <c r="L18" s="61"/>
       <c r="Q18" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R18" s="62" t="s">
         <v>201</v>
@@ -36770,7 +36781,7 @@
       </c>
       <c r="L19" s="61"/>
       <c r="Q19" s="62" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R19" s="62" t="s">
         <v>201</v>
@@ -36920,7 +36931,7 @@
         <v>0.00684755364735877</v>
       </c>
       <c r="L22" s="61" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36964,7 +36975,7 @@
         <v>0.00408028602961991</v>
       </c>
       <c r="L23" s="61" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37092,7 +37103,7 @@
         <v>0.00121270175094724</v>
       </c>
       <c r="L26" s="61" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37166,7 +37177,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="75" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E31" s="76" t="n">
         <v>4529555</v>

</xml_diff>

<commit_message>
Manish: 29.10 order book belongs to Axis Direct (Manish)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SpzJBuAvXmgDRsRccNu7gm
</commit_message>
<xml_diff>
--- a/Consolidated_Portfolios_28.10.2026.xlsx
+++ b/Consolidated_Portfolios_28.10.2026.xlsx
@@ -768,13 +768,13 @@
     <t xml:space="preserve">Holdings as of 23.10.2026 (live, ~11:23 IST). Statement prices: Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged). Market value uses the common Ref Price from the Prices sheet so all portfolios are valued alike.</t>
   </si>
   <si>
-    <t xml:space="preserve">HDFC Securities (Manish) order book of 29.10.2026 – 5 executed buys; order book carries no fill price, so cost uses its Close Price column (previous close) until the tradebook is supplied</t>
+    <t xml:space="preserve">Axis Direct (Manish) order book of 29.10.2026 – 5 executed buys; order book carries no fill price, so cost uses its Close Price column (previous close) until the tradebook is supplied</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504; 29.10 buy 40 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
+    <t xml:space="preserve">Axis Direct Shilpa 226; Axis Direct Manish 3205; HDFC Securities Manish 504; incl. 29.10 buy 40 (Axis Direct Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
     <t xml:space="preserve">29.10.2026 10:31–10:42</t>
@@ -786,10 +786,10 @@
     <t xml:space="preserve">Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56; 29.10 buy 14 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
+    <t xml:space="preserve">Axis Direct Shilpa 58; Axis Direct Manish 913; HDFC Securities Manish 56; incl. 29.10 buy 14 (Axis Direct Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8; 29.10 buy 21 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
+    <t xml:space="preserve">Axis Direct Shilpa 206; Axis Direct Manish 1201; HDFC Securities Manish 8; incl. 29.10 buy 21 (Axis Direct Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct (Manish)</t>
@@ -801,7 +801,7 @@
     <t xml:space="preserve">Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99; 29.10 buy 48 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
+    <t xml:space="preserve">Axis Direct Shilpa 267; Axis Direct Manish 3444; HDFC Securities Manish 99; incl. 29.10 buy 48 (Axis Direct Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6</t>
@@ -837,7 +837,7 @@
     <t xml:space="preserve">Axis Direct Shilpa 3; Axis Direct Manish 7</t>
   </si>
   <si>
-    <t xml:space="preserve">Axis Direct Shilpa 93; Axis Direct Manish 75; 29.10 buy 1 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)</t>
+    <t xml:space="preserve">Axis Direct Shilpa 93; Axis Direct Manish 76; incl. 29.10 buy 1 (Axis Direct Manish, costed at order-book Close Price, fill price not given)</t>
   </si>
   <si>
     <t xml:space="preserve">Axis Direct Shilpa 2; Axis Direct Manish 4</t>
@@ -960,10 +960,10 @@
     <t xml:space="preserve">New position 09.10.2026</t>
   </si>
   <si>
-    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3810.0, 436419.72, null, "Axis Direct Shilpa 267; Axis Direct Manish 3396; HDFC Securities Manish 99; 29.10 buy 48 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 169.0, 15473.53, null, "Axis Direct Shilpa 93; Axis Direct Manish 75; 29.10 buy 1 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3935.0, 2948869.0, null, "Axis Direct Shilpa 226; Axis Direct Manish 3165; HDFC Securities Manish 504; 29.10 buy 40 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1027.0, 822205.8, null, "Axis Direct Shilpa 58; Axis Direct Manish 899; HDFC Securities Manish 56; 29.10 buy 14 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1415.0, 630971.8, null, "Axis Direct Shilpa 206; Axis Direct Manish 1180; HDFC Securities Manish 8; 29.10 buy 21 (HDFC Securities Manish, costed at order-book Close Price, fill price not given)"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "HDFC Securities (Manish) order book of 29.10.2026 – 5 executed buys; order book carries no fill price, so cost uses its Close Price column (previous close) until the tradebook is supplied", "trades": [["29.10.2026 10:31–10:42", "BUY", "HDFC Gold ETF", 1.0, 119.53, 119.53], ["29.10.2026 10:31–10:42", "BUY", "HDFC Bank Ltd", 14.0, 680.2, 9522.8], ["29.10.2026 10:31–10:42", "BUY", "Poonawalla Fincorp Ltd", 21.0, 402.8, 8458.8], ["29.10.2026 10:31–10:42", "BUY", "Bajaj Housing Finance Ltd", 48.0, 77.64, 3726.72], ["29.1</t>
+    <t xml:space="preserve">{"built": "28.10.2026", "close_date": "28.10.2026 live (~11:35 IST)", "prev_date": "27.10.2026", "closes": {"AFCOM Holdings Ltd": [1315.9, 1314.65], "Aarti Drugs Ltd": [451.0, 402.25], "Abbott India Ltd": [26025.0, 25515.0], "Affle 3i Ltd": [1372.3, 1354.8], "Alkyl Amines Chemicals Ltd": [1654.5, 1646.3], "Ambuja Cements Ltd": [351.8, 348.8], "Ashoka Buildcon Ltd": [96.37, 97.4], "Asian Paints Ltd": [2259.5, 2277.0], "Avenue Supermarts (DMart) Ltd": [3135.9, 3200.0], "Bagmane Prime Office REIT": [104.1, 104.25], "Bajaj Finance Ltd": [907.6, 912.0], "Bajaj Housing Finance Ltd": [77.29, 77.64], "Bharti Airtel Ltd": [1946.8, 1978.8], "Brigade Enterprises Ltd": [536.45, 552.1], "Capacite Infraprojects Ltd": [148.93, 149.43], "Central Depository Services (India) Ltd": [1220.1, 1222.0], "Clean Science and Technology Ltd": [736.65, 744.0], "Connplex Cinemas Ltd": [236.8, 225.0], "Container Corporation of India Ltd": [414.3, 425.15], "Cyient Ltd": [1157.3, 1182.3], "Deepak Nitrite Ltd": [1468.6, 1431.5], "Dr Lal PathLabs Ltd": [1932.4, 1901.8], "Eicher Motors Ltd": [7150.5, 7165.0], "Eternal Ltd": [325.6, 331.0], "Eureka Forbes Ltd": [316.35, 316.0], "Fineotex Chemical Ltd": [50.01, 48.31], "GSPL Transmission Ltd": [120.0, 115.24], "Garware Technical Fibres Ltd": [748.85, 775.55], "Godrej Consumer Products Ltd": [817.7, 828.8], "Great Eastern Shipping Co Ltd": [1530.5, 1550.9], "Gujarat Energy": [212.59, 212.68], "HCL Technologies Ltd": [1383.8, 1420.0], "HDFC Bank Ltd": [675.15, 680.2], "HUDCO Ltd": [144.51, 143.33], "ICICI Prudential Life Insurance Co Ltd": [406.6, 409.55], "Indian Energy Exchange Ltd": [101.96, 103.49], "Indian Railway Finance Corp Ltd": [73.76, 74.56], "Indraprastha Gas Ltd": [141.15, 139.52], "Indus Towers Ltd": [378.85, 385.3], "Infosys Ltd": [1108.5, 1163.0], "InterGlobe Aviation Ltd (IndiGo)": [4614.6, 4596.5], "JK Tyre &amp; Industries Ltd": [301.9, 303.65], "Jio Financial Services Ltd": [205.36, 207.24], "Jubilant FoodWorks Ltd": [420.25, 429.5], "Kotak Mahindra Bank Ltd": [440.05, 442.5], "L&amp;T Technology Services Ltd": [4037.9, 4174.2], "LTM Ltd (formerly LTIMindtree)": [4021.7, 4059.7], "Mold-Tek Technologies Ltd": [89.79, 86.14], "NCC Ltd": [114.14, 115.41], "NTPC Green Energy Ltd": [82.92, 83.13], "Nestle India Ltd": [1158.3, 1180.5], "Orient Cement Ltd": [113.15, 112.83], "Orient Electric Ltd": [186.45, 187.44], "Page Industries Ltd": [33665.0, 34610.0], "Persistent Systems Ltd": [5758.0, 5832.5], "Pfizer Ltd": [3725.2, 3709.8], "Poonawalla Fincorp Ltd": [400.35, 402.8], "REC Ltd": [289.8, 286.5], "RITES Ltd": [193.92, 197.67], "Rategain Travel Technologies Ltd": [796.95, 800.4], "Reliance Industries Ltd": [1176.7, 1196.2], "Shakti Pumps (India) Ltd": [366.45, 365.8], "Shriram Properties Ltd": [63.0, 64.05], "Sonata Software Ltd": [225.8, 231.45], "Syngene International Ltd": [381.95, 366.2], "Tanla Platforms Ltd": [593.6, 579.15], "Tata Consultancy Services Ltd": [2421.2, 2496.9], "Tata Elxsi Ltd": [3701.5, 3723.4], "Titan Company Ltd": [4303.6, 4365.9], "Trent Ltd": [2842.2, 2820.6], "Utkarsh Small Finance Bank Ltd": [11.83, 11.8], "VRL Logistics Ltd": [268.0, 267.55], "Vaibhav Global Ltd": [186.71, 185.98], "Vedant Fashions (Manyavar) Ltd": [473.4, 476.9], "Vedanta Power (VEDPOWER)": [28.72, 28.96], "Vinati Organics Ltd": [1076.9, 1095.3], "Vinyl Chemicals (India) Ltd": [245.1, 257.84], "Waaree Energies Ltd": [2183.0, 2275.0], "Waaree Renewable Technologies Ltd": [664.35, 679.45]}, "screener_urls": {"Bajaj Finance Ltd": "/company/BAJFINANCE/consolidated/", "Titan Company Ltd": "/company/TITAN/consolidated/", "Poonawalla Fincorp Ltd": "/company/POONAWALLA/consolidated/", "HDFC Bank Ltd": "/company/HDFCBANK/consolidated/", "HCL Technologies Ltd": "/company/HCLTECH/consolidated/", "Bajaj Housing Finance Ltd": "/company/BAJAJHFL/", "LTM Ltd (formerly LTIMindtree)": "/company/LTM/", "Affle 3i Ltd": "/company/AFFLE/consolidated/", "L&amp;T Technology Services Ltd": "/company/LTTS/consolidated/", "Fineotex Chemical Ltd": "/company/FCL/consolidated/", "AFCOM Holdings Ltd": "/company/544224/", "Connplex Cinemas Ltd": "/company/CONNPLEX/", "Vinati Organics Ltd": "/company/VINATIORGA/", "Persistent Systems Ltd": "/company/PERSISTENT/consolidated/", "Tata Consultancy Services Ltd": "/company/TCS/consolidated/", "Tata Elxsi Ltd": "/company/TATAELXSI/", "Trent Ltd": "/company/TRENT/consolidated/", "Avenue Supermarts (DMart) Ltd": "/company/DMART/consolidated/", "Nestle India Ltd": "/company/NESTLEIND/", "Eicher Motors Ltd": "/company/EICHERMOT/consolidated/", "InterGlobe Aviation Ltd (IndiGo)": "/company/INDIGO/", "Waaree Energies Ltd": "/company/WAAREEENER/consolidated/", "Rategain Travel Technologies Ltd": "/company/RATEGAIN/consolidated/", "International Gemmological Institute (India) Ltd": "/company/IGIL/", "Shriram Properties Ltd": "/company/SHRIRAMPPS/consolidated/", "Bagmane Prime Office REIT": "/company/BAGMANE/consolidated/", "Bharti Airtel Ltd": "/company/BHARTIARTL/consolidated/", "Orient Electric Ltd": "/company/ORIENTELEC/", "Reliance Industries Ltd": "/company/RELIANCE/", "Jio Financial Services Ltd": "/company/JIOFIN/", "NCC Ltd": "/company/NCC/", "Capacite Infraprojects Ltd": "/company/CAPACITE/", "Indus Towers Ltd": "/company/INDUSTOWER/", "Vedanta Power (VEDPOWER)": "/company/VEDPOWER/consolidated/", "Moschip Technologies Ltd": "/company/MOSCHIP/", "Godrej Consumer Products Ltd": "/company/GODREJCP/", "Vedant Fashions (Manyavar) Ltd": "/company/MANYAVAR/", "Indian Railway Finance Corp Ltd": "/company/IRFC/", "RITES Ltd": "/company/RITES/", "Indraprastha Gas Ltd": "/company/IGL/", "Great Eastern Shipping Co Ltd": "/company/GESHIP/", "HUDCO Ltd": "/company/HUDCO/", "NTPC Green Energy Ltd": "/company/NTPCGREEN/", "Brigade Enterprises Ltd": "/company/BRIGADE/", "GFL Ltd": "/company/GFLLIMITED/", "Sonata Software Ltd": "/company/SONATSOFTW/", "Syngene International Ltd": "/company/SYNGENE/", "Ambuja Cements Ltd": "/company/AMBUJACEM/", "Astec LifeSciences Ltd": "/company/ASTEC/", "Gujarat Energy": "/company/GUJENERGY/consolidated/", "Indian Energy Exchange Ltd": "/company/IEX/", "Vinyl Chemicals (India) Ltd": "/company/VINYLINDIA/", "JK Tyre &amp; Industries Ltd": "/company/JKTYRE/", "REC Ltd": "/company/RECLTD/", "Shakti Pumps (India) Ltd": "/company/SHAKTIPUMP/", "Ashoka Buildcon Ltd": "/company/ASHOKA/", "Cyient Ltd": "/company/CYIENT/", "Utkarsh Small Finance Bank Ltd": "/company/UTKARSHBNK/", "Orient Cement Ltd": "/company/ORIENTCEM/", "Waaree Renewable Technologies Ltd": "/company/WAAREERTL/consolidated/", "Eureka Forbes Ltd": "/company/EUREKAFORB/", "Eternal Ltd": "/company/ETERNAL/consolidated/", "VRL Logistics Ltd": "/company/VRLLOG/", "Kotak Mahindra Bank Ltd": "/company/KOTAKBANK/consolidated/", "Alkyl Amines Chemicals Ltd": "/company/ALKYLAMINE/", "Pfizer Ltd": "/company/PFIZER/", "Garware Technical Fibres Ltd": "/company/GARFIBRES/consolidated/", "Central Depository Services (India) Ltd": "/company/CDSL/consolidated/", "Abbott India Ltd": "/company/ABBOTINDIA/", "Tanla Platforms Ltd": "/company/TANLA/consolidated/", "Vaibhav Global Ltd": "/company/VAIBHAVGBL/consolidated/", "Asian Paints Ltd": "/company/ASIANPAINT/consolidated/", "Aarti Drugs Ltd": "/company/AARTIDRUGS/consolidated/", "Deepak Nitrite Ltd": "/company/DEEPAKNTR/consolidated/", "Infosys Ltd": "/company/INFY/consolidated/", "Dr Lal PathLabs Ltd": "/company/LALPATHLAB/consolidated/", "Page Industries Ltd": "/company/PAGEIND/", "Clean Science and Technology Ltd": "/company/CLEAN/consolidated/", "Jubilant FoodWorks Ltd": "/company/JUBLFOOD/consolidated/", "ICICI Prudential Life Insurance Co Ltd": "/company/ICICILIFE/", "Container Corporation of India Ltd": "/company/CONCOR/", "GSPL Transmission Ltd": "/company/GSPLTRANS/", "Mold-Tek Technologies Ltd": "/company/MOLDTECH/"}, "notes": ["No exchange close for the 4 ETFs (Nifty 50 BeES, Gold BeES, Liquid BeES, HDFC Gold ETF), the Utkarsh SFB rights entitlement, NEPC Agro and PSL Ltd – these stay at statement price (Liquid BeES holds near ₹1,000).", "Names aligned across statements: LTM Ltd = LTIMindtree (DA); Connplex Cinemas = Connplex Smart Theatres (DA); AFCOM = Afcom Holdings.", "Trades blended into holdings and listed on each tab: Vidushi 05.10.2026 (3 buys, ₹9,889); Dr Umesh 09.10.2026 (13 buys, ₹5.01 L, incl. new Eicher Motors and Rategain).", "Dr Umesh holds ₹36,000 uninvested cash at ICICI Direct – row 'Cash – ICICI Direct' at ₹1 per unit, counted in totals but not as a holding.", "Statement invested/market totals reconcile to transcribed rows within ₹2 (rupee rounding on the statements).", "Gautam: NEPC Agro Foods (144 sh) and PSL Ltd (1,000 sh) still have no cost or price on the statement – carried at nil.", "Manish Shilpa: Axis and HDFC CSVs carry short names (e.g. 'Nip. India Nifty', 'C D S L', 'Waaree Renewab.'); aligned to canonical names. 'Nippon ETF Infra' is carried as Nippon India ETF Infra BeES. ETFs have no exchange close and stay on the statement price.", "Manish Shilpa is new (23.10.2026): Axis Direct (Shilpa), Axis Direct (Manish), HDFC Securities (Manish) and Manish's Axis mutual fund (UTI Nifty 50 Index Fund – 2 folios, ₹1,99,990 invested) merged into one account. A stock held in more than one demat is one row; the row note lists the split. Statement totals: invested ₹98,57,779, market value ₹1,16,36,410 (equity at live ~11:23 IST prices, MF at statement NAV).", "Saloni Mehra is new (Angel One): 26-holding statement of 20.10.2026 (invested ₹1,10,23,244; market value ₹1,13,95,012) rolled forward with the 15 trades of 21–22.10.2026 and the 24 buys of 23.10.2026 (₹7,25,477 at executed prices). 21–22.10 buys include all charges; 23.10 charges are not yet shown by Angel One, so those buys are at executed price only. Kotak Mahindra Bank (1,580 sh, realised ≈ ₹62,288) and LIC Housing Finance (700 sh, realised ≈ ₹-29,271) were sold out; Trent is a new position. Statement invested is the row sum (no printed total after trades); rows touched by trades have no statement value, so 'Stmt Market Value' covers untraded rows only.", "DA refreshed from the HDFC (Invest Right, a/c 2754467) and Kotak statements of 23.10.2026 (53 holdings; invested ₹45,74,421 vs statements ₹45,74,422; market value ₹39,94,524 vs ₹39,94,524). Changes vs the 04.10 file are derived: 3 exits (GFL, Moschip, Astec LifeSciences) and several adds incl. new Container Corporation, GSPL Transmission and Mold-Tek; sells valued at the 04.10 statement price. Stocks held at both brokers are one row.", "Gautam: HDFC statement of 23.10.2026 (31 lines; invested ₹55,01,448) rolled forward with the 28.10.2026 Invest Right tradebook: buys of ₹821,182 across 17 stocks at executed price (no charges shown) and the sale of 325 Nippon India ETF Nifty 1D Rate Liquid BeES at ₹999.99 (₹3,24,997; realised ≈ ₹-3 on cost ₹3,25,000), which exits the position. Changes between the 05.10 and 23.10 statements are no longer listed.", "Prices: Screener.in live prices as at about 11:35 IST on 28.10.2026 (market open); the 1-day change is against the 27.10.2026 close. Connplex Cinemas had no 28.10 print yet and stays at its 27.10 close (₹236.80). Vidushi and Dr Umesh have no new statements since 09.10 and are only repriced."], "portfolios": [{"key": "Gautam", "tab": "Gautam", "name": "Gautam", "broker": "HDFC Securities", "holdings_date": "23.10.2026 + trades of 28.10.2026", "price_basis": "HDFC statement 23.10.2026 rolled forward with the 28.10.2026 Invest Right tradebook", "stmt_invested": 6000656.23, "stmt_mv": 1023697, "basis_label": "Gautam stmt – 23.10 + trades", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Securities", 2296.0, 2271492.7, null, "28.10 buys at executed price (charges not yet shown)"], ["Poonawalla Fincorp Ltd", "HDFC Securities", 1357.0, 617510.15, null, "28.10 buys at executed price (charges not yet shown)"], ["HDFC Bank Ltd", "HDFC Securities", 534.0, 379199.35, null, "28.10 buys at executed price (charges not yet shown)"], ["LTM Ltd (formerly LTIMindtree)", "HDFC Securities", 60, 273840, 256440, "Shown as LTM Limited"], ["Tata Consultancy Services Ltd", "HDFC Securities", 92, 210588, 230644, ""], ["Titan Company Ltd", "HDFC Securities", 57.0, 266973.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Connplex Cinemas Ltd", "HDFC Securities", 800, 211200, 192000, ""], ["AFCOM Holdings Ltd", "HDFC Securities", 120, 199920, 165240, "Shown as AFCOM"], ["Tata Elxsi Ltd", "HDFC Securities", 54.0, 188438.8, null, "28.10 buys at executed price (charges not yet shown)"], ["Eicher Motors Ltd", "HDFC Securities", 24.0, 176238.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Bajaj Housing Finance Ltd", "HDFC Securities", 2064.0, 168875.93, null, "28.10 buys at executed price (charges not yet shown)"], ["L&amp;T Technology Services Ltd", "HDFC Securities", 39.0, 140938.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Persistent Systems Ltd", "HDFC Securities", 23.0, 128540.0, null, "28.10 buys at executed price (charges not yet shown)"], ["InterGlobe Aviation Ltd (IndiGo)", "HDFC Securities", 20, 103860, 92160, "Shown as InterGlobe Aviation Ltd (Indigo)"], ["Affle 3i Ltd", "HDFC Securities", 79.0, 123975.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Trent Ltd", "HDFC Securities", 36.0, 100307.4, null, "28.10 buys at executed price (charges not yet shown)"], ["Avenue Supermarts (DMart) Ltd", "HDFC Securities", 29.0, 105666.0, null, "28.10 buys at executed price (charges not yet shown)"], ["Waaree Energies Ltd", "HDFC Securities", 33.0, 81468.2, null, "28.10 buys at executed price (charges not yet shown)"], ["Rategain Travel Technologies Ltd", "HDFC Securities", 87.0, 71614.05, null, "28.10 buys at executed price (charges not yet shown)"], ["Fineotex Chemical Ltd", "HDFC Securities", 1068.0, 58659.11, null, "28.10 buys at executed price (charges not yet shown)"], ["Nestle India Ltd", "HDFC Securities", 22, 27683, 26180, ""], ["Shriram Properties Ltd", "HDFC Securities", 250, 19250, 16925, ""], ["Bagmane Prime Office REIT", "HDFC Securities", 150, 16050, 15900, ""], ["Nippon India ETF Gold BeES", "HDFC Securities", 121, 13310, 14883, ""], ["Vinati Organics Ltd", "HDFC Securities", 24.0, 27036.1, null, "28.10 buys at executed price (charges not yet shown)"], ["Bharti Airtel Ltd", "HDFC Securities", 5, 9610, 9475, ""], ["Orient Electric Ltd", "HDFC Securities", 25, 4500, 3850, ""], ["HDFC Gold ETF", "HDFC Securities", 29.0, 3913.34, null, "28.10 buys at executed price (charges not yet shown)"], ["NEPC Agro Foods Ltd", "HDFC Securities", 144, null, null, "No cost or price on statement (marked *) – carried at nil"], ["PSL Ltd (formerly PSL Holdings Ltd)", "HDFC Securities", 1000, null, null, "No cost or price on statement (marked *) – carried at nil"]], "trades": [["28.10.2026 11:03–11:25", "BUY", "HDFC Gold ETF", 2.0, 120.67, 241.34], ["28.10.2026 11:03–11:25", "BUY", "Waaree Energies Ltd", 6.0, 2184.2, 13105.2], ["28.10.2026 11:03–11:25", "BUY", "Vinati Organics Ltd", 14.0, 1078.22, 15095.1], ["28.10.2026 11:03–11:25", "BUY", "Fineotex Chemical Ltd", 238.0, 50.24, 11957.11], ["28.10.2026 11:03–11:25", "BUY", "Avenue Supermarts (DMart) Ltd", 5.0, 3144.0, 15720.0], ["28.10.2026 11:03–11:25", "BUY", "Trent Ltd", 5.0, 2860.28, 14301.4], ["28.10.2026 11:03–11:25", "BUY", "Eicher Motors Ltd", 4.0, 7206.0, 28824.0], ["28.10.2026 11:03–11:25", "BUY", "Rategain Travel Technologies Ltd", 15.0, 798.54, 11978.05], ["28.10.2026 11:03–11:25", "BUY", "Affle 3i Ltd", 13.0, 1373.85, 17860.1], ["28.10.2026 11:03–11:25", "BUY", "Persistent Systems Ltd", 4.0, 5776.0, 23104.0], ["28.10.2026 11:03–11:25", "BUY", "L&amp;T Technology Services Ltd", 9.0, 4045.22, 36407.0], ["28.10.2026 11:03–11:25", "BUY", "Tata Elxsi Ltd", 13.0, 3689.6, 47964.8], ["28.10.2026 11:03–11:25", "BUY", "Titan Company Ltd", 10.0, 4307.5, 43075.0], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Housing Finance Ltd", 464.0, 77.47, 35945.93], ["28.10.2026 11:03–11:25", "BUY", "HDFC Bank Ltd", 87.0, 679.05, 59077.35], ["28.10.2026 11:03–11:25", "BUY", "Poonawalla Fincorp Ltd", 225.0, 401.5, 90338.15], ["28.10.2026 11:03–11:25", "BUY", "Bajaj Finance Ltd", 395.0, 909.4, 359213.7], ["28.10.2026 11:03–11:25", "SELL", "Nippon India ETF Nifty 1D Rate Liquid BeES", 325.0, 999.99, 324996.75]], "trades_title": "Invest Right tradebook of 28.10.2026 (buys at executed price, no charges shown; blended into Wtd Avg Cost)", "base": {"label": "Year 0 base", "amount": 2264444, "cash": [["Cash added", 3250000], ["Cash added 28.10.2026", 500000]]}}, {"key": "DA", "tab": "DA", "name": "DA", "broker": "HDFC Securities + Kotak Securities", "holdings_date": "23.10.2026", "price_basis": "HDFC and Kotak statement prices 23.10.2026", "stmt_invested": 4574422.02, "stmt_mv": 3994524.08, "basis_label": "DA stmt – 23.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "HDFC Sec + Kotak", 919, 970744, 853705, ""], ["Poonawalla Fincorp Ltd", "HDFC Sec + Kotak", 798, 380517, 329574, ""], ["HDFC Bank Ltd", "HDFC Sec + Kotak", 379, 281511, 262571, ""], ["Titan Company Ltd", "HDFC Sec + Kotak", 59, 260559, 253682, ""], ["Reliance Industries Ltd", "HDFC Securities", 153, 207940, 182070, ""], ["Connplex Cinemas Ltd", "Kotak Securities", 800, 180246, 174760, ""], ["AFCOM Holdings Ltd", "Kotak Securities", 120, 169264, 157866, "Shown as AFCOM-EQ"], ["Bajaj Housing Finance Ltd", "HDFC Sec + Kotak", 1881, 185750, 145683, ""], ["L&amp;T Technology Services Ltd", "HDFC Sec + Kotak", 27, 96792, 105578, ""], ["Persistent Systems Ltd", "HDFC Sec + Kotak", 18, 92120, 103095, ""], ["Fineotex Chemical Ltd", "HDFC Securities", 2030, 68633, 99714, ""], ["Jio Financial Services Ltd", "HDFC Securities", 416, 104362, 85292, ""], ["Tata Elxsi Ltd", "HDFC Sec + Kotak", 23, 85943, 85100, ""], ["HCL Technologies Ltd", "Kotak Securities", 50, 69140, 71110, ""], ["Tata Consultancy Services Ltd", "HDFC Sec + Kotak", 26, 60830, 65780, ""], ["Eicher Motors Ltd", "HDFC Sec + Kotak", 9, 72272, 63594, ""], ["Nestle India Ltd", "Kotak Securities", 53, 66976, 62275, ""], ["Vedant Fashions (Manyavar) Ltd", "HDFC Securities", 127, 76989, 61144, ""], ["Affle 3i Ltd", "HDFC Sec + Kotak", 46, 76729, 61005, ""], ["Trent Ltd", "HDFC Sec + Kotak", 20, 60183, 54550, ""], ["LTM Ltd (formerly LTIMindtree)", "HDFC Sec + Kotak", 12, 56618, 49608, ""], ["NCC Ltd", "HDFC Securities", 416, 73236, 48331, ""], ["Avenue Supermarts (DMart) Ltd", "HDFC Sec + Kotak", 14, 55642, 44208, ""], ["Brigade Enterprises Ltd", "Kotak Securities", 80, 53311, 43808, ""], ["Indus Towers Ltd", "Kotak Securities", 111, 45554, 42180, ""], ["Great Eastern Shipping Co Ltd", "HDFC Securities", 25, 35051, 37415, ""], ["HDFC Gold ETF", "HDFC Securities", 294, 37444, 35209, ""], ["Capacite Infraprojects Ltd", "HDFC Securities", 230, 64328, 34321, ""], ["Godrej Consumer Products Ltd", "HDFC Securities", 40, 41534, 34254, ""], ["Vedanta Power (VEDPOWER)", "Kotak Securities", 1072, 46148, 30295, ""], ["Gujarat Energy", "Kotak Securities", 110, 30362, 23571, "Name as on statement"], ["Indraprastha Gas Ltd", "Kotak Securities", 166, 33939, 23524, ""], ["Indian Railway Finance Corp Ltd", "Kotak Securities", 302, 47882, 22484, ""], ["RITES Ltd", "Kotak Securities", 116, 29715, 21970, ""], ["NTPC Green Energy Ltd", "Kotak Securities", 245, 27130, 19896, ""], ["Waaree Energies Ltd", "HDFC Securities", 8, 14061, 18839, ""], ["Syngene International Ltd", "Kotak Securities", 51, 30824, 18709, ""], ["HUDCO Ltd", "Kotak Securities", 124, 28041, 18106, ""], ["Sonata Software Ltd", "Kotak Securities", 76, 31099, 17643, ""], ["Ambuja Cements Ltd", "Kotak Securities", 49, 25814, 17586, ""], ["REC Ltd", "Kotak Securities", 54, 27444, 15873, ""], ["Vinyl Chemicals (India) Ltd", "HDFC Securities", 78, 30012, 15605, ""], ["Indian Energy Exchange Ltd", "Kotak Securities", 150, 24070, 15180, ""], ["JK Tyre &amp; Industries Ltd", "Kotak Securities", 48, 19409, 14839, ""], ["Shakti Pumps (India) Ltd", "Kotak Securities", 35, 18902, 13531, ""], ["Ashoka Buildcon Ltd", "Kotak Securities", 132, 23436, 13001, ""], ["Cyient Ltd", "Kotak Securities", 9, 12115, 11097, ""], ["Utkarsh Small Finance Bank Ltd", "HDFC Securities", 560, 30952, 6703, ""], ["GSPL Transmission Ltd", "Kotak Securities", 36, 5419, 4116, ""], ["Orient Cement Ltd", "Kotak Securities", 20, 6321, 2320, ""], ["Utkarsh SFB – Rights Entitlement", "HDFC Securities", 344, 0, 1235, "Rights entitlement – nil cost"], ["Mold-Tek Technologies Ltd", "Kotak Securities", 6, 593, 506, ""], ["Container Corporation of India Ltd", "Kotak Securities", 1, 515, 410, ""]], "trades": [["04.10–23.10.2026", "BUY", "Affle 3i Ltd", 1, 1815.0, 1815], ["04.10–23.10.2026", "SELL", "Astec LifeSciences Ltd", 33, 700.0, 23100], ["04.10–23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 1, 3820.0, 3820], ["04.10–23.10.2026", "BUY", "Bajaj Finance Ltd", 4, 1656.75, 6627], ["04.10–23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 149, 87.37, 13018], ["04.10–23.10.2026", "BUY", "Brigade Enterprises Ltd", 45, 635.58, 28601], ["04.10–23.10.2026", "BUY", "Container Corporation of India Ltd", 1, 515.0, 515], ["04.10–23.10.2026", "BUY", "Eicher Motors Ltd", 1, 7925.0, 7925], ["04.10–23.10.2026", "SELL", "GFL Ltd", 380, 58.0, 22040], ["04.10–23.10.2026", "BUY", "GSPL Transmission Ltd", 36, 150.53, 5419], ["04.10–23.10.2026", "BUY", "Great Eastern Shipping Co Ltd", 6, 1354.67, 8128], ["04.10–23.10.2026", "BUY", "HCL Technologies Ltd", 17, 1289.24, 21917], ["04.10–23.10.2026", "BUY", "HDFC Bank Ltd", 42, 727.38, 30550], ["04.10–23.10.2026", "BUY", "HDFC Gold ETF", 195, 129.57, 25267], ["04.10–23.10.2026", "BUY", "Jio Financial Services Ltd", 42, 223.0, 9366], ["04.10–23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3656.0, 10968], ["04.10–23.10.2026", "BUY", "LTM Ltd (formerly LTIMindtree)", 7, 4708.29, 32958], ["04.10–23.10.2026", "BUY", "Mold-Tek Technologies Ltd", 6, 98.83, 593], ["04.10–23.10.2026", "SELL", "Moschip Technologies Ltd", 187, 210.0, 39270], ["04.10–23.10.2026", "BUY", "NCC Ltd", 17, 153.71, 2613], ["04.10–23.10.2026", "BUY", "Nestle India Ltd", 1, 1196.0, 1196], ["04.10–23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 6, 664.0, 3984], ["04.10–23.10.2026", "BUY", "Reliance Industries Ltd", 7, 1277.43, 8942], ["04.10–23.10.2026", "BUY", "Shakti Pumps (India) Ltd", 2, 508.0, 1016], ["04.10–23.10.2026", "BUY", "Sonata Software Ltd", 9, 328.78, 2959], ["04.10–23.10.2026", "BUY", "Tata Consultancy Services Ltd", 13, 2283.23, 29682], ["04.10–23.10.2026", "BUY", "Tata Elxsi Ltd", 3, 3741.0, 11223], ["04.10–23.10.2026", "BUY", "Trent Ltd", 2, 3126.0, 6252], ["04.10–23.10.2026", "BUY", "Vedant Fashions (Manyavar) Ltd", 61, 550.18, 33561]], "trades_title": "Changes between 04.10 and 23.10 statements (derived; buys at implied avg cost, sells at 04.10 statement price)", "base": {"label": "Year 0 base (as on 14.08.2026)", "amount": 4111335, "cash": []}}, {"key": "Manish", "tab": "Manish Shilpa", "name": "Manish Shilpa", "broker": "Axis Direct + HDFC Securities", "holdings_date": "23.10.2026 (live, ~11:23 IST)", "price_basis": "Live LTP 23.10.2026 ~11:23 IST (equity); MF NAV per Axis statement 23.10.2026 (three demats + MF merged)", "basis_label": "Manish Shilpa stmt – live 23.10", "stale_prices": false, "stmt_invested": 9857779, "stmt_mv": 11636410.18, "rows": [["Bajaj Housing Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3810.0, 436419.72, null, "Axis Direct Shilpa 267; Axis Direct Manish 3444; HDFC Securities Manish 99; incl. 29.10 buy 48 (Axis Direct Manish, costed at order-book Close Price, fill price not given)"], ["Nippon India ETF Nifty 1D Rate Liquid BeES", "Axis Direct (Shilpa) + Axis Direct (Manish)", 4.0, 5559, 5559, "Axis Direct Shilpa 1; Axis Direct Manish 3"], ["Eicher Motors Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 43747, 41760, "Axis Direct Shilpa 1; Axis Direct Manish 5"], ["Waaree Renewable Technologies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 5.0, 5105, 3398, "Axis Direct Shilpa 1; Axis Direct Manish 4"], ["Vinati Organics Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 17.0, 29694, 18142, "Axis Direct Shilpa 1; Axis Direct Manish 15; HDFC Securities Manish 1"], ["Nippon India ETF Nifty 50 BeES", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 11160.0, 1687580, 2864693, "Axis Direct Shilpa 10; Axis Direct Manish 11049; HDFC Securities Manish 101"], ["Affle 3i Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 47.0, 76969, 62254, "Axis Direct Shilpa 18; Axis Direct Manish 25; HDFC Securities Manish 4"], ["Eureka Forbes Ltd", "Axis Direct (Shilpa)", 35.0, 19821, 10747, ""], ["HDFC Gold ETF", "Axis Direct (Shilpa) + Axis Direct (Manish)", 169.0, 15473.53, null, "Axis Direct Shilpa 93; Axis Direct Manish 76; incl. 29.10 buy 1 (Axis Direct Manish, costed at order-book Close Price, fill price not given)"], ["Eternal Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 34.0, 10336, 10411, "Axis Direct Shilpa 9; Axis Direct Manish 25"], ["VRL Logistics Ltd", "Axis Direct (Shilpa)", 50.0, 13962, 12668, ""], ["Tata Elxsi Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 32.0, 212270, 120470, "Axis Direct Shilpa 1; Axis Direct Manish 31"], ["Waaree Energies Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 18946, 13900, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["Bajaj Finance Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 3935.0, 2948869.0, null, "Axis Direct Shilpa 226; Axis Direct Manish 3205; HDFC Securities Manish 504; incl. 29.10 buy 40 (Axis Direct Manish, costed at order-book Close Price, fill price not given)"], ["Persistent Systems Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 11.0, 49823, 63648, "Axis Direct Shilpa 3; Axis Direct Manish 8"], ["Kotak Mahindra Bank Ltd", "Axis Direct (Shilpa) + HDFC Securities (Manish)", 160.0, 63501, 69298, "Axis Direct Shilpa 30; HDFC Securities Manish 130"], ["Trent Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 10.0, 30536, 27130, "Axis Direct Shilpa 3; Axis Direct Manish 7"], ["LTM Ltd (formerly LTIMindtree)", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 66.0, 348137, 276816, "Axis Direct Shilpa 2; Axis Direct Manish 52; HDFC Securities Manish 12"], ["Avenue Supermarts (DMart) Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish)", 6.0, 23637, 18758, "Axis Direct Shilpa 2; Axis Direct Manish 4"], ["HDFC Bank Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1027.0, 822205.8, null, "Axis Direct Shilpa 58; Axis Direct Manish 913; HDFC Securities Manish 56; incl. 29.10 buy 14 (Axis Direct Manish, costed at order-book Close Price, fill price not given)"], ["L&amp;T Technology Services Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 72.0, 303467, 282588, "Axis Direct Shilpa 2; Axis Direct Manish 64; HDFC Securities Manish 6"], ["Titan Company Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 165.0, 564530, 700725, "Axis Direct Shilpa 7; Axis Direct Manish 153; HDFC Securities Manish 5"], ["Poonawalla Fincorp Ltd", "Axis Direct (Shilpa) + Axis Direct (Manish) + HDFC Securities (Manish)", 1415.0, 630971.8, null, "Axis Direct Shilpa 206; Axis Direct Manish 1201; HDFC Securities Manish 8; incl. 29.10 buy 21 (Axis Direct Manish, costed at order-book Close Price, fill price not given)"], ["Alkyl Amines Chemicals Ltd", "Axis Direct (Manish)", 3.0, 12327, 4865, ""], ["Indian Energy Exchange Ltd", "Axis Direct (Manish)", 12.0, 2262, 1209, ""], ["Pfizer Ltd", "Axis Direct (Manish)", 1.0, 6103, 3601, ""], ["Jio Financial Services Ltd", "Axis Direct (Manish)", 32.0, 3256, 6556, ""], ["Garware Technical Fibres Ltd", "Axis Direct (Manish)", 5.0, 3380, 3606, ""], ["Reliance Industries Ltd", "Axis Direct (Manish)", 32.0, 38635, 37526, ""], ["Central Depository Services (India) Ltd", "Axis Direct (Manish)", 134.0, 51658, 158643, ""], ["Connplex Cinemas Ltd", "Axis Direct (Manish)", 800.0, 188075, 175200, ""], ["Tata Consultancy Services Ltd", "Axis Direct (Manish)", 29.0, 97994, 74127, ""], ["Abbott India Ltd", "Axis Direct (Manish)", 3.0, 54700, 74400, ""], ["Tanla Platforms Ltd", "Axis Direct (Manish)", 33.0, 40602, 18610, ""], ["Fineotex Chemical Ltd", "Axis Direct (Manish)", 3500.0, 117474, 167755, ""], ["Nippon India ETF Infra BeES", "Axis Direct (Manish)", 34.0, 14923, 29819, ""], ["Vaibhav Global Ltd", "Axis Direct (Manish)", 5.0, 1680, 936, ""], ["Asian Paints Ltd", "Axis Direct (Manish)", 22.0, 78545, 50046, ""], ["Aarti Drugs Ltd", "Axis Direct (Manish)", 6.0, 3768, 2241, ""], ["Deepak Nitrite Ltd", "Axis Direct (Manish)", 1.0, 2393, 1427, ""], ["Infosys Ltd", "Axis Direct (Manish)", 64.0, 102862, 74240, ""], ["Rategain Travel Technologies Ltd", "Axis Direct (Manish)", 5.0, 3317, 3815, ""], ["AFCOM Holdings Ltd", "Axis Direct (Manish)", 360.0, 362724, 457200, ""], ["Clean Science and Technology Ltd", "Axis Direct (Manish)", 14.0, 22090, 10168, ""], ["Dr Lal PathLabs Ltd", "HDFC Securities (Manish)", 44.0, 52231, 80313, ""], ["Page Industries Ltd", "HDFC Securities (Manish)", 2.0, 93537, 67650, ""], ["UTI Nifty 50 Index Fund - Growth", "Axis Direct (Manish) MF", 2004.589, 199990, 315380.18, "Mutual fund, 2 folios (1,804.130 + 200.459 units); NAV ₹157.3291 per Axis statement 23.10.2026 – no exchange close, statement NAV used"]], "trades_title": "Axis Direct (Manish) order book of 29.10.2026 – 5 executed buys; order book carries no fill price, so cost uses its Close Price column (previous close) until the tradebook is supplied", "trades": [["29.10.2026 10:31–10:42", "BUY", "HDFC Gold ETF", 1.0, 119.53, 119.53], ["29.10.2026 10:31–10:42", "BUY", "HDFC Bank Ltd", 14.0, 680.2, 9522.8], ["29.10.2026 10:31–10:42", "BUY", "Poonawalla Fincorp Ltd", 21.0, 402.8, 8458.8], ["29.10.2026 10:31–10:42", "BUY", "Bajaj Housing Finance Ltd", 48.0, 77.64, 3726.72], </t>
   </si>
   <si>
-    <t xml:space="preserve">0.2026 10:31–10:42", "BUY", "Bajaj Finance Ltd", 40.0, 912.0, 36480.0]], "base": {"label": "Year 3 base", "amount": 11949395, "cash": [["Cash added", 850000], ["Cash added 29.10.2026", 60000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
+    <t xml:space="preserve">["29.10.2026 10:31–10:42", "BUY", "Bajaj Finance Ltd", 40.0, 912.0, 36480.0]], "base": {"label": "Year 3 base", "amount": 11949395, "cash": [["Cash added", 850000], ["Cash added 29.10.2026", 60000]]}}, {"key": "Saloni", "tab": "Saloni Mehra", "name": "Saloni Mehra", "broker": "Angel One", "holdings_date": "20.10.2026 + trades of 21–23.10.2026", "price_basis": "20.10.2026 statement prices (only for rows with no trades since)", "basis_label": "Saloni stmt – 20.10", "stale_prices": true, "stmt_invested": 11739506, "stmt_mv": 2974667, "rows": [["Bajaj Finance Ltd", "Angel One", 4940, 4650978, null, "Trades 21.10 buy 362 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Titan Company Ltd", "Angel One", 250, 1071947, null, "Trades 21.10 buy 9 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Jubilant FoodWorks Ltd", "Angel One", 2000, 845300, 827000, ""], ["Tata Consultancy Services Ltd", "Angel One", 305, 659410, 750575, ""], ["HDFC Bank Ltd", "Angel One", 1140, 876490, null, "Trades 21.10 buy 79 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["AFCOM Holdings Ltd", "Angel One", 360, 361080, 536742, ""], ["LTM Ltd (formerly LTIMindtree)", "Angel One", 83, 323526, 353987, ""], ["ICICI Prudential Life Insurance Co Ltd", "Angel One", 700, 340305, 306600, ""], ["Bajaj Housing Finance Ltd", "Angel One", 4227, 360078, null, "Trades 21.10 buy 547 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Fineotex Chemical Ltd", "Angel One", 5141, 224820, null, "23.10 buys at executed price, charges not yet known"], ["L&amp;T Technology Services Ltd", "Angel One", 78, 269544, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Tata Elxsi Ltd", "Angel One", 65, 262060, null, "Trades 22.10 buy 6 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Connplex Cinemas Ltd", "Angel One", 800, 170200, 198400, ""], ["Poonawalla Fincorp Ltd", "Angel One", 1918, 824630, null, "Trades 21.10 buy 970 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Affle 3i Ltd", "Angel One", 78, 114527, null, "Trades 22.10 buy 8 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Vinati Organics Ltd", "Angel One", 68, 84214, null, "23.10 buys at executed price, charges not yet known"], ["Rategain Travel Technologies Ltd", "Angel One", 82, 70997, null, "Trades 22.10 buy 10 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Persistent Systems Ltd", "Angel One", 13, 68506, null, "Trades 22.10 buy 1 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Waaree Energies Ltd", "Angel One", 11, 31435, null, "23.10 buys at executed price, charges not yet known"], ["Eicher Motors Ltd", "Angel One", 8, 57444, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Avenue Supermarts (DMart) Ltd", "Angel One", 10, 35107, null, "Trades 22.10 buy 4 (charges included in cost); 23.10 buys at executed price, charges not yet known"], ["Nestle India Ltd", "Angel One", 7, 9110, null, "23.10 buys at executed price, charges not yet known"], ["Waaree Renewable Technologies Ltd", "Angel One", 5, 4281, null, "23.10 buys at executed price, charges not yet known"], ["HDFC Gold ETF", "Angel One", 11, 1387, 1363, ""], ["Trent Ltd", "Angel One", 8, 22130, null, "New position, bought 22.10 (charges included in cost); no statement value; 23.10 buys at executed price, charges not yet known"]], "trades_title": "Angel One trades 21–23.10.2026 (blended into holdings; 21–22.10 buys include charges, 23.10 buys at executed price)", "trades": [["21.10.2026", "SELL", "Kotak Mahindra Bank Ltd", 1580, 445.65, 704127], ["21.10.2026", "BUY", "Bajaj Housing Finance Ltd", 547, 81.76, 44723], ["21.10.2026", "BUY", "Titan Company Ltd", 9, 4419.44, 39775], ["21.10.2026", "BUY", "HDFC Bank Ltd", 79, 710.85, 56157], ["21.10.2026", "BUY", "Poonawalla Fincorp Ltd", 970, 445.53, 432164], ["21.10.2026", "SELL", "LIC Housing Finance Ltd", 700, 512.6, 358820], ["21.10.2026", "BUY", "Bajaj Finance Ltd", 362, 935.65, 338705], ["22.10.2026", "BUY", "Persistent Systems Ltd", 1, 5818.0, 5818], ["22.10.2026", "BUY", "Tata Elxsi Ltd", 6, 3852.22, 23113], ["22.10.2026", "BUY", "L&amp;T Technology Services Ltd", 1, 3930.0, 3930], ["22.10.2026", "BUY", "Trent Ltd", 5, 2780.9, 13904], ["22.10.2026", "BUY", "Affle 3i Ltd", 8, 1380.9, 11047], ["22.10.2026", "BUY", "Eicher Motors Ltd", 4, 7063.5, 28254], ["22.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 4, 3191.1, 12764], ["22.10.2026", "BUY", "Rategain Travel Technologies Ltd", 10, 776.5, 7765], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 78, 47.85, 3732], ["23.10.2026", "BUY", "Vinati Organics Ltd", 5, 1067.72, 5339], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.4, 676], ["23.10.2026", "BUY", "Waaree Energies Ltd", 1, 2311.9, 2312], ["23.10.2026", "BUY", "Nestle India Ltd", 3, 1169.4, 3508], ["23.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3130.8, 9392], ["23.10.2026", "BUY", "Trent Ltd", 3, 2730.9, 8193], ["23.10.2026", "BUY", "Eicher Motors Ltd", 2, 6965.5, 13931], ["23.10.2026", "BUY", "Rategain Travel Technologies Ltd", 6, 756.6, 4540], ["23.10.2026", "BUY", "Affle 3i Ltd", 5, 1328.62, 6643], ["23.10.2026", "BUY", "Titan Company Ltd", 6, 4246.32, 25478], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3933.2, 11800], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5795.5, 11591], ["23.10.2026", "BUY", "Tata Elxsi Ltd", 4, 3785.9, 15144], ["23.10.2026", "BUY", "Bajaj Housing Finance Ltd", 367, 77.4, 28406], ["23.10.2026", "BUY", "HDFC Bank Ltd", 51, 688.6, 35119], ["23.10.2026", "BUY", "Poonawalla Fincorp Ltd", 651, 417.5, 271792], ["23.10.2026", "BUY", "Bajaj Finance Ltd", 227, 933.48, 211900], ["23.10.2026", "BUY", "Waaree Renewable Technologies Ltd", 1, 676.95, 677], ["23.10.2026", "BUY", "Waaree Energies Ltd", 2, 2297.9, 4596], ["23.10.2026", "BUY", "Fineotex Chemical Ltd", 233, 48.17, 11224], ["23.10.2026", "BUY", "Vinati Organics Ltd", 15, 1071.81, 16077], ["23.10.2026", "BUY", "Persistent Systems Ltd", 2, 5779.5, 11559], ["23.10.2026", "BUY", "L&amp;T Technology Services Ltd", 3, 3949.8, 11849]], "base": {"label": "Year 1 base", "amount": 10914339, "cash": [["Cash added", 1488000], ["Cash added", 729481]]}}, {"key": "Vidushi", "tab": "Vidushi Malhotra", "name": "Vidushi Malhotra", "broker": "Zerodha", "holdings_date": "04.10.2026 (+ trades of 05.10.2026)", "price_basis": "LTP 05.10.2026", "stmt_invested": 201361, "stmt_mv": 230319, "basis_label": "Vidushi stmt – LTP 05.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "Zerodha", 121, 92928, 117842, ""], ["Titan Company Ltd", "Zerodha", 9, 28441, 41130, ""], ["Poonawalla Fincorp Ltd", "Zerodha", 38, 17192, 17123, ""], ["HDFC Bank Ltd", "Zerodha", 21, 16598, 14863, ""], ["HCL Technologies Ltd", "Zerodha", 9, 10284, 10815, ""], ["Bajaj Housing Finance Ltd", "Zerodha", 121, 13968, 9898, ""], ["LTM Ltd (formerly LTIMindtree)", "Zerodha", 2, 10198, 7972, ""], ["Affle 3i Ltd", "Zerodha", 3, 4954, 4370, ""], ["L&amp;T Technology Services Ltd", "Zerodha", 1, 4607, 3219, ""], ["Fineotex Chemical Ltd", "Zerodha", 50, 1877, 2711, ""], ["Nippon India ETF Nifty 50 BeES", "Zerodha", 1, 251, 257, ""], ["Nippon India ETF Gold BeES", "Zerodha", 1, 63, 121, ""]], "trades_title": "Trades executed 05.10.2026 (already blended into Wtd Avg Cost)", "trades": [["2026-10-05 12:46:57", "BUY", "Poonawalla Fincorp Ltd", 8, 451, 3606], ["2026-10-05 12:46:33", "BUY", "HDFC Bank Ltd", 2, 707, 1414], ["2026-10-05 12:46:00", "BUY", "Bajaj Finance Ltd", 5, 974, 4869]], "base": {"label": "Year 1 base", "amount": 167022, "cash": [["Cash added", 60500]]}}, {"key": "Umesh", "tab": "Dr Umesh Choudhry", "name": "Dr Umesh Choudhry", "broker": "ICICI Direct", "holdings_date": "04.10.2026 + trades of 09.10.2026", "price_basis": "NSE live 09.10.2026 ~09:45 IST", "stmt_invested": 5222229.03, "stmt_mv": 5467267.23, "basis_label": "Umesh stmt – NSE live 09.10", "stale_prices": false, "rows": [["Bajaj Finance Ltd", "ICICI Direct", 2412, 1930286, 2318776, ""], ["Titan Company Ltd", "ICICI Direct", 172, 617467, 751984, ""], ["HDFC Bank Ltd", "ICICI Direct", 673, 599414, 472547, ""], ["AFCOM Holdings Ltd", "ICICI Direct", 240, 203179, 342000, "SME"], ["Poonawalla Fincorp Ltd", "ICICI Direct", 769, 346990, 340513, ""], ["Connplex Cinemas Ltd", "ICICI Direct", 800, 183992, 196000, "SME"], ["Bajaj Housing Finance Ltd", "ICICI Direct", 2198, 255800, 180698, ""], ["LTM Ltd (formerly LTIMindtree)", "ICICI Direct", 37, 216602, 149365, "Shown as LTM Limited"], ["Fineotex Chemical Ltd", "ICICI Direct", 2370, 94397, 133502, ""], ["L&amp;T Technology Services Ltd", "ICICI Direct", 32, 151039, 102480, ""], ["Persistent Systems Ltd", "ICICI Direct", 17, 86733, 95634, ""], ["Vinati Organics Ltd", "ICICI Direct", 82, 160741, 92480, ""], ["Tata Elxsi Ltd", "ICICI Direct", 22, 86278, 67571, ""], ["Affle 3i Ltd", "ICICI Direct", 47, 72448, 66876, ""], ["Tata Consultancy Services Ltd", "ICICI Direct", 29, 122603, 63165, ""], ["Eicher Motors Ltd", "ICICI Direct", 3, 20717, 20805, "New position 09.10.2026"], ["Trent Ltd", "ICICI Direct", 5, 14549, 14550, ""], ["Avenue Supermarts (DMart) Ltd", "ICICI Direct", 4, 14740, 14270, ""], ["Rategain Travel Technologies Ltd", "ICICI Direct", 8, 6760, 6727, "New position 09.10.2026"], ["Nestle India Ltd", "ICICI Direct", 1, 1494, 1325, ""], ["Cash – ICICI Direct", "ICICI Direct", 36000, 36000, 36000, "Uninvested cash, valued at ₹1 per unit"]], "trades_title": "Buys on 09.10.2026 (derived: statement 09.10 minus 04.10; already blended into Wtd Avg Cost)", "trades": [["09.10.2026", "BUY", "Bajaj Finance Ltd", 237, 962.39, 228087], ["09.10.2026", "BUY", "Poonawalla Fincorp Ltd", 176, 442.07, 77804], ["09.10.2026", "BUY", "HDFC Bank Ltd", 55, 701.55, 38585], ["09.10.2026", "BUY", "Titan Company Ltd", 6, 4375.0, 26250], ["09.10.2026", "BUY", "Bajaj Housing Finance Ltd", 280, 82.46, 23089], ["09.10.2026", "BUY", "Persistent Systems Ltd", 4, 5588.0, 22352], ["09.10.2026", "BUY", "Tata Elxsi Ltd", 7, 3081.0, 21567], ["09.10.2026", "BUY", "Eicher Motors Ltd", 3, 6905.67, 20717], ["09.10.2026", "BUY", "Avenue Supermarts (DMart) Ltd", 3, 3560.33, 10681], ["09.10.2026", "BUY", "Affle 3i Ltd", 7, 1415.0, 9905], ["09.10.2026", "BUY", "Trent Ltd", 3, 2885.0, 8655], ["09.10.2026", "BUY", "Rategain Travel Technologies Ltd", 8, 845.0, 6760], ["09.10.2026", "BUY", "L&amp;T Technology Services Ltd", 2, 3185.0, 6370]], "base": {"label": "Year 1 base", "amount": 4529555, "cash": [["Cash added", 436000]]}}]}</t>
   </si>
 </sst>
 </file>

</xml_diff>